<commit_message>
Adopt the owner's README layout and name Aptos on every font
The owner restyled the README sheet in Excel. Its sheet XML and button
positions are taken from that workbook into the repository template; its
17 cell styles, with their fonts, fills and borders, and its strings are
remapped into the template's tables, and the duplicate modern form
controls Excel added are dropped in favour of the legacy buttons the
template uses. Nothing else is taken from that workbook: no VBA, document
properties, sensitivity label or run outputs.

The fonts followed the workbook theme (scheme minor), so sheets copied
into a workbook with a Calibri theme showed Calibri. Every font now names
Aptos without the theme link. The README note on the cap basis named
Results columns X-AA, which the margin columns moved to Z-AC.

Validated: python tools/check.py, all gates pass; template XML parses;
README cells equal the owner's apart from that note; the other eleven
sheets are unchanged. Not opened in Excel.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2814" uniqueCount="943">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2814" uniqueCount="945">
   <si>
     <t>SA-CCR Calculator</t>
   </si>
@@ -2903,6 +2903,12 @@
   </si>
   <si>
     <t>Not implemented: declare SHARED under Margin agreements; the netting set is rejected.</t>
+  </si>
+  <si>
+    <t>Unmargined maturity factors; collateral basis per regime (see Results columns Z-AC).</t>
+  </si>
+  <si>
+    <t>ReadMe</t>
   </si>
 </sst>
 </file>
@@ -2925,13 +2931,12 @@
     <numFmt numFmtId="176" formatCode="0.0E+00"/>
     <numFmt numFmtId="177" formatCode="0.000000000"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -2939,7 +2944,6 @@
       <color rgb="FF1F3864"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
@@ -2947,7 +2951,6 @@
       <color rgb="FF595959"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -2955,7 +2958,6 @@
       <color rgb="FF1F3864"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -2963,14 +2965,12 @@
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -2978,14 +2978,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF595959"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
@@ -2993,14 +2991,12 @@
       <color rgb="FF595959"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF595959"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -3008,7 +3004,6 @@
       <color rgb="FFC00000"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
@@ -3016,7 +3011,6 @@
       <color rgb="FF7F6000"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
@@ -3030,7 +3024,6 @@
       <color rgb="FF375623"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -3038,31 +3031,93 @@
       <color rgb="FF9C0006"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF375623"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="16"/>
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFFC000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFC000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="0"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF1F3864"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF595959"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1F3864"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF1F3864"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3099,8 +3154,23 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -3141,13 +3211,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -3315,6 +3401,57 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="20" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="7" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3629,508 +3766,538 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="shReadme">
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="C3:E72"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:X71"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="4" customWidth="1"/>
-    <col min="3" max="3" width="2.7109375" customWidth="1"/>
-    <col min="4" max="4" width="30.7109375" customWidth="1"/>
-    <col min="5" max="5" width="100.7109375" customWidth="1"/>
+    <col min="1" max="2" width="4" style="57" customWidth="1"/>
+    <col min="3" max="3" width="46" style="57" customWidth="1"/>
+    <col min="4" max="4" width="126.85546875" style="57" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" style="57" customWidth="1"/>
+    <col min="6" max="24" width="0" style="57" hidden="1"/>
+    <col min="25" max="16384" width="9.140625" style="57" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" s="55" customFormat="1"/>
-    <row r="2" ht="26" customHeight="1" s="56" customFormat="1"/>
-    <row r="3" spans="4:5" ht="34" customHeight="1">
-      <c r="D3" s="1" t="s">
+    <row r="1" spans="2:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="58" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="4:5">
-      <c r="D4" s="2" t="s">
+      <c r="C1" s="60"/>
+      <c r="D1" s="59"/>
+      <c r="S1" s="61"/>
+    </row>
+    <row r="2" spans="2:19" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="62" t="s">
+        <v>944</v>
+      </c>
+      <c r="C2" s="64"/>
+      <c r="D2" s="63"/>
+      <c r="S2" s="61"/>
+    </row>
+    <row r="3" spans="2:19" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="65"/>
+    </row>
+    <row r="4" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="C4" s="66" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="4:5">
-      <c r="D7" s="3" t="s">
+    <row r="5" spans="2:19" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="4:5" ht="28" customHeight="1">
-      <c r="D8" s="4" t="s">
+      <c r="D6" s="67"/>
+    </row>
+    <row r="7" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="D7" s="71" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="4:5" ht="28" customHeight="1">
-      <c r="D9" s="4" t="s">
+    <row r="8" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="D8" s="71" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="4:5" ht="28" customHeight="1">
-      <c r="D10" s="4" t="s">
+    <row r="9" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="D9" s="71" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="4:5" ht="16" customHeight="1">
-      <c r="D11" s="4" t="s">
+    <row r="10" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="D10" s="71" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="4:5" ht="28" customHeight="1">
-      <c r="D12" s="4" t="s">
+    <row r="11" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="D11" s="71" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="4:5" ht="28" customHeight="1">
-      <c r="D13" s="4" t="s">
+    <row r="12" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="D12" s="71" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="4:5" ht="28" customHeight="1">
-      <c r="D14" s="4" t="s">
+    <row r="13" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="D13" s="71" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="4:5">
-      <c r="D16" s="3" t="s">
+    <row r="14" spans="2:19" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="70"/>
+      <c r="D14" s="72"/>
+    </row>
+    <row r="15" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" spans="4:5" ht="40" customHeight="1">
-      <c r="D17" s="4" t="s">
+      <c r="D15" s="73"/>
+    </row>
+    <row r="16" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="D16" s="71" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="4:5" ht="40" customHeight="1">
-      <c r="D18" s="4" t="s">
+    <row r="17" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="D17" s="71" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="4:5" ht="40" customHeight="1">
-      <c r="D19" s="4" t="s">
+    <row r="18" spans="3:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="C18" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="D18" s="71" t="s">
         <v>903</v>
       </c>
     </row>
-    <row r="20" spans="4:5" ht="28" customHeight="1">
-      <c r="D20" s="4" t="s">
+    <row r="19" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="D19" s="71" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="4:5" ht="40" customHeight="1">
-      <c r="D21" s="4" t="s">
+    <row r="20" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="D20" s="71" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="4:5" ht="28" customHeight="1">
-      <c r="D22" s="4" t="s">
+    <row r="21" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="D21" s="71" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="4:5" ht="40" customHeight="1">
-      <c r="D23" s="4" t="s">
+    <row r="22" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="D22" s="71" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="4:5">
-      <c r="D25" s="3" t="s">
+    <row r="23" spans="3:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C23" s="70"/>
+      <c r="D23" s="72"/>
+    </row>
+    <row r="24" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C24" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="E25" s="3"/>
-    </row>
-    <row r="26" spans="4:5" ht="28" customHeight="1">
-      <c r="D26" s="4" t="s">
+      <c r="D24" s="73"/>
+    </row>
+    <row r="25" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="D25" s="71" t="s">
         <v>917</v>
       </c>
     </row>
-    <row r="27" spans="4:5">
-      <c r="D27" s="4" t="s">
+    <row r="26" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="D26" s="71" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="4:5">
-      <c r="D28" s="4" t="s">
+    <row r="27" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C27" s="69" t="s">
         <v>37</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="D27" s="71" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="4:5" ht="28" customHeight="1">
-      <c r="D29" s="4" t="s">
+    <row r="28" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C28" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="D28" s="71" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="4:5">
-      <c r="D30" s="4" t="s">
+    <row r="29" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C29" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="D29" s="71" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="4:5" ht="28" customHeight="1">
-      <c r="D31" s="4" t="s">
+    <row r="30" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C30" s="69" t="s">
         <v>43</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="D30" s="71" t="s">
         <v>918</v>
       </c>
     </row>
-    <row r="32" spans="4:5" ht="28" customHeight="1">
-      <c r="D32" s="4" t="s">
+    <row r="31" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C31" s="69" t="s">
         <v>45</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="D31" s="71" t="s">
         <v>904</v>
       </c>
     </row>
-    <row r="33" spans="4:5">
-      <c r="D33" s="4" t="s">
+    <row r="32" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C32" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="E33" s="5" t="s">
+      <c r="D32" s="71" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="34" spans="4:5">
-      <c r="D34" s="4" t="s">
+    <row r="33" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="D33" s="71" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="35" spans="4:5" ht="28" customHeight="1">
-      <c r="D35" s="4" t="s">
+    <row r="34" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C34" s="69" t="s">
         <v>51</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="D34" s="71" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="36" spans="4:5">
-      <c r="D36" s="4" t="s">
+    <row r="35" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="D35" s="71" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="38" spans="4:5">
-      <c r="D38" s="3" t="s">
+    <row r="36" spans="3:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C36" s="70"/>
+      <c r="D36" s="72"/>
+    </row>
+    <row r="37" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="E38" s="3"/>
-    </row>
-    <row r="39" spans="4:5">
-      <c r="D39" s="4" t="s">
+      <c r="D37" s="73"/>
+    </row>
+    <row r="38" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C38" s="69" t="s">
         <v>56</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="D38" s="71" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="4:5">
-      <c r="D40" s="4" t="s">
+    <row r="39" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="D39" s="71" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="4:5">
-      <c r="D41" s="4" t="s">
+    <row r="40" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C40" s="69" t="s">
         <v>60</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="D40" s="71" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="42" spans="4:5">
-      <c r="D42" s="4" t="s">
+    <row r="41" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C41" s="69" t="s">
         <v>62</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="D41" s="71" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="43" spans="4:5">
-      <c r="D43" s="4" t="s">
+    <row r="42" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C42" s="69" t="s">
         <v>64</v>
       </c>
-      <c r="E43" s="5" t="s">
+      <c r="D42" s="71" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="4:5">
-      <c r="D44" s="4" t="s">
+    <row r="43" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C43" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="E44" s="5" t="s">
+      <c r="D43" s="71" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="45" spans="4:5">
-      <c r="D45" s="4" t="s">
+    <row r="44" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C44" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="D44" s="71" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="46" spans="4:5">
-      <c r="D46" s="4" t="s">
+    <row r="45" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C45" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="D45" s="71" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="47" spans="4:5">
-      <c r="D47" s="4" t="s">
+    <row r="46" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C46" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="E47" s="5" t="s">
+      <c r="D46" s="71" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="48" spans="4:5">
-      <c r="D48" s="4" t="s">
+    <row r="47" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C47" s="69" t="s">
         <v>74</v>
       </c>
-      <c r="E48" s="5" t="s">
+      <c r="D47" s="71" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="49" spans="4:5">
-      <c r="D49" s="4" t="s">
+    <row r="48" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C48" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="E49" s="5" t="s">
+      <c r="D48" s="71" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="51" spans="4:5">
-      <c r="D51" s="3" t="s">
+    <row r="49" spans="3:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C49" s="70"/>
+      <c r="D49" s="72"/>
+    </row>
+    <row r="50" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="68" t="s">
         <v>78</v>
       </c>
-      <c r="E51" s="3"/>
-    </row>
-    <row r="52" spans="4:5">
-      <c r="D52" s="4" t="s">
+      <c r="D50" s="73"/>
+    </row>
+    <row r="51" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C51" s="69" t="s">
         <v>79</v>
       </c>
-      <c r="E52" s="5" t="s">
+      <c r="D51" s="71" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="53" spans="4:5">
-      <c r="D53" s="4" t="s">
+    <row r="52" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C52" s="69" t="s">
         <v>81</v>
       </c>
-      <c r="E53" s="5" t="s">
+      <c r="D52" s="71" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="54" spans="4:5">
-      <c r="D54" s="4" t="s">
+    <row r="53" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="E54" s="5" t="s">
+      <c r="D53" s="71" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="55" spans="4:5">
-      <c r="D55" s="4" t="s">
+    <row r="54" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C54" s="69" t="s">
         <v>84</v>
       </c>
-      <c r="E55" s="5" t="s">
+      <c r="D54" s="71" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="56" spans="4:5">
-      <c r="D56" s="4" t="s">
+    <row r="55" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C55" s="69" t="s">
         <v>86</v>
       </c>
-      <c r="E56" s="5" t="s">
+      <c r="D55" s="71" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="57" spans="4:5">
-      <c r="D57" s="4" t="s">
+    <row r="56" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C56" s="69" t="s">
         <v>88</v>
       </c>
-      <c r="E57" s="5" t="s">
+      <c r="D56" s="71" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="58" spans="4:5">
-      <c r="D58" s="4" t="s">
+    <row r="57" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C57" s="69" t="s">
         <v>90</v>
       </c>
-      <c r="E58" s="5" t="s">
+      <c r="D57" s="71" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="59" spans="4:5">
-      <c r="D59" s="4" t="s">
+    <row r="58" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C58" s="69" t="s">
         <v>92</v>
       </c>
-      <c r="E59" s="5" t="s">
+      <c r="D58" s="71" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="60" spans="4:5">
-      <c r="D60" s="4" t="s">
+    <row r="59" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C59" s="69" t="s">
         <v>94</v>
       </c>
-      <c r="E60" s="5" t="s">
+      <c r="D59" s="71" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="61" spans="4:5">
-      <c r="D61" s="4" t="s">
+    <row r="60" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C60" s="69" t="s">
         <v>96</v>
       </c>
-      <c r="E61" s="5" t="s">
+      <c r="D60" s="71" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="63" spans="4:5">
-      <c r="D63" s="3" t="s">
+    <row r="61" spans="3:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C61" s="70"/>
+      <c r="D61" s="72"/>
+    </row>
+    <row r="62" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C62" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="E63" s="3"/>
-    </row>
-    <row r="64" spans="4:5" ht="28" customHeight="1">
-      <c r="D64" s="4" t="s">
+      <c r="D62" s="73"/>
+    </row>
+    <row r="63" spans="3:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="C63" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="E64" s="5" t="s">
+      <c r="D63" s="71" t="s">
         <v>905</v>
       </c>
     </row>
-    <row r="65" spans="4:5" ht="28" customHeight="1">
-      <c r="D65" s="4" t="s">
+    <row r="64" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C64" s="69" t="s">
         <v>907</v>
       </c>
-      <c r="E65" s="5" t="s">
+      <c r="D64" s="71" t="s">
         <v>906</v>
       </c>
     </row>
-    <row r="66" spans="4:5">
-      <c r="D66" s="4" t="s">
+    <row r="65" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C65" s="69" t="s">
         <v>103</v>
       </c>
-      <c r="E66" s="5" t="s">
+      <c r="D65" s="71" t="s">
         <v>919</v>
       </c>
     </row>
-    <row r="67" spans="4:5">
-      <c r="D67" s="4" t="s">
+    <row r="66" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C66" s="69" t="s">
         <v>105</v>
       </c>
-      <c r="E67" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="68" spans="4:5">
-      <c r="D68" s="4" t="s">
+      <c r="D66" s="71" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="67" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C67" s="69" t="s">
         <v>107</v>
       </c>
-      <c r="E68" s="5" t="s">
+      <c r="D67" s="71" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="69" spans="4:5" ht="28" customHeight="1">
-      <c r="D69" s="4" t="s">
+    <row r="68" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C68" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="E69" s="5" t="s">
+      <c r="D68" s="71" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="71" spans="4:5">
-      <c r="D71" s="3" t="s">
+    <row r="69" spans="3:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C69" s="70"/>
+      <c r="D69" s="72"/>
+    </row>
+    <row r="70" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C70" s="68" t="s">
         <v>111</v>
       </c>
-      <c r="E71" s="3"/>
-    </row>
-    <row r="72" spans="4:5" ht="28" customHeight="1">
-      <c r="D72" s="4" t="s">
+      <c r="D70" s="73"/>
+    </row>
+    <row r="71" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C71" s="69" t="s">
         <v>112</v>
       </c>
-      <c r="E72" s="5" t="s">
+      <c r="D71" s="71" t="s">
         <v>113</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D71:E71"/>
-  </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
Set the README zoom, header size and engine label
As asked by the owner: README opens at 120% zoom, its seven section
headers (How to use to Code) use a 14 pt font, and C4 names the engine
v1.0.0 instead of the prototype's v1.1.0. The header style was used only
by those seven cells; it gets its own 14 pt font, so the other cells that
shared the 12 pt font are unchanged.

Validated: python tools/check.py, all gates pass; template XML parses;
README text differs only in C4; the other sheets are unchanged. Not
opened in Excel.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -79,7 +79,7 @@
     <t>SA-CCR Calculator</t>
   </si>
   <si>
-    <t>Standardised approach for counterparty credit risk - common Basel CRE52 core with an EU CRR (Art. 274-280f) rules layer. VBA engine v1.1.0.</t>
+    <t>Standardised approach for counterparty credit risk - common Basel CRE52 core with an EU CRR (Art. 274-280f) rules layer. VBA engine v1.0.0.</t>
   </si>
   <si>
     <t>How to use</t>
@@ -2931,7 +2931,7 @@
     <numFmt numFmtId="176" formatCode="0.0E+00"/>
     <numFmt numFmtId="177" formatCode="0.000000000"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3112,6 +3112,13 @@
     <font>
       <b/>
       <sz val="9"/>
+      <color rgb="FF1F3864"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color rgb="FF1F3864"/>
       <name val="Aptos"/>
       <family val="2"/>
@@ -3434,7 +3441,7 @@
     <xf numFmtId="0" fontId="24" fillId="7" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="7" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="7" borderId="4" xfId="0" applyFont="1" applyAlignment="1">

</xml_diff>

<commit_message>
Validate the supervisory-factor and FX tables on Params
SF table (rows 29 to 54): SF_Key text and unique; asset class list
(messages added to the existing list); supervisory factor and
correlation 0 to 100%; option volatility 0 to 500%; commodity hedging
set ENERGY, METALS, AGRICULTURAL, OTHER or CLIMATIC; regimes BOTH, CRR
or BCBS (messages added to the existing list).

FX table (rows 58 to 77, so currencies added below the last row are
covered): currency a unique three-letter code; rate a number above zero,
and 1 for the reporting currency.

Validated: python tools/check.py, all gates pass; openpyxl reads all 29
validations and every current SF and FX value satisfies its rule. Only
sheet2.xml changed in the package. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -8925,7 +8925,7 @@
     </row>
     <row r="64" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="22">
+  <dataValidations count="29">
     <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid reporting date" error="Enter a date between 2000 and 2100." promptTitle="Reporting date" prompt="Date the exposures are calculated for. Maturities and dates are measured from it." sqref="E6">
       <formula1>36526</formula1>
       <formula2>73415</formula2>
@@ -8999,11 +8999,35 @@
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J29:J54" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid or duplicate key" error="Enter a text key that is not already used in this table." promptTitle="Supervisory factor key" prompt="Unique key of the row, e.g. CR_BBB. A key listed twice with different values stops the run." sqref="C29:C54">
+      <formula1>AND(ISTEXT(C29),COUNTIF($C$29:$C$54,C29)=1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid asset class" error="Choose IR, FX, CR, EQ, CO or OT." promptTitle="Asset class" prompt="IR, FX, CR (credit), EQ (equity), CO (commodity) or OT (other risks, CRR Art. 280f)." sqref="D29:D55">
+      <formula1>"IR,FX,CR,EQ,CO,OT"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid supervisory factor" error="Enter a percentage from 0% to 100%." promptTitle="Supervisory factor" prompt="Supervisory factor as a percentage (CRE52.72; CRR Art. 280a to 280f)." sqref="F29:F54">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid correlation" error="Enter a percentage from 0% to 100%." promptTitle="Correlation" prompt="Correlation with the systematic factor, for credit, equity and commodity (CRE52.72). Leave blank for IR, FX and OT." sqref="G29:G54">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid volatility" error="Enter a percentage from 0% to 500%." promptTitle="Supervisory option volatility" prompt="Volatility used in the supervisory delta of options (CRE52.72)." sqref="H29:H54">
+      <formula1>0</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid hedging set" error="Choose ENERGY, METALS, AGRICULTURAL, OTHER or CLIMATIC." promptTitle="Commodity hedging set" prompt="Commodity rows only (CRE52.69). CLIMATIC is the CRR climatic-conditions hedging set (Art. 277a(1)(e)). Leave blank for other asset classes." sqref="I29:I54">
+      <formula1>"ENERGY,METALS,AGRICULTURAL,OTHER,CLIMATIC"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid regime" error="Choose BOTH, CRR or BCBS." promptTitle="Regimes" prompt="Regimes in which the row applies: BOTH, CRR only or BCBS only." sqref="J29:J54">
       <formula1>"BOTH,CRR,BCBS"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D29:D55" xr:uid="{92FC5665-A317-49D8-9552-6AF5B626BBD5}">
-      <formula1>"IR,FX,CR,EQ,CO,OT"</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid or duplicate currency" error="Enter a three-letter ISO code that is not already in the table." promptTitle="Currency" prompt="ISO code, e.g. USD. Add currencies directly below the last row, with no blank rows." sqref="C58:C77">
+      <formula1>AND(ISTEXT(C58),LEN(C58)=3,COUNTIF($C$58:$C$77,C58)=1)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid FX rate" error="Enter a number greater than zero; the reporting currency's rate must be 1." promptTitle="FX rate" prompt="Units of the reporting currency per 1 unit of this currency. The reporting currency itself is 1." sqref="E58:E77">
+      <formula1>AND(ISNUMBER(E58),E58&gt;0,OR(UPPER(C58)&lt;&gt;UPPER(ReportingCcy),E58=1))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Highlight repeated IDs and explain the Trades netting-set list
Data validation is not applied to pasted values, so a duplicate
netting-set ID pasted into NettingSets was accepted (owner's Excel
check). Conditional formatting now shows a repeated value in red
(the template's existing light-red style) on NettingSets C7:C206,
the supervisory-factor keys (Params C29:C54) and the FX currencies
(Params C58:C77), however it was entered. The engine still rejects a
repeated netting-set ID at run time.

The Trades NettingSetID drop-down (D7:D5002, list from NettingSets
C7:C206, warning style) already existed; it now has an input message
and a warning that a trade whose netting set is not listed is rejected,
as the engine does ("unknown netting set").

Validated: python tools/check.py, all gates pass; openpyxl reads the
three rules and the list's messages. Only sheet2, sheet3 and sheet4 XML
changed in the package. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -9099,6 +9099,16 @@
     </row>
     <row r="64" spans="3:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <conditionalFormatting sqref="C29:C54">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>AND(C29&lt;&gt;"",COUNTIF($C$29:$C$54,C29)&gt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C58:C77">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>AND(C58&lt;&gt;"",COUNTIF($C$58:$C$77,C58)&gt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="29">
     <dataValidation type="date" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid reporting date" error="Enter a date between 2000 and 2100." promptTitle="Reporting date" prompt="Date the exposures are calculated for. Maturities and dates are measured from it." sqref="E6">
       <formula1>36526</formula1>
@@ -13376,6 +13386,11 @@
     <row r="433" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="434" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <conditionalFormatting sqref="C7:C206">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>AND(C7&lt;&gt;"",COUNTIF($C$7:$C$206,C7)&gt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="14">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Duplicate ID" error="This netting set ID is already used. Enter a unique ID." promptTitle="Netting set ID" prompt="Unique ID of the legally enforceable netting set. Trades refer to it. A repeated ID makes the set INVALID." sqref="C7:C206">
       <formula1>COUNTIF($C$7:$C$206,C7)=1</formula1>
@@ -25070,7 +25085,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K7:K5002">
       <formula1>"Standard,Basis,Volatility"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D5002">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Netting set not listed" error="This ID is not on NettingSets. Add the netting set there, or the trade will be rejected. Continue anyway?" promptTitle="Netting set" prompt="Choose the ID of a netting set listed on NettingSets. A trade whose netting set is not listed there is rejected." sqref="D7:D5002">
       <formula1>NettingSets!$C$7:$C$206</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Show the Tests unit-test formulas without the @ operator
Tests F8:F29 call the SACCR_* worksheet functions. They were stored as
pre-dynamic-array formulas, so Excel 365 displayed them with the
implicit-intersection operator (=@SACCR_OptionDelta(...)), as it does
for any VBA function in that format. They are now stored as
dynamic-array formulas, like the status formula in Results C5, and
display as entered. Results are unchanged: each function returns one
value.

Validated: python tools/check.py, all gates pass; the 22 cells checked
in the package XML; the template opens in LibreOffice. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -6936,8 +6936,8 @@
       <c r="E8" s="125">
         <v>7.8693868057473324</v>
       </c>
-      <c r="F8" s="125">
-        <f>SACCR_SupervisoryDuration(0,10)</f>
+      <c r="F8" s="125" cm="1">
+        <f t="array" ref="F8">SACCR_SupervisoryDuration(0,10)</f>
         <v>7.8693868057473315</v>
       </c>
       <c r="G8" s="126">
@@ -6959,8 +6959,8 @@
       <c r="E9" s="125">
         <v>7.4855922824045473</v>
       </c>
-      <c r="F9" s="125">
-        <f>SACCR_SupervisoryDuration(1,11)</f>
+      <c r="F9" s="125" cm="1">
+        <f t="array" ref="F9">SACCR_SupervisoryDuration(1,11)</f>
         <v>7.4855922824045473</v>
       </c>
       <c r="G9" s="126">
@@ -6982,8 +6982,8 @@
       <c r="E10" s="125">
         <v>0.04</v>
       </c>
-      <c r="F10" s="125">
-        <f>SACCR_SupervisoryDuration(0,0.01,10/250)</f>
+      <c r="F10" s="125" cm="1">
+        <f t="array" ref="F10">SACCR_SupervisoryDuration(0,0.01,10/250)</f>
         <v>0.04</v>
       </c>
       <c r="G10" s="126">
@@ -7005,8 +7005,8 @@
       <c r="E11" s="125">
         <v>0.8660254037844386</v>
       </c>
-      <c r="F11" s="125">
-        <f>SACCR_MaturityFactor(0.75)</f>
+      <c r="F11" s="125" cm="1">
+        <f t="array" ref="F11">SACCR_MaturityFactor(0.75)</f>
         <v>0.8660254037844386</v>
       </c>
       <c r="G11" s="126">
@@ -7028,8 +7028,8 @@
       <c r="E12" s="125">
         <v>0.2</v>
       </c>
-      <c r="F12" s="125">
-        <f>SACCR_MaturityFactor(3/365)</f>
+      <c r="F12" s="125" cm="1">
+        <f t="array" ref="F12">SACCR_MaturityFactor(3/365)</f>
         <v>0.2</v>
       </c>
       <c r="G12" s="126">
@@ -7051,8 +7051,8 @@
       <c r="E13" s="125">
         <v>0.3</v>
       </c>
-      <c r="F13" s="125">
-        <f>SACCR_MaturityFactor(0,TRUE,10)</f>
+      <c r="F13" s="125" cm="1">
+        <f t="array" ref="F13">SACCR_MaturityFactor(0,TRUE,10)</f>
         <v>0.30000000000000004</v>
       </c>
       <c r="G13" s="126">
@@ -7074,8 +7074,8 @@
       <c r="E14" s="125">
         <v>-0.26939521771053271</v>
       </c>
-      <c r="F14" s="125">
-        <f>SACCR_OptionDelta(0.06,0.05,1,0.5,FALSE,TRUE)</f>
+      <c r="F14" s="125" cm="1">
+        <f t="array" ref="F14">SACCR_OptionDelta(0.06,0.05,1,0.5,FALSE,TRUE)</f>
         <v>-0.26939521771053271</v>
       </c>
       <c r="G14" s="126">
@@ -7097,8 +7097,8 @@
       <c r="E15" s="125">
         <v>-0.37901134582780288</v>
       </c>
-      <c r="F15" s="125">
-        <f>SACCR_OptionDelta(100,110,0.5,0.32,TRUE,FALSE)</f>
+      <c r="F15" s="125" cm="1">
+        <f t="array" ref="F15">SACCR_OptionDelta(100,110,0.5,0.32,TRUE,FALSE)</f>
         <v>-0.37901134582780294</v>
       </c>
       <c r="G15" s="126">
@@ -7120,8 +7120,8 @@
       <c r="E16" s="125">
         <v>0.46143935794124907</v>
       </c>
-      <c r="F16" s="125">
-        <f>SACCR_OptionDelta(-0.002,0.001,2,0.5,TRUE,TRUE,0.01)</f>
+      <c r="F16" s="125" cm="1">
+        <f t="array" ref="F16">SACCR_OptionDelta(-0.002,0.001,2,0.5,TRUE,TRUE,0.01)</f>
         <v>0.46143935794124913</v>
       </c>
       <c r="G16" s="126">
@@ -7143,8 +7143,8 @@
       <c r="E17" s="125">
         <v>5.740967544396816</v>
       </c>
-      <c r="F17" s="125">
-        <f>SACCR_CDODelta(0.03,0.06,TRUE)</f>
+      <c r="F17" s="125" cm="1">
+        <f t="array" ref="F17">SACCR_CDODelta(0.03,0.06,TRUE)</f>
         <v>5.740967544396816</v>
       </c>
       <c r="G17" s="126">
@@ -7166,8 +7166,8 @@
       <c r="E18" s="125">
         <v>59269.963463710403</v>
       </c>
-      <c r="F18" s="125">
-        <f>SACCR_IREffectiveNotional(0,-36253.8493844036,78693.8680574733)</f>
+      <c r="F18" s="125" cm="1">
+        <f t="array" ref="F18">SACCR_IREffectiveNotional(0,-36253.8493844036,78693.8680574733)</f>
         <v>59269.963463710395</v>
       </c>
       <c r="G18" s="126">
@@ -7189,8 +7189,8 @@
       <c r="E19" s="125">
         <v>282.1288318596666</v>
       </c>
-      <c r="F19" s="125">
-        <f>SACCR_FactorAggregation({105.861937916956,-279.916321663744,168.111404865732},{0.5,0.5,0.8})</f>
+      <c r="F19" s="125" cm="1">
+        <f t="array" ref="F19">SACCR_FactorAggregation({105.861937916956,-279.916321663744,168.111404865732},{0.5,0.5,0.8})</f>
         <v>282.12883185966604</v>
       </c>
       <c r="G19" s="126">
@@ -7212,8 +7212,8 @@
       <c r="E20" s="125">
         <v>0.96519268118719448</v>
       </c>
-      <c r="F20" s="125">
-        <f>SACCR_Multiplier(-20,282)</f>
+      <c r="F20" s="125" cm="1">
+        <f t="array" ref="F20">SACCR_Multiplier(-20,282)</f>
         <v>0.96519268118719448</v>
       </c>
       <c r="G20" s="126">
@@ -7235,8 +7235,8 @@
       <c r="E21" s="125">
         <v>1</v>
       </c>
-      <c r="F21" s="125">
-        <f>SACCR_Multiplier(10,282)</f>
+      <c r="F21" s="125" cm="1">
+        <f t="array" ref="F21">SACCR_Multiplier(10,282)</f>
         <v>1</v>
       </c>
       <c r="G21" s="126">
@@ -7258,8 +7258,8 @@
       <c r="E22" s="125">
         <v>8</v>
       </c>
-      <c r="F22" s="125">
-        <f>SACCR_ReplacementCost(5,10,TRUE,0,10,2)</f>
+      <c r="F22" s="125" cm="1">
+        <f t="array" ref="F22">SACCR_ReplacementCost(5,10,TRUE,0,10,2)</f>
         <v>8</v>
       </c>
       <c r="G22" s="126">
@@ -7281,8 +7281,8 @@
       <c r="E23" s="125">
         <v>0.97500210485177952</v>
       </c>
-      <c r="F23" s="125">
-        <f>SACCR_NormCDF(1.96)</f>
+      <c r="F23" s="125" cm="1">
+        <f t="array" ref="F23">SACCR_NormCDF(1.96)</f>
         <v>0.97500210485177952</v>
       </c>
       <c r="G23" s="126">
@@ -7304,8 +7304,8 @@
       <c r="E24" s="125">
         <v>6.2209605742718194E-16</v>
       </c>
-      <c r="F24" s="125">
-        <f>SACCR_NormCDF(-8)</f>
+      <c r="F24" s="125" cm="1">
+        <f t="array" ref="F24">SACCR_NormCDF(-8)</f>
         <v>6.2209605201427843E-16</v>
       </c>
       <c r="G24" s="126">
@@ -7327,8 +7327,8 @@
       <c r="E25" s="125">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="F25" s="125">
-        <f>SACCR_LambdaCRR(-0.002,0.001,TRUE)</f>
+      <c r="F25" s="125" cm="1">
+        <f t="array" ref="F25">SACCR_LambdaCRR(-0.002,0.001,TRUE)</f>
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="G25" s="126">
@@ -7350,8 +7350,8 @@
       <c r="E26" s="125">
         <v>0</v>
       </c>
-      <c r="F26" s="125">
-        <f>SACCR_LambdaCRR(0.02,0.03,TRUE)</f>
+      <c r="F26" s="125" cm="1">
+        <f t="array" ref="F26">SACCR_LambdaCRR(0.02,0.03,TRUE)</f>
         <v>0</v>
       </c>
       <c r="G26" s="126">
@@ -7373,8 +7373,8 @@
       <c r="E27" s="125">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="F27" s="125">
-        <f>SACCR_LambdaCRR(0.0005,0.01,TRUE)</f>
+      <c r="F27" s="125" cm="1">
+        <f t="array" ref="F27">SACCR_LambdaCRR(0.0005,0.01,TRUE)</f>
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G27" s="126">
@@ -7396,8 +7396,8 @@
       <c r="E28" s="125">
         <v>5.5</v>
       </c>
-      <c r="F28" s="125">
-        <f>SACCR_LambdaCRR(-5,-4,FALSE)</f>
+      <c r="F28" s="125" cm="1">
+        <f t="array" ref="F28">SACCR_LambdaCRR(-5,-4,FALSE)</f>
         <v>5.5</v>
       </c>
       <c r="G28" s="126">
@@ -7419,8 +7419,8 @@
       <c r="E29" s="125">
         <v>0</v>
       </c>
-      <c r="F29" s="125">
-        <f>SACCR_LambdaCRR(40,35,FALSE)</f>
+      <c r="F29" s="125" cm="1">
+        <f t="array" ref="F29">SACCR_LambdaCRR(40,35,FALSE)</f>
         <v>0</v>
       </c>
       <c r="G29" s="126">

</xml_diff>

<commit_message>
Tests: show each unit test's formula with FORMULATEXT
Column D of Tests held each formula of column F as typed text. The text
drifted from the formulas (D18 and D19 showed more decimals than Excel
stores in F18 and F19), followed whatever was typed in it rather than
the test, and editing a cell that starts with "=" makes Excel parse it
as a formula, which fails with a different argument separator. D8:D29
are now FORMULATEXT of the cell beside them, so they always show the
formula actually tested, in the user's own separators.

Validated: python tools/check.py, all gates pass; the 22 cells checked
in the package XML; FORMULATEXT evaluates in LibreOffice. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -6930,8 +6930,9 @@
       <c r="C8" s="128" t="s">
         <v>516</v>
       </c>
-      <c r="D8" s="24" t="s">
-        <v>517</v>
+      <c r="D8" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F8)</f>
+        <v>=SACCR_SupervisoryDuration(0,10)</v>
       </c>
       <c r="E8" s="125">
         <v>7.8693868057473324</v>
@@ -6953,8 +6954,9 @@
       <c r="C9" s="128" t="s">
         <v>518</v>
       </c>
-      <c r="D9" s="24" t="s">
-        <v>519</v>
+      <c r="D9" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F9)</f>
+        <v>=SACCR_SupervisoryDuration(1,11)</v>
       </c>
       <c r="E9" s="125">
         <v>7.4855922824045473</v>
@@ -6976,8 +6978,9 @@
       <c r="C10" s="128" t="s">
         <v>520</v>
       </c>
-      <c r="D10" s="24" t="s">
-        <v>521</v>
+      <c r="D10" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F10)</f>
+        <v>=SACCR_SupervisoryDuration(0,0.01,10/250)</v>
       </c>
       <c r="E10" s="125">
         <v>0.04</v>
@@ -6999,8 +7002,9 @@
       <c r="C11" s="128" t="s">
         <v>522</v>
       </c>
-      <c r="D11" s="24" t="s">
-        <v>523</v>
+      <c r="D11" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F11)</f>
+        <v>=SACCR_MaturityFactor(0.75)</v>
       </c>
       <c r="E11" s="125">
         <v>0.8660254037844386</v>
@@ -7022,8 +7026,9 @@
       <c r="C12" s="128" t="s">
         <v>524</v>
       </c>
-      <c r="D12" s="24" t="s">
-        <v>525</v>
+      <c r="D12" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F12)</f>
+        <v>=SACCR_MaturityFactor(3/365)</v>
       </c>
       <c r="E12" s="125">
         <v>0.2</v>
@@ -7045,8 +7050,9 @@
       <c r="C13" s="128" t="s">
         <v>526</v>
       </c>
-      <c r="D13" s="24" t="s">
-        <v>527</v>
+      <c r="D13" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F13)</f>
+        <v>=SACCR_MaturityFactor(0,TRUE,10)</v>
       </c>
       <c r="E13" s="125">
         <v>0.3</v>
@@ -7068,8 +7074,9 @@
       <c r="C14" s="128" t="s">
         <v>528</v>
       </c>
-      <c r="D14" s="24" t="s">
-        <v>529</v>
+      <c r="D14" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F14)</f>
+        <v>=SACCR_OptionDelta(0.06,0.05,1,0.5,FALSE,TRUE)</v>
       </c>
       <c r="E14" s="125">
         <v>-0.26939521771053271</v>
@@ -7091,8 +7098,9 @@
       <c r="C15" s="128" t="s">
         <v>530</v>
       </c>
-      <c r="D15" s="24" t="s">
-        <v>531</v>
+      <c r="D15" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F15)</f>
+        <v>=SACCR_OptionDelta(100,110,0.5,0.32,TRUE,FALSE)</v>
       </c>
       <c r="E15" s="125">
         <v>-0.37901134582780288</v>
@@ -7114,8 +7122,9 @@
       <c r="C16" s="128" t="s">
         <v>532</v>
       </c>
-      <c r="D16" s="24" t="s">
-        <v>533</v>
+      <c r="D16" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F16)</f>
+        <v>=SACCR_OptionDelta(-0.002,0.001,2,0.5,TRUE,TRUE,0.01)</v>
       </c>
       <c r="E16" s="125">
         <v>0.46143935794124907</v>
@@ -7137,8 +7146,9 @@
       <c r="C17" s="128" t="s">
         <v>534</v>
       </c>
-      <c r="D17" s="24" t="s">
-        <v>535</v>
+      <c r="D17" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F17)</f>
+        <v>=SACCR_CDODelta(0.03,0.06,TRUE)</v>
       </c>
       <c r="E17" s="125">
         <v>5.740967544396816</v>
@@ -7160,8 +7170,9 @@
       <c r="C18" s="128" t="s">
         <v>536</v>
       </c>
-      <c r="D18" s="24" t="s">
-        <v>537</v>
+      <c r="D18" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F18)</f>
+        <v>=SACCR_IREffectiveNotional(0,-36253.8493844036,78693.8680574733)</v>
       </c>
       <c r="E18" s="125">
         <v>59269.963463710403</v>
@@ -7183,8 +7194,9 @@
       <c r="C19" s="128" t="s">
         <v>538</v>
       </c>
-      <c r="D19" s="24" t="s">
-        <v>539</v>
+      <c r="D19" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F19)</f>
+        <v>=SACCR_FactorAggregation({105.861937916956,-279.916321663744,168.111404865732},{0.5,0.5,0.8})</v>
       </c>
       <c r="E19" s="125">
         <v>282.1288318596666</v>
@@ -7206,8 +7218,9 @@
       <c r="C20" s="128" t="s">
         <v>540</v>
       </c>
-      <c r="D20" s="24" t="s">
-        <v>541</v>
+      <c r="D20" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F20)</f>
+        <v>=SACCR_Multiplier(-20,282)</v>
       </c>
       <c r="E20" s="125">
         <v>0.96519268118719448</v>
@@ -7229,8 +7242,9 @@
       <c r="C21" s="128" t="s">
         <v>542</v>
       </c>
-      <c r="D21" s="24" t="s">
-        <v>543</v>
+      <c r="D21" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F21)</f>
+        <v>=SACCR_Multiplier(10,282)</v>
       </c>
       <c r="E21" s="125">
         <v>1</v>
@@ -7252,8 +7266,9 @@
       <c r="C22" s="128" t="s">
         <v>544</v>
       </c>
-      <c r="D22" s="24" t="s">
-        <v>545</v>
+      <c r="D22" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F22)</f>
+        <v>=SACCR_ReplacementCost(5,10,TRUE,0,10,2)</v>
       </c>
       <c r="E22" s="125">
         <v>8</v>
@@ -7275,8 +7290,9 @@
       <c r="C23" s="128" t="s">
         <v>546</v>
       </c>
-      <c r="D23" s="24" t="s">
-        <v>547</v>
+      <c r="D23" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F23)</f>
+        <v>=SACCR_NormCDF(1.96)</v>
       </c>
       <c r="E23" s="125">
         <v>0.97500210485177952</v>
@@ -7298,8 +7314,9 @@
       <c r="C24" s="128" t="s">
         <v>548</v>
       </c>
-      <c r="D24" s="24" t="s">
-        <v>549</v>
+      <c r="D24" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F24)</f>
+        <v>=SACCR_NormCDF(-8)</v>
       </c>
       <c r="E24" s="125">
         <v>6.2209605742718194E-16</v>
@@ -7321,8 +7338,9 @@
       <c r="C25" s="128" t="s">
         <v>550</v>
       </c>
-      <c r="D25" s="24" t="s">
-        <v>551</v>
+      <c r="D25" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F25)</f>
+        <v>=SACCR_LambdaCRR(-0.002,0.001,TRUE)</v>
       </c>
       <c r="E25" s="125">
         <v>3.0000000000000001E-3</v>
@@ -7344,8 +7362,9 @@
       <c r="C26" s="128" t="s">
         <v>552</v>
       </c>
-      <c r="D26" s="24" t="s">
-        <v>553</v>
+      <c r="D26" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F26)</f>
+        <v>=SACCR_LambdaCRR(0.02,0.03,TRUE)</v>
       </c>
       <c r="E26" s="125">
         <v>0</v>
@@ -7367,8 +7386,9 @@
       <c r="C27" s="128" t="s">
         <v>554</v>
       </c>
-      <c r="D27" s="24" t="s">
-        <v>555</v>
+      <c r="D27" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F27)</f>
+        <v>=SACCR_LambdaCRR(0.0005,0.01,TRUE)</v>
       </c>
       <c r="E27" s="125">
         <v>5.0000000000000001E-4</v>
@@ -7390,8 +7410,9 @@
       <c r="C28" s="128" t="s">
         <v>556</v>
       </c>
-      <c r="D28" s="24" t="s">
-        <v>557</v>
+      <c r="D28" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F28)</f>
+        <v>=SACCR_LambdaCRR(-5,-4,FALSE)</v>
       </c>
       <c r="E28" s="125">
         <v>5.5</v>
@@ -7413,8 +7434,9 @@
       <c r="C29" s="128" t="s">
         <v>558</v>
       </c>
-      <c r="D29" s="24" t="s">
-        <v>559</v>
+      <c r="D29" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F29)</f>
+        <v>=SACCR_LambdaCRR(40,35,FALSE)</v>
       </c>
       <c r="E29" s="125">
         <v>0</v>

</xml_diff>

<commit_message>
Tests: formulas without the @ operator, formula column from FORMULATEXT (#162)
Tests F8:F29 are stored as dynamic-array formulas, so Excel 365 no
longer shows them with the implicit-intersection operator. D8:D29 are
FORMULATEXT of column F instead of typed copies, which had drifted (D18,
D19) and could not be edited with a ';' argument separator.

Validated: python tools/check.py, all gates pass. Excel: owner opened
the template; column D shows the formulas in the local separators.
Column F was not evaluated (template without modules).
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -6930,14 +6930,15 @@
       <c r="C8" s="128" t="s">
         <v>516</v>
       </c>
-      <c r="D8" s="24" t="s">
-        <v>517</v>
+      <c r="D8" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F8)</f>
+        <v>=SACCR_SupervisoryDuration(0,10)</v>
       </c>
       <c r="E8" s="125">
         <v>7.8693868057473324</v>
       </c>
-      <c r="F8" s="125">
-        <f>SACCR_SupervisoryDuration(0,10)</f>
+      <c r="F8" s="125" cm="1">
+        <f t="array" ref="F8">SACCR_SupervisoryDuration(0,10)</f>
         <v>7.8693868057473315</v>
       </c>
       <c r="G8" s="126">
@@ -6953,14 +6954,15 @@
       <c r="C9" s="128" t="s">
         <v>518</v>
       </c>
-      <c r="D9" s="24" t="s">
-        <v>519</v>
+      <c r="D9" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F9)</f>
+        <v>=SACCR_SupervisoryDuration(1,11)</v>
       </c>
       <c r="E9" s="125">
         <v>7.4855922824045473</v>
       </c>
-      <c r="F9" s="125">
-        <f>SACCR_SupervisoryDuration(1,11)</f>
+      <c r="F9" s="125" cm="1">
+        <f t="array" ref="F9">SACCR_SupervisoryDuration(1,11)</f>
         <v>7.4855922824045473</v>
       </c>
       <c r="G9" s="126">
@@ -6976,14 +6978,15 @@
       <c r="C10" s="128" t="s">
         <v>520</v>
       </c>
-      <c r="D10" s="24" t="s">
-        <v>521</v>
+      <c r="D10" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F10)</f>
+        <v>=SACCR_SupervisoryDuration(0,0.01,10/250)</v>
       </c>
       <c r="E10" s="125">
         <v>0.04</v>
       </c>
-      <c r="F10" s="125">
-        <f>SACCR_SupervisoryDuration(0,0.01,10/250)</f>
+      <c r="F10" s="125" cm="1">
+        <f t="array" ref="F10">SACCR_SupervisoryDuration(0,0.01,10/250)</f>
         <v>0.04</v>
       </c>
       <c r="G10" s="126">
@@ -6999,14 +7002,15 @@
       <c r="C11" s="128" t="s">
         <v>522</v>
       </c>
-      <c r="D11" s="24" t="s">
-        <v>523</v>
+      <c r="D11" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F11)</f>
+        <v>=SACCR_MaturityFactor(0.75)</v>
       </c>
       <c r="E11" s="125">
         <v>0.8660254037844386</v>
       </c>
-      <c r="F11" s="125">
-        <f>SACCR_MaturityFactor(0.75)</f>
+      <c r="F11" s="125" cm="1">
+        <f t="array" ref="F11">SACCR_MaturityFactor(0.75)</f>
         <v>0.8660254037844386</v>
       </c>
       <c r="G11" s="126">
@@ -7022,14 +7026,15 @@
       <c r="C12" s="128" t="s">
         <v>524</v>
       </c>
-      <c r="D12" s="24" t="s">
-        <v>525</v>
+      <c r="D12" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F12)</f>
+        <v>=SACCR_MaturityFactor(3/365)</v>
       </c>
       <c r="E12" s="125">
         <v>0.2</v>
       </c>
-      <c r="F12" s="125">
-        <f>SACCR_MaturityFactor(3/365)</f>
+      <c r="F12" s="125" cm="1">
+        <f t="array" ref="F12">SACCR_MaturityFactor(3/365)</f>
         <v>0.2</v>
       </c>
       <c r="G12" s="126">
@@ -7045,14 +7050,15 @@
       <c r="C13" s="128" t="s">
         <v>526</v>
       </c>
-      <c r="D13" s="24" t="s">
-        <v>527</v>
+      <c r="D13" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F13)</f>
+        <v>=SACCR_MaturityFactor(0,TRUE,10)</v>
       </c>
       <c r="E13" s="125">
         <v>0.3</v>
       </c>
-      <c r="F13" s="125">
-        <f>SACCR_MaturityFactor(0,TRUE,10)</f>
+      <c r="F13" s="125" cm="1">
+        <f t="array" ref="F13">SACCR_MaturityFactor(0,TRUE,10)</f>
         <v>0.30000000000000004</v>
       </c>
       <c r="G13" s="126">
@@ -7068,14 +7074,15 @@
       <c r="C14" s="128" t="s">
         <v>528</v>
       </c>
-      <c r="D14" s="24" t="s">
-        <v>529</v>
+      <c r="D14" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F14)</f>
+        <v>=SACCR_OptionDelta(0.06,0.05,1,0.5,FALSE,TRUE)</v>
       </c>
       <c r="E14" s="125">
         <v>-0.26939521771053271</v>
       </c>
-      <c r="F14" s="125">
-        <f>SACCR_OptionDelta(0.06,0.05,1,0.5,FALSE,TRUE)</f>
+      <c r="F14" s="125" cm="1">
+        <f t="array" ref="F14">SACCR_OptionDelta(0.06,0.05,1,0.5,FALSE,TRUE)</f>
         <v>-0.26939521771053271</v>
       </c>
       <c r="G14" s="126">
@@ -7091,14 +7098,15 @@
       <c r="C15" s="128" t="s">
         <v>530</v>
       </c>
-      <c r="D15" s="24" t="s">
-        <v>531</v>
+      <c r="D15" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F15)</f>
+        <v>=SACCR_OptionDelta(100,110,0.5,0.32,TRUE,FALSE)</v>
       </c>
       <c r="E15" s="125">
         <v>-0.37901134582780288</v>
       </c>
-      <c r="F15" s="125">
-        <f>SACCR_OptionDelta(100,110,0.5,0.32,TRUE,FALSE)</f>
+      <c r="F15" s="125" cm="1">
+        <f t="array" ref="F15">SACCR_OptionDelta(100,110,0.5,0.32,TRUE,FALSE)</f>
         <v>-0.37901134582780294</v>
       </c>
       <c r="G15" s="126">
@@ -7114,14 +7122,15 @@
       <c r="C16" s="128" t="s">
         <v>532</v>
       </c>
-      <c r="D16" s="24" t="s">
-        <v>533</v>
+      <c r="D16" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F16)</f>
+        <v>=SACCR_OptionDelta(-0.002,0.001,2,0.5,TRUE,TRUE,0.01)</v>
       </c>
       <c r="E16" s="125">
         <v>0.46143935794124907</v>
       </c>
-      <c r="F16" s="125">
-        <f>SACCR_OptionDelta(-0.002,0.001,2,0.5,TRUE,TRUE,0.01)</f>
+      <c r="F16" s="125" cm="1">
+        <f t="array" ref="F16">SACCR_OptionDelta(-0.002,0.001,2,0.5,TRUE,TRUE,0.01)</f>
         <v>0.46143935794124913</v>
       </c>
       <c r="G16" s="126">
@@ -7137,14 +7146,15 @@
       <c r="C17" s="128" t="s">
         <v>534</v>
       </c>
-      <c r="D17" s="24" t="s">
-        <v>535</v>
+      <c r="D17" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F17)</f>
+        <v>=SACCR_CDODelta(0.03,0.06,TRUE)</v>
       </c>
       <c r="E17" s="125">
         <v>5.740967544396816</v>
       </c>
-      <c r="F17" s="125">
-        <f>SACCR_CDODelta(0.03,0.06,TRUE)</f>
+      <c r="F17" s="125" cm="1">
+        <f t="array" ref="F17">SACCR_CDODelta(0.03,0.06,TRUE)</f>
         <v>5.740967544396816</v>
       </c>
       <c r="G17" s="126">
@@ -7160,14 +7170,15 @@
       <c r="C18" s="128" t="s">
         <v>536</v>
       </c>
-      <c r="D18" s="24" t="s">
-        <v>537</v>
+      <c r="D18" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F18)</f>
+        <v>=SACCR_IREffectiveNotional(0,-36253.8493844036,78693.8680574733)</v>
       </c>
       <c r="E18" s="125">
         <v>59269.963463710403</v>
       </c>
-      <c r="F18" s="125">
-        <f>SACCR_IREffectiveNotional(0,-36253.8493844036,78693.8680574733)</f>
+      <c r="F18" s="125" cm="1">
+        <f t="array" ref="F18">SACCR_IREffectiveNotional(0,-36253.8493844036,78693.8680574733)</f>
         <v>59269.963463710395</v>
       </c>
       <c r="G18" s="126">
@@ -7183,14 +7194,15 @@
       <c r="C19" s="128" t="s">
         <v>538</v>
       </c>
-      <c r="D19" s="24" t="s">
-        <v>539</v>
+      <c r="D19" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F19)</f>
+        <v>=SACCR_FactorAggregation({105.861937916956,-279.916321663744,168.111404865732},{0.5,0.5,0.8})</v>
       </c>
       <c r="E19" s="125">
         <v>282.1288318596666</v>
       </c>
-      <c r="F19" s="125">
-        <f>SACCR_FactorAggregation({105.861937916956,-279.916321663744,168.111404865732},{0.5,0.5,0.8})</f>
+      <c r="F19" s="125" cm="1">
+        <f t="array" ref="F19">SACCR_FactorAggregation({105.861937916956,-279.916321663744,168.111404865732},{0.5,0.5,0.8})</f>
         <v>282.12883185966604</v>
       </c>
       <c r="G19" s="126">
@@ -7206,14 +7218,15 @@
       <c r="C20" s="128" t="s">
         <v>540</v>
       </c>
-      <c r="D20" s="24" t="s">
-        <v>541</v>
+      <c r="D20" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F20)</f>
+        <v>=SACCR_Multiplier(-20,282)</v>
       </c>
       <c r="E20" s="125">
         <v>0.96519268118719448</v>
       </c>
-      <c r="F20" s="125">
-        <f>SACCR_Multiplier(-20,282)</f>
+      <c r="F20" s="125" cm="1">
+        <f t="array" ref="F20">SACCR_Multiplier(-20,282)</f>
         <v>0.96519268118719448</v>
       </c>
       <c r="G20" s="126">
@@ -7229,14 +7242,15 @@
       <c r="C21" s="128" t="s">
         <v>542</v>
       </c>
-      <c r="D21" s="24" t="s">
-        <v>543</v>
+      <c r="D21" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F21)</f>
+        <v>=SACCR_Multiplier(10,282)</v>
       </c>
       <c r="E21" s="125">
         <v>1</v>
       </c>
-      <c r="F21" s="125">
-        <f>SACCR_Multiplier(10,282)</f>
+      <c r="F21" s="125" cm="1">
+        <f t="array" ref="F21">SACCR_Multiplier(10,282)</f>
         <v>1</v>
       </c>
       <c r="G21" s="126">
@@ -7252,14 +7266,15 @@
       <c r="C22" s="128" t="s">
         <v>544</v>
       </c>
-      <c r="D22" s="24" t="s">
-        <v>545</v>
+      <c r="D22" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F22)</f>
+        <v>=SACCR_ReplacementCost(5,10,TRUE,0,10,2)</v>
       </c>
       <c r="E22" s="125">
         <v>8</v>
       </c>
-      <c r="F22" s="125">
-        <f>SACCR_ReplacementCost(5,10,TRUE,0,10,2)</f>
+      <c r="F22" s="125" cm="1">
+        <f t="array" ref="F22">SACCR_ReplacementCost(5,10,TRUE,0,10,2)</f>
         <v>8</v>
       </c>
       <c r="G22" s="126">
@@ -7275,14 +7290,15 @@
       <c r="C23" s="128" t="s">
         <v>546</v>
       </c>
-      <c r="D23" s="24" t="s">
-        <v>547</v>
+      <c r="D23" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F23)</f>
+        <v>=SACCR_NormCDF(1.96)</v>
       </c>
       <c r="E23" s="125">
         <v>0.97500210485177952</v>
       </c>
-      <c r="F23" s="125">
-        <f>SACCR_NormCDF(1.96)</f>
+      <c r="F23" s="125" cm="1">
+        <f t="array" ref="F23">SACCR_NormCDF(1.96)</f>
         <v>0.97500210485177952</v>
       </c>
       <c r="G23" s="126">
@@ -7298,14 +7314,15 @@
       <c r="C24" s="128" t="s">
         <v>548</v>
       </c>
-      <c r="D24" s="24" t="s">
-        <v>549</v>
+      <c r="D24" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F24)</f>
+        <v>=SACCR_NormCDF(-8)</v>
       </c>
       <c r="E24" s="125">
         <v>6.2209605742718194E-16</v>
       </c>
-      <c r="F24" s="125">
-        <f>SACCR_NormCDF(-8)</f>
+      <c r="F24" s="125" cm="1">
+        <f t="array" ref="F24">SACCR_NormCDF(-8)</f>
         <v>6.2209605201427843E-16</v>
       </c>
       <c r="G24" s="126">
@@ -7321,14 +7338,15 @@
       <c r="C25" s="128" t="s">
         <v>550</v>
       </c>
-      <c r="D25" s="24" t="s">
-        <v>551</v>
+      <c r="D25" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F25)</f>
+        <v>=SACCR_LambdaCRR(-0.002,0.001,TRUE)</v>
       </c>
       <c r="E25" s="125">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="F25" s="125">
-        <f>SACCR_LambdaCRR(-0.002,0.001,TRUE)</f>
+      <c r="F25" s="125" cm="1">
+        <f t="array" ref="F25">SACCR_LambdaCRR(-0.002,0.001,TRUE)</f>
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="G25" s="126">
@@ -7344,14 +7362,15 @@
       <c r="C26" s="128" t="s">
         <v>552</v>
       </c>
-      <c r="D26" s="24" t="s">
-        <v>553</v>
+      <c r="D26" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F26)</f>
+        <v>=SACCR_LambdaCRR(0.02,0.03,TRUE)</v>
       </c>
       <c r="E26" s="125">
         <v>0</v>
       </c>
-      <c r="F26" s="125">
-        <f>SACCR_LambdaCRR(0.02,0.03,TRUE)</f>
+      <c r="F26" s="125" cm="1">
+        <f t="array" ref="F26">SACCR_LambdaCRR(0.02,0.03,TRUE)</f>
         <v>0</v>
       </c>
       <c r="G26" s="126">
@@ -7367,14 +7386,15 @@
       <c r="C27" s="128" t="s">
         <v>554</v>
       </c>
-      <c r="D27" s="24" t="s">
-        <v>555</v>
+      <c r="D27" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F27)</f>
+        <v>=SACCR_LambdaCRR(0.0005,0.01,TRUE)</v>
       </c>
       <c r="E27" s="125">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="F27" s="125">
-        <f>SACCR_LambdaCRR(0.0005,0.01,TRUE)</f>
+      <c r="F27" s="125" cm="1">
+        <f t="array" ref="F27">SACCR_LambdaCRR(0.0005,0.01,TRUE)</f>
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G27" s="126">
@@ -7390,14 +7410,15 @@
       <c r="C28" s="128" t="s">
         <v>556</v>
       </c>
-      <c r="D28" s="24" t="s">
-        <v>557</v>
+      <c r="D28" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F28)</f>
+        <v>=SACCR_LambdaCRR(-5,-4,FALSE)</v>
       </c>
       <c r="E28" s="125">
         <v>5.5</v>
       </c>
-      <c r="F28" s="125">
-        <f>SACCR_LambdaCRR(-5,-4,FALSE)</f>
+      <c r="F28" s="125" cm="1">
+        <f t="array" ref="F28">SACCR_LambdaCRR(-5,-4,FALSE)</f>
         <v>5.5</v>
       </c>
       <c r="G28" s="126">
@@ -7413,14 +7434,15 @@
       <c r="C29" s="128" t="s">
         <v>558</v>
       </c>
-      <c r="D29" s="24" t="s">
-        <v>559</v>
+      <c r="D29" s="24" t="str">
+        <f>_xlfn.FORMULATEXT(F29)</f>
+        <v>=SACCR_LambdaCRR(40,35,FALSE)</v>
       </c>
       <c r="E29" s="125">
         <v>0</v>
       </c>
-      <c r="F29" s="125">
-        <f>SACCR_LambdaCRR(40,35,FALSE)</f>
+      <c r="F29" s="125" cm="1">
+        <f t="array" ref="F29">SACCR_LambdaCRR(40,35,FALSE)</f>
         <v>0</v>
       </c>
       <c r="G29" s="126">

</xml_diff>

<commit_message>
Tests: one editable tolerance for every unit test
The pass criterion was 1e-9 relative, written into each Result formula.
D5 now holds the tolerance (default 0.001%, input style, validated above
0% and at most 1%) under the workbook name Tests_Tolerance, and every
Result reads it: a row passes when |Function - Expected| is at most the
tolerance times max(1, |Expected|).

Correction to the previous commit: its LibreOffice comparison read the
values cached in the file rather than recalculating. Validated here with
the cached values removed: LibreOffice recalculates all 22 Expected
formulas and they match the Python computation of the rules; with a
substituted function value 7.9e-6 relative off the row passes and with
1.4e-5 it fails. python tools/check.py, all gates pass. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -48,6 +48,7 @@
     <definedName name="SACCR_RunInputs" hidden="1">""</definedName>
     <definedName name="SDFloorBD">Params!$E$13</definedName>
     <definedName name="SF_Table">Params!$C$28:$K$54</definedName>
+    <definedName name="Tests_Tolerance">Tests!$D$5</definedName>
     <definedName name="Trades_Header">Trades!$C$4</definedName>
     <definedName name="VolatilityFactor">Params!$E$18</definedName>
   </definedNames>
@@ -91,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="895">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="896">
   <si>
     <t>SA-CCR Calculator</t>
   </si>
@@ -2788,6 +2789,9 @@
   </si>
   <si>
     <t>Rule</t>
+  </si>
+  <si>
+    <t>Tolerance: a test passes when |Function - Expected| &lt;= tolerance x max(1, |Expected|)</t>
   </si>
 </sst>
 </file>
@@ -3214,7 +3218,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3607,6 +3611,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7017,7 +7024,14 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="128" t="s">
+        <v>895</v>
+      </c>
+      <c r="D5" s="131">
+        <v>1.0000000000000001E-5</v>
+      </c>
+    </row>
     <row r="6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="48" t="s">
         <v>509</v>
@@ -7093,7 +7107,7 @@
         <v>0.0</v>
       </c>
       <c r="O8" s="127" t="str">
-        <f>IF(ISNUMBER(N8),IF(N8&lt;=0.000000001*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N8),IF(N8&lt;=Tests_Tolerance*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P8" s="130" t="s">
@@ -7126,7 +7140,7 @@
         <v>0.0</v>
       </c>
       <c r="O9" s="127" t="str">
-        <f>IF(ISNUMBER(N9),IF(N9&lt;=0.000000001*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N9),IF(N9&lt;=Tests_Tolerance*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P9" s="130" t="s">
@@ -7163,7 +7177,7 @@
         <v>0.0</v>
       </c>
       <c r="O10" s="127" t="str">
-        <f>IF(ISNUMBER(N10),IF(N10&lt;=0.000000001*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N10),IF(N10&lt;=Tests_Tolerance*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P10" s="130" t="s">
@@ -7193,7 +7207,7 @@
         <v>0.0</v>
       </c>
       <c r="O11" s="127" t="str">
-        <f>IF(ISNUMBER(N11),IF(N11&lt;=0.000000001*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N11),IF(N11&lt;=Tests_Tolerance*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P11" s="130" t="s">
@@ -7224,7 +7238,7 @@
         <v>0.0</v>
       </c>
       <c r="O12" s="127" t="str">
-        <f>IF(ISNUMBER(N12),IF(N12&lt;=0.000000001*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N12),IF(N12&lt;=Tests_Tolerance*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P12" s="130" t="s">
@@ -7260,7 +7274,7 @@
         <v>0.0</v>
       </c>
       <c r="O13" s="127" t="str">
-        <f>IF(ISNUMBER(N13),IF(N13&lt;=0.000000001*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N13),IF(N13&lt;=Tests_Tolerance*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P13" s="130" t="s">
@@ -7305,7 +7319,7 @@
         <v>0.0</v>
       </c>
       <c r="O14" s="127" t="str">
-        <f>IF(ISNUMBER(N14),IF(N14&lt;=0.000000001*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N14),IF(N14&lt;=Tests_Tolerance*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P14" s="130" t="s">
@@ -7350,7 +7364,7 @@
         <v>0.0</v>
       </c>
       <c r="O15" s="127" t="str">
-        <f>IF(ISNUMBER(N15),IF(N15&lt;=0.000000001*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N15),IF(N15&lt;=Tests_Tolerance*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P15" s="130" t="s">
@@ -7398,7 +7412,7 @@
         <v>0.0</v>
       </c>
       <c r="O16" s="127" t="str">
-        <f>IF(ISNUMBER(N16),IF(N16&lt;=0.000000001*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N16),IF(N16&lt;=Tests_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P16" s="130" t="s">
@@ -7434,7 +7448,7 @@
         <v>8.881784197001252e-16</v>
       </c>
       <c r="O17" s="127" t="str">
-        <f>IF(ISNUMBER(N17),IF(N17&lt;=0.000000001*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N17),IF(N17&lt;=Tests_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P17" s="130" t="s">
@@ -7470,7 +7484,7 @@
         <v>0.0</v>
       </c>
       <c r="O18" s="127" t="str">
-        <f>IF(ISNUMBER(N18),IF(N18&lt;=0.000000001*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N18),IF(N18&lt;=Tests_Tolerance*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P18" s="130" t="s">
@@ -7515,7 +7529,7 @@
         <v>0.0</v>
       </c>
       <c r="O19" s="127" t="str">
-        <f>IF(ISNUMBER(N19),IF(N19&lt;=0.000000001*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N19),IF(N19&lt;=Tests_Tolerance*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P19" s="130" t="s">
@@ -7548,7 +7562,7 @@
         <v>0.0</v>
       </c>
       <c r="O20" s="127" t="str">
-        <f>IF(ISNUMBER(N20),IF(N20&lt;=0.000000001*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N20),IF(N20&lt;=Tests_Tolerance*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P20" s="130" t="s">
@@ -7581,7 +7595,7 @@
         <v>0.0</v>
       </c>
       <c r="O21" s="127" t="str">
-        <f>IF(ISNUMBER(N21),IF(N21&lt;=0.000000001*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N21),IF(N21&lt;=Tests_Tolerance*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P21" s="130" t="s">
@@ -7626,7 +7640,7 @@
         <v>0.0</v>
       </c>
       <c r="O22" s="127" t="str">
-        <f>IF(ISNUMBER(N22),IF(N22&lt;=0.000000001*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N22),IF(N22&lt;=Tests_Tolerance*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P22" s="130" t="s">
@@ -7656,7 +7670,7 @@
         <v>0.0</v>
       </c>
       <c r="O23" s="127" t="str">
-        <f>IF(ISNUMBER(N23),IF(N23&lt;=0.000000001*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N23),IF(N23&lt;=Tests_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P23" s="130" t="s">
@@ -7686,7 +7700,7 @@
         <v>5.4129035033506995e-24</v>
       </c>
       <c r="O24" s="127" t="str">
-        <f>IF(ISNUMBER(N24),IF(N24&lt;=0.000000001*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N24),IF(N24&lt;=Tests_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P24" s="130" t="s">
@@ -7722,7 +7736,7 @@
         <v>0.0</v>
       </c>
       <c r="O25" s="127" t="str">
-        <f>IF(ISNUMBER(N25),IF(N25&lt;=0.000000001*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N25),IF(N25&lt;=Tests_Tolerance*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P25" s="130" t="s">
@@ -7758,7 +7772,7 @@
         <v>0.0</v>
       </c>
       <c r="O26" s="127" t="str">
-        <f>IF(ISNUMBER(N26),IF(N26&lt;=0.000000001*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N26),IF(N26&lt;=Tests_Tolerance*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P26" s="130" t="s">
@@ -7794,7 +7808,7 @@
         <v>0.0</v>
       </c>
       <c r="O27" s="127" t="str">
-        <f>IF(ISNUMBER(N27),IF(N27&lt;=0.000000001*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N27),IF(N27&lt;=Tests_Tolerance*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P27" s="130" t="s">
@@ -7830,7 +7844,7 @@
         <v>0.0</v>
       </c>
       <c r="O28" s="127" t="str">
-        <f>IF(ISNUMBER(N28),IF(N28&lt;=0.000000001*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N28),IF(N28&lt;=Tests_Tolerance*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P28" s="130" t="s">
@@ -7866,7 +7880,7 @@
         <v>0.0</v>
       </c>
       <c r="O29" s="127" t="str">
-        <f>IF(ISNUMBER(N29),IF(N29&lt;=0.000000001*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N29),IF(N29&lt;=Tests_Tolerance*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P29" s="130" t="s">
@@ -7874,6 +7888,12 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%." sqref="D5">
+      <formula1>0.0000000000000001</formula1>
+      <formula2>0.01</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
 </worksheet>

</xml_diff>

<commit_message>
Tests: Expected formulas apply the functions' boundary rules
Three Expected formulas left out a rule the VBA applies, so a valid
edited input reported FAIL: the supervisory duration floors a negative
start S at 0 (rows 8-10), the multiplier is 1 when the add-on is zero or
negative (rows 20-21), and the IR effective notional floors the sum
under the square root at 0 (row 18). The formulas now apply the same
rules. The other functions already matched; option and CDO deltas
return #NUM! outside their domain, as the Excel formulas do.

Validated: python tools/check.py, all gates pass; LibreOffice with the
cached values removed recalculates the shipped inputs to the same 22
values, gives SD(0, 11) = 8.4610038 for S = -1, E = 11, and 1 for a
zero add-on. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -7095,7 +7095,7 @@
         <v>10</v>
       </c>
       <c r="L8" s="125">
-        <f>(EXP(-0.05*$E8)-EXP(-0.05*$F8))/0.05</f>
+        <f>(EXP(-0.05*MAX($E8,0))-EXP(-0.05*$F8))/0.05</f>
         <v>7.8693868057473315</v>
       </c>
       <c r="M8" s="125" cm="1">
@@ -7128,7 +7128,7 @@
         <v>11</v>
       </c>
       <c r="L9" s="125">
-        <f>(EXP(-0.05*$E9)-EXP(-0.05*$F9))/0.05</f>
+        <f>(EXP(-0.05*MAX($E9,0))-EXP(-0.05*$F9))/0.05</f>
         <v>7.485592282404547</v>
       </c>
       <c r="M9" s="125" cm="1">
@@ -7165,7 +7165,7 @@
         <v>0.04</v>
       </c>
       <c r="L10" s="125">
-        <f>MAX((EXP(-0.05*$E10)-EXP(-0.05*$F10))/0.05,$G10)</f>
+        <f>MAX((EXP(-0.05*MAX($E10,0))-EXP(-0.05*$F10))/0.05,$G10)</f>
         <v>0.04</v>
       </c>
       <c r="M10" s="125" cm="1">
@@ -7472,7 +7472,7 @@
         <v>78693.8680574733</v>
       </c>
       <c r="L18" s="125">
-        <f>SQRT($E18^2+$F18^2+$G18^2+1.4*$E18*$F18+1.4*$F18*$G18+0.6*$E18*$G18)</f>
+        <f>SQRT(MAX($E18^2+$F18^2+$G18^2+1.4*$E18*$F18+1.4*$F18*$G18+0.6*$E18*$G18,0))</f>
         <v>59269.963463710395</v>
       </c>
       <c r="M18" s="125" cm="1">
@@ -7550,7 +7550,7 @@
         <v>282</v>
       </c>
       <c r="L20" s="125">
-        <f>MIN(1,0.05+0.95*EXP($E20/(2*0.95*$F20)))</f>
+        <f>IF($F20&lt;=0,1,MIN(1,0.05+0.95*EXP($E20/(2*0.95*$F20))))</f>
         <v>0.9651926811871945</v>
       </c>
       <c r="M20" s="125" cm="1">
@@ -7583,7 +7583,7 @@
         <v>282</v>
       </c>
       <c r="L21" s="125">
-        <f>MIN(1,0.05+0.95*EXP($E21/(2*0.95*$F21)))</f>
+        <f>IF($F21&lt;=0,1,MIN(1,0.05+0.95*EXP($E21/(2*0.95*$F21))))</f>
         <v>1</v>
       </c>
       <c r="M21" s="125" cm="1">

</xml_diff>

<commit_message>
Tests: expected values from Excel formulas on editable inputs (#163)
The 22 unit tests of the SACCR_* worksheet functions hold their
arguments in input cells (E:K) read by both sides: Expected computes the
rule with Excel's own functions, including the functions' boundary rules,
and Function calls the VBA. One tolerance cell (D5, Tests_Tolerance,
default 0.001%) sets the pass criterion; each row cites its rule.
Workbook guide and CHANGELOG updated.

Validated: python tools/check.py, all gates pass; LibreOffice with cached
values removed recalculates all 22 Expected formulas to the Python
computation of the rules, and the tolerance and boundary probes behave
as specified. Merged on the owner's instruction; no Excel run reported.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -48,6 +48,7 @@
     <definedName name="SACCR_RunInputs" hidden="1">""</definedName>
     <definedName name="SDFloorBD">Params!$E$13</definedName>
     <definedName name="SF_Table">Params!$C$28:$K$54</definedName>
+    <definedName name="Tests_Tolerance">Tests!$D$5</definedName>
     <definedName name="Trades_Header">Trades!$C$4</definedName>
     <definedName name="VolatilityFactor">Params!$E$18</definedName>
   </definedNames>
@@ -91,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="859">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="896">
   <si>
     <t>SA-CCR Calculator</t>
   </si>
@@ -1617,7 +1618,7 @@
     <t>Message</t>
   </si>
   <si>
-    <t>Unit tests call the SACCR_* worksheet functions (macros enabled); portfolio tests are on TestCatalogue.</t>
+    <t>Unit tests call the SACCR_* worksheet functions (macros enabled) on the yellow inputs. Expected computes the same rule with Excel's own functions, so changing an input tests the function on new values. Portfolio tests are on TestCatalogue.</t>
   </si>
   <si>
     <t>Unit tests of the worksheet functions</t>
@@ -2680,6 +2681,117 @@
   </si>
   <si>
     <t>No results yet: build the workbook from the source, then press Run SA-CCR.</t>
+  </si>
+  <si>
+    <t>S, E (years)</t>
+  </si>
+  <si>
+    <t>CRE52.34; CRR Art. 279b(1)(a)</t>
+  </si>
+  <si>
+    <t>S, E, floor (years)</t>
+  </si>
+  <si>
+    <t>M (years)</t>
+  </si>
+  <si>
+    <t>CRE52.48; CRR Art. 279c(1)(a)</t>
+  </si>
+  <si>
+    <t>M (years), margined, MPOR (business days)</t>
+  </si>
+  <si>
+    <t>CRE52.52; CRR Art. 279c(1)(b)</t>
+  </si>
+  <si>
+    <t>P, K, T, volatility, call, bought</t>
+  </si>
+  <si>
+    <t>CRE52.40; CRR Art. 279a(1)(a)</t>
+  </si>
+  <si>
+    <t>P, K, T, volatility, call, bought, lambda</t>
+  </si>
+  <si>
+    <t>CRE52.40 FAQ; CRR-RTS Art. 5(1)</t>
+  </si>
+  <si>
+    <t>A, D, long</t>
+  </si>
+  <si>
+    <t>CRE52.41; CRR Art. 279a(1)(c)</t>
+  </si>
+  <si>
+    <t>D1, D2, D3 (bucket effective notionals)</t>
+  </si>
+  <si>
+    <t>CRE52.57(5); CRR Art. 280a</t>
+  </si>
+  <si>
+    <t>Add-ons A1, A2, A3, correlations 1, 2, 3</t>
+  </si>
+  <si>
+    <t>CRE52.61; CRR Art. 280c</t>
+  </si>
+  <si>
+    <t>V - C, add-on</t>
+  </si>
+  <si>
+    <t>CRE52.23; CRR Art. 278(3)</t>
+  </si>
+  <si>
+    <t>V, C, margined, TH, MTA, NICA</t>
+  </si>
+  <si>
+    <t>CRE52.10, .18; CRR Art. 275(1), (2)</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Standard normal distribution</t>
+  </si>
+  <si>
+    <t>P, K, interest rate</t>
+  </si>
+  <si>
+    <t>CRR-RTS Art. 5(2)</t>
+  </si>
+  <si>
+    <t>Arguments</t>
+  </si>
+  <si>
+    <t>Input 1</t>
+  </si>
+  <si>
+    <t>Input 2</t>
+  </si>
+  <si>
+    <t>Input 3</t>
+  </si>
+  <si>
+    <t>Input 4</t>
+  </si>
+  <si>
+    <t>Input 5</t>
+  </si>
+  <si>
+    <t>Input 6</t>
+  </si>
+  <si>
+    <t>Input 7</t>
+  </si>
+  <si>
+    <t>Expected (Excel)</t>
+  </si>
+  <si>
+    <t>Function (VBA)</t>
+  </si>
+  <si>
+    <t>Rule</t>
+  </si>
+  <si>
+    <t>Tolerance: a test passes when |Function - Expected| &lt;= tolerance x max(1, |Expected|)</t>
   </si>
 </sst>
 </file>
@@ -3106,7 +3218,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3493,6 +3605,15 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6826,11 +6947,14 @@
   <cols>
     <col min="1" max="2" width="4" customWidth="1"/>
     <col min="3" max="3" width="40.75" customWidth="1"/>
-    <col min="4" max="4" width="89.125" customWidth="1"/>
-    <col min="5" max="12" width="14.75" customWidth="1"/>
+    <col min="4" max="4" width="36.75" customWidth="1"/>
+    <col min="5" max="11" width="11.75" customWidth="1"/>
+    <col min="12" max="13" width="14.75" customWidth="1"/>
+    <col min="14" max="15" width="10.75" customWidth="1"/>
+    <col min="16" max="16" width="30.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
@@ -6861,7 +6985,7 @@
       <c r="AA1" s="66"/>
       <c r="AB1" s="66"/>
     </row>
-    <row r="2" spans="2:28" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="30" t="s">
         <v>70</v>
       </c>
@@ -6892,569 +7016,884 @@
       <c r="AA2" s="68"/>
       <c r="AB2" s="68"/>
     </row>
-    <row r="3" spans="2:28" ht="21" x14ac:dyDescent="0.25">
+    <row r="3" ht="21" x14ac:dyDescent="0.25">
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="2" t="s">
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="128" t="s">
+        <v>895</v>
+      </c>
+      <c r="D5" s="131">
+        <v>1.0000000000000001E-5</v>
+      </c>
+    </row>
+    <row r="6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="48" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="7" spans="2:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="54" t="s">
         <v>510</v>
       </c>
       <c r="D7" s="54" t="s">
-        <v>511</v>
+        <v>884</v>
       </c>
       <c r="E7" s="55" t="s">
-        <v>512</v>
+        <v>885</v>
       </c>
       <c r="F7" s="55" t="s">
-        <v>513</v>
+        <v>886</v>
       </c>
       <c r="G7" s="55" t="s">
+        <v>887</v>
+      </c>
+      <c r="H7" s="55" t="s">
+        <v>888</v>
+      </c>
+      <c r="I7" s="55" t="s">
+        <v>889</v>
+      </c>
+      <c r="J7" s="55" t="s">
+        <v>890</v>
+      </c>
+      <c r="K7" s="55" t="s">
+        <v>891</v>
+      </c>
+      <c r="L7" s="55" t="s">
+        <v>892</v>
+      </c>
+      <c r="M7" s="55" t="s">
+        <v>893</v>
+      </c>
+      <c r="N7" s="55" t="s">
         <v>514</v>
       </c>
-      <c r="H7" s="55" t="s">
+      <c r="O7" s="55" t="s">
         <v>515</v>
       </c>
-    </row>
-    <row r="8" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P7" s="54" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="128" t="s">
         <v>516</v>
       </c>
-      <c r="D8" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F8)</f>
-        <v>=SACCR_SupervisoryDuration(0,10)</v>
-      </c>
-      <c r="E8" s="125">
-        <v>7.8693868057473324</v>
-      </c>
-      <c r="F8" s="125" cm="1">
-        <f t="array" ref="F8">SACCR_SupervisoryDuration(0,10)</f>
+      <c r="D8" s="24" t="s">
+        <v>859</v>
+      </c>
+      <c r="E8" s="129">
+        <v>0</v>
+      </c>
+      <c r="F8" s="129">
+        <v>10</v>
+      </c>
+      <c r="L8" s="125">
+        <f>(EXP(-0.05*MAX($E8,0))-EXP(-0.05*$F8))/0.05</f>
         <v>7.8693868057473315</v>
       </c>
-      <c r="G8" s="126">
-        <f t="shared" ref="G8:G29" si="0">IFERROR(ABS(F8-E8),"")</f>
-        <v>8.8817841970012523E-16</v>
-      </c>
-      <c r="H8" s="127" t="str">
-        <f t="shared" ref="H8:H29" si="1">IF(ISNUMBER(G8),IF(G8&lt;=0.000000001*MAX(1,ABS(E8)),"PASS","FAIL"),"FAIL")</f>
+      <c r="M8" s="125" cm="1">
+        <f t="array" ref="M8">SACCR_SupervisoryDuration($E8,$F8)</f>
+        <v>7.8693868057473315</v>
+      </c>
+      <c r="N8" s="126">
+        <f>IFERROR(ABS(M8-L8),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O8" s="127" t="str">
+        <f>IF(ISNUMBER(N8),IF(N8&lt;=Tests_Tolerance*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="9" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P8" s="130" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="128" t="s">
         <v>518</v>
       </c>
-      <c r="D9" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F9)</f>
-        <v>=SACCR_SupervisoryDuration(1,11)</v>
-      </c>
-      <c r="E9" s="125">
-        <v>7.4855922824045473</v>
-      </c>
-      <c r="F9" s="125" cm="1">
-        <f t="array" ref="F9">SACCR_SupervisoryDuration(1,11)</f>
-        <v>7.4855922824045473</v>
-      </c>
-      <c r="G9" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="D9" s="24" t="s">
+        <v>859</v>
+      </c>
+      <c r="E9" s="129">
+        <v>1</v>
+      </c>
+      <c r="F9" s="129">
+        <v>11</v>
+      </c>
+      <c r="L9" s="125">
+        <f>(EXP(-0.05*MAX($E9,0))-EXP(-0.05*$F9))/0.05</f>
+        <v>7.485592282404547</v>
+      </c>
+      <c r="M9" s="125" cm="1">
+        <f t="array" ref="M9">SACCR_SupervisoryDuration($E9,$F9)</f>
+        <v>7.485592282404547</v>
+      </c>
+      <c r="N9" s="126">
+        <f>IFERROR(ABS(M9-L9),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O9" s="127" t="str">
+        <f>IF(ISNUMBER(N9),IF(N9&lt;=Tests_Tolerance*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="10" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P9" s="130" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="128" t="s">
         <v>520</v>
       </c>
-      <c r="D10" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F10)</f>
-        <v>=SACCR_SupervisoryDuration(0,0.01,10/250)</v>
-      </c>
-      <c r="E10" s="125">
+      <c r="D10" s="24" t="s">
+        <v>861</v>
+      </c>
+      <c r="E10" s="129">
+        <v>0</v>
+      </c>
+      <c r="F10" s="129">
+        <v>0.01</v>
+      </c>
+      <c r="G10" s="129">
+        <f>10/250</f>
         <v>0.04</v>
       </c>
-      <c r="F10" s="125" cm="1">
-        <f t="array" ref="F10">SACCR_SupervisoryDuration(0,0.01,10/250)</f>
+      <c r="L10" s="125">
+        <f>MAX((EXP(-0.05*MAX($E10,0))-EXP(-0.05*$F10))/0.05,$G10)</f>
         <v>0.04</v>
       </c>
-      <c r="G10" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H10" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M10" s="125" cm="1">
+        <f t="array" ref="M10">SACCR_SupervisoryDuration($E10,$F10,$G10)</f>
+        <v>0.04</v>
+      </c>
+      <c r="N10" s="126">
+        <f>IFERROR(ABS(M10-L10),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O10" s="127" t="str">
+        <f>IF(ISNUMBER(N10),IF(N10&lt;=Tests_Tolerance*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="11" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P10" s="130" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="128" t="s">
         <v>522</v>
       </c>
-      <c r="D11" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F11)</f>
-        <v>=SACCR_MaturityFactor(0.75)</v>
-      </c>
-      <c r="E11" s="125">
+      <c r="D11" s="24" t="s">
+        <v>862</v>
+      </c>
+      <c r="E11" s="129">
+        <v>0.75</v>
+      </c>
+      <c r="L11" s="125">
+        <f>SQRT(MIN(MAX($E11,10/250),1))</f>
         <v>0.8660254037844386</v>
       </c>
-      <c r="F11" s="125" cm="1">
-        <f t="array" ref="F11">SACCR_MaturityFactor(0.75)</f>
+      <c r="M11" s="125" cm="1">
+        <f t="array" ref="M11">SACCR_MaturityFactor($E11)</f>
         <v>0.8660254037844386</v>
       </c>
-      <c r="G11" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H11" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="N11" s="126">
+        <f>IFERROR(ABS(M11-L11),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O11" s="127" t="str">
+        <f>IF(ISNUMBER(N11),IF(N11&lt;=Tests_Tolerance*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="12" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P11" s="130" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="128" t="s">
         <v>524</v>
       </c>
-      <c r="D12" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F12)</f>
-        <v>=SACCR_MaturityFactor(3/365)</v>
-      </c>
-      <c r="E12" s="125">
+      <c r="D12" s="24" t="s">
+        <v>862</v>
+      </c>
+      <c r="E12" s="129">
+        <f>3/365</f>
+        <v>0.00821917808219178</v>
+      </c>
+      <c r="L12" s="125">
+        <f>SQRT(MIN(MAX($E12,10/250),1))</f>
         <v>0.2</v>
       </c>
-      <c r="F12" s="125" cm="1">
-        <f t="array" ref="F12">SACCR_MaturityFactor(3/365)</f>
+      <c r="M12" s="125" cm="1">
+        <f t="array" ref="M12">SACCR_MaturityFactor($E12)</f>
         <v>0.2</v>
       </c>
-      <c r="G12" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H12" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="N12" s="126">
+        <f>IFERROR(ABS(M12-L12),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O12" s="127" t="str">
+        <f>IF(ISNUMBER(N12),IF(N12&lt;=Tests_Tolerance*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="13" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P12" s="130" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="128" t="s">
         <v>526</v>
       </c>
-      <c r="D13" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F13)</f>
-        <v>=SACCR_MaturityFactor(0,TRUE,10)</v>
-      </c>
-      <c r="E13" s="125">
-        <v>0.3</v>
-      </c>
-      <c r="F13" s="125" cm="1">
-        <f t="array" ref="F13">SACCR_MaturityFactor(0,TRUE,10)</f>
+      <c r="D13" s="24" t="s">
+        <v>864</v>
+      </c>
+      <c r="E13" s="129">
+        <v>0</v>
+      </c>
+      <c r="F13" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="129">
+        <v>10</v>
+      </c>
+      <c r="L13" s="125">
+        <f>IF($F13,1.5*SQRT($G13/250),SQRT(MIN(MAX($E13,10/250),1)))</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="G13" s="126">
-        <f t="shared" si="0"/>
-        <v>5.5511151231257827E-17</v>
-      </c>
-      <c r="H13" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M13" s="125" cm="1">
+        <f t="array" ref="M13">SACCR_MaturityFactor($E13,$F13,$G13)</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="N13" s="126">
+        <f>IFERROR(ABS(M13-L13),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O13" s="127" t="str">
+        <f>IF(ISNUMBER(N13),IF(N13&lt;=Tests_Tolerance*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="14" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P13" s="130" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="128" t="s">
         <v>528</v>
       </c>
-      <c r="D14" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F14)</f>
-        <v>=SACCR_OptionDelta(0.06,0.05,1,0.5,FALSE,TRUE)</v>
-      </c>
-      <c r="E14" s="125">
-        <v>-0.26939521771053271</v>
-      </c>
-      <c r="F14" s="125" cm="1">
-        <f t="array" ref="F14">SACCR_OptionDelta(0.06,0.05,1,0.5,FALSE,TRUE)</f>
-        <v>-0.26939521771053271</v>
-      </c>
-      <c r="G14" s="126">
-        <f t="shared" si="0"/>
+      <c r="D14" s="24" t="s">
+        <v>866</v>
+      </c>
+      <c r="E14" s="129">
+        <v>0.06</v>
+      </c>
+      <c r="F14" s="129">
+        <v>0.05</v>
+      </c>
+      <c r="G14" s="129">
+        <v>1</v>
+      </c>
+      <c r="H14" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="I14" s="129" t="b">
         <v>0</v>
       </c>
-      <c r="H14" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="J14" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="125">
+        <f>IF($I14,_xlfn.NORM.S.DIST((LN(($E14+$K14)/($F14+$K14))+$H14^2*$G14/2)/($H14*SQRT($G14)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E14+$K14)/($F14+$K14))+$H14^2*$G14/2)/($H14*SQRT($G14)),TRUE))*IF($J14,1,-1)</f>
+        <v>-0.2693952177105327</v>
+      </c>
+      <c r="M14" s="125" cm="1">
+        <f t="array" ref="M14">SACCR_OptionDelta($E14,$F14,$G14,$H14,$I14,$J14)</f>
+        <v>-0.2693952177105327</v>
+      </c>
+      <c r="N14" s="126">
+        <f>IFERROR(ABS(M14-L14),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O14" s="127" t="str">
+        <f>IF(ISNUMBER(N14),IF(N14&lt;=Tests_Tolerance*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="15" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P14" s="130" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="128" t="s">
         <v>530</v>
       </c>
-      <c r="D15" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F15)</f>
-        <v>=SACCR_OptionDelta(100,110,0.5,0.32,TRUE,FALSE)</v>
-      </c>
-      <c r="E15" s="125">
-        <v>-0.37901134582780288</v>
-      </c>
-      <c r="F15" s="125" cm="1">
-        <f t="array" ref="F15">SACCR_OptionDelta(100,110,0.5,0.32,TRUE,FALSE)</f>
+      <c r="D15" s="24" t="s">
+        <v>866</v>
+      </c>
+      <c r="E15" s="129">
+        <v>100</v>
+      </c>
+      <c r="F15" s="129">
+        <v>110</v>
+      </c>
+      <c r="G15" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="H15" s="129">
+        <v>0.32</v>
+      </c>
+      <c r="I15" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" s="129" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" s="125">
+        <f>IF($I15,_xlfn.NORM.S.DIST((LN(($E15+$K15)/($F15+$K15))+$H15^2*$G15/2)/($H15*SQRT($G15)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E15+$K15)/($F15+$K15))+$H15^2*$G15/2)/($H15*SQRT($G15)),TRUE))*IF($J15,1,-1)</f>
         <v>-0.37901134582780294</v>
       </c>
-      <c r="G15" s="126">
-        <f t="shared" si="0"/>
-        <v>5.5511151231257827E-17</v>
-      </c>
-      <c r="H15" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M15" s="125" cm="1">
+        <f t="array" ref="M15">SACCR_OptionDelta($E15,$F15,$G15,$H15,$I15,$J15)</f>
+        <v>-0.37901134582780294</v>
+      </c>
+      <c r="N15" s="126">
+        <f>IFERROR(ABS(M15-L15),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O15" s="127" t="str">
+        <f>IF(ISNUMBER(N15),IF(N15&lt;=Tests_Tolerance*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="16" spans="2:28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P15" s="130" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="128" t="s">
         <v>532</v>
       </c>
-      <c r="D16" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F16)</f>
-        <v>=SACCR_OptionDelta(-0.002,0.001,2,0.5,TRUE,TRUE,0.01)</v>
-      </c>
-      <c r="E16" s="125">
-        <v>0.46143935794124907</v>
-      </c>
-      <c r="F16" s="125" cm="1">
-        <f t="array" ref="F16">SACCR_OptionDelta(-0.002,0.001,2,0.5,TRUE,TRUE,0.01)</f>
+      <c r="D16" s="24" t="s">
+        <v>868</v>
+      </c>
+      <c r="E16" s="129">
+        <v>-0.002</v>
+      </c>
+      <c r="F16" s="129">
+        <v>0.001</v>
+      </c>
+      <c r="G16" s="129">
+        <v>2</v>
+      </c>
+      <c r="H16" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="I16" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" s="129">
+        <v>0.01</v>
+      </c>
+      <c r="L16" s="125">
+        <f>IF($I16,_xlfn.NORM.S.DIST((LN(($E16+$K16)/($F16+$K16))+$H16^2*$G16/2)/($H16*SQRT($G16)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E16+$K16)/($F16+$K16))+$H16^2*$G16/2)/($H16*SQRT($G16)),TRUE))*IF($J16,1,-1)</f>
         <v>0.46143935794124913</v>
       </c>
-      <c r="G16" s="126">
-        <f t="shared" si="0"/>
-        <v>5.5511151231257827E-17</v>
-      </c>
-      <c r="H16" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M16" s="125" cm="1">
+        <f t="array" ref="M16">SACCR_OptionDelta($E16,$F16,$G16,$H16,$I16,$J16,$K16)</f>
+        <v>0.46143935794124913</v>
+      </c>
+      <c r="N16" s="126">
+        <f>IFERROR(ABS(M16-L16),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O16" s="127" t="str">
+        <f>IF(ISNUMBER(N16),IF(N16&lt;=Tests_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="17" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P16" s="130" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="128" t="s">
         <v>534</v>
       </c>
-      <c r="D17" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F17)</f>
-        <v>=SACCR_CDODelta(0.03,0.06,TRUE)</v>
-      </c>
-      <c r="E17" s="125">
+      <c r="D17" s="24" t="s">
+        <v>870</v>
+      </c>
+      <c r="E17" s="129">
+        <v>0.03</v>
+      </c>
+      <c r="F17" s="129">
+        <v>0.06</v>
+      </c>
+      <c r="G17" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" s="125">
+        <f>15/((1+14*$E17)*(1+14*$F17))*IF($G17,1,-1)</f>
+        <v>5.740967544396817</v>
+      </c>
+      <c r="M17" s="125" cm="1">
+        <f t="array" ref="M17">SACCR_CDODelta($E17,$F17,$G17)</f>
         <v>5.740967544396816</v>
       </c>
-      <c r="F17" s="125" cm="1">
-        <f t="array" ref="F17">SACCR_CDODelta(0.03,0.06,TRUE)</f>
-        <v>5.740967544396816</v>
-      </c>
-      <c r="G17" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H17" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="N17" s="126">
+        <f>IFERROR(ABS(M17-L17),"")</f>
+        <v>8.881784197001252e-16</v>
+      </c>
+      <c r="O17" s="127" t="str">
+        <f>IF(ISNUMBER(N17),IF(N17&lt;=Tests_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="18" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P17" s="130" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="128" t="s">
         <v>536</v>
       </c>
-      <c r="D18" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F18)</f>
-        <v>=SACCR_IREffectiveNotional(0,-36253.8493844036,78693.8680574733)</v>
-      </c>
-      <c r="E18" s="125">
-        <v>59269.963463710403</v>
-      </c>
-      <c r="F18" s="125" cm="1">
-        <f t="array" ref="F18">SACCR_IREffectiveNotional(0,-36253.8493844036,78693.8680574733)</f>
+      <c r="D18" s="24" t="s">
+        <v>872</v>
+      </c>
+      <c r="E18" s="129">
+        <v>0</v>
+      </c>
+      <c r="F18" s="129">
+        <v>-36253.8493844036</v>
+      </c>
+      <c r="G18" s="129">
+        <v>78693.8680574733</v>
+      </c>
+      <c r="L18" s="125">
+        <f>SQRT(MAX($E18^2+$F18^2+$G18^2+1.4*$E18*$F18+1.4*$F18*$G18+0.6*$E18*$G18,0))</f>
         <v>59269.963463710395</v>
       </c>
-      <c r="G18" s="126">
-        <f t="shared" si="0"/>
-        <v>7.2759576141834259E-12</v>
-      </c>
-      <c r="H18" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M18" s="125" cm="1">
+        <f t="array" ref="M18">SACCR_IREffectiveNotional($E18,$F18,$G18)</f>
+        <v>59269.963463710395</v>
+      </c>
+      <c r="N18" s="126">
+        <f>IFERROR(ABS(M18-L18),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O18" s="127" t="str">
+        <f>IF(ISNUMBER(N18),IF(N18&lt;=Tests_Tolerance*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="19" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P18" s="130" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="128" t="s">
         <v>538</v>
       </c>
-      <c r="D19" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F19)</f>
-        <v>=SACCR_FactorAggregation({105.861937916956,-279.916321663744,168.111404865732},{0.5,0.5,0.8})</v>
-      </c>
-      <c r="E19" s="125">
-        <v>282.1288318596666</v>
-      </c>
-      <c r="F19" s="125" cm="1">
-        <f t="array" ref="F19">SACCR_FactorAggregation({105.861937916956,-279.916321663744,168.111404865732},{0.5,0.5,0.8})</f>
+      <c r="D19" s="24" t="s">
+        <v>874</v>
+      </c>
+      <c r="E19" s="129">
+        <v>105.861937916956</v>
+      </c>
+      <c r="F19" s="129">
+        <v>-279.916321663744</v>
+      </c>
+      <c r="G19" s="129">
+        <v>168.111404865732</v>
+      </c>
+      <c r="H19" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="I19" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="J19" s="129">
+        <v>0.8</v>
+      </c>
+      <c r="L19" s="125">
+        <f>SQRT(SUMPRODUCT($E19:$G19,$H19:$J19)^2+SUMPRODUCT((1-$H19:$J19^2)*$E19:$G19^2))</f>
         <v>282.12883185966604</v>
       </c>
-      <c r="G19" s="126">
-        <f t="shared" si="0"/>
-        <v>5.6843418860808015E-13</v>
-      </c>
-      <c r="H19" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M19" s="125" cm="1">
+        <f t="array" ref="M19">SACCR_FactorAggregation($E19:$G19,$H19:$J19)</f>
+        <v>282.12883185966604</v>
+      </c>
+      <c r="N19" s="126">
+        <f>IFERROR(ABS(M19-L19),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O19" s="127" t="str">
+        <f>IF(ISNUMBER(N19),IF(N19&lt;=Tests_Tolerance*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="20" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P19" s="130" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="128" t="s">
         <v>540</v>
       </c>
-      <c r="D20" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F20)</f>
-        <v>=SACCR_Multiplier(-20,282)</v>
-      </c>
-      <c r="E20" s="125">
-        <v>0.96519268118719448</v>
-      </c>
-      <c r="F20" s="125" cm="1">
-        <f t="array" ref="F20">SACCR_Multiplier(-20,282)</f>
-        <v>0.96519268118719448</v>
-      </c>
-      <c r="G20" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H20" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="D20" s="24" t="s">
+        <v>876</v>
+      </c>
+      <c r="E20" s="129">
+        <v>-20</v>
+      </c>
+      <c r="F20" s="129">
+        <v>282</v>
+      </c>
+      <c r="L20" s="125">
+        <f>IF($F20&lt;=0,1,MIN(1,0.05+0.95*EXP($E20/(2*0.95*$F20))))</f>
+        <v>0.9651926811871945</v>
+      </c>
+      <c r="M20" s="125" cm="1">
+        <f t="array" ref="M20">SACCR_Multiplier($E20,$F20)</f>
+        <v>0.9651926811871945</v>
+      </c>
+      <c r="N20" s="126">
+        <f>IFERROR(ABS(M20-L20),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O20" s="127" t="str">
+        <f>IF(ISNUMBER(N20),IF(N20&lt;=Tests_Tolerance*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="21" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P20" s="130" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="128" t="s">
         <v>542</v>
       </c>
-      <c r="D21" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F21)</f>
-        <v>=SACCR_Multiplier(10,282)</v>
-      </c>
-      <c r="E21" s="125">
+      <c r="D21" s="24" t="s">
+        <v>876</v>
+      </c>
+      <c r="E21" s="129">
+        <v>10</v>
+      </c>
+      <c r="F21" s="129">
+        <v>282</v>
+      </c>
+      <c r="L21" s="125">
+        <f>IF($F21&lt;=0,1,MIN(1,0.05+0.95*EXP($E21/(2*0.95*$F21))))</f>
         <v>1</v>
       </c>
-      <c r="F21" s="125" cm="1">
-        <f t="array" ref="F21">SACCR_Multiplier(10,282)</f>
-        <v>1</v>
-      </c>
-      <c r="G21" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H21" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M21" s="125" cm="1">
+        <f t="array" ref="M21">SACCR_Multiplier($E21,$F21)</f>
+        <v>1.0</v>
+      </c>
+      <c r="N21" s="126">
+        <f>IFERROR(ABS(M21-L21),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O21" s="127" t="str">
+        <f>IF(ISNUMBER(N21),IF(N21&lt;=Tests_Tolerance*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="22" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P21" s="130" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="22" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="128" t="s">
         <v>544</v>
       </c>
-      <c r="D22" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F22)</f>
-        <v>=SACCR_ReplacementCost(5,10,TRUE,0,10,2)</v>
-      </c>
-      <c r="E22" s="125">
+      <c r="D22" s="24" t="s">
+        <v>878</v>
+      </c>
+      <c r="E22" s="129">
+        <v>5</v>
+      </c>
+      <c r="F22" s="129">
+        <v>10</v>
+      </c>
+      <c r="G22" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="129">
+        <v>0</v>
+      </c>
+      <c r="I22" s="129">
+        <v>10</v>
+      </c>
+      <c r="J22" s="129">
+        <v>2</v>
+      </c>
+      <c r="L22" s="125">
+        <f>IF($G22,MAX($E22-$F22,$H22+$I22-$J22,0),MAX($E22-$F22,0))</f>
         <v>8</v>
       </c>
-      <c r="F22" s="125" cm="1">
-        <f t="array" ref="F22">SACCR_ReplacementCost(5,10,TRUE,0,10,2)</f>
-        <v>8</v>
-      </c>
-      <c r="G22" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H22" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M22" s="125" cm="1">
+        <f t="array" ref="M22">SACCR_ReplacementCost($E22,$F22,$G22,$H22,$I22,$J22)</f>
+        <v>8.0</v>
+      </c>
+      <c r="N22" s="126">
+        <f>IFERROR(ABS(M22-L22),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O22" s="127" t="str">
+        <f>IF(ISNUMBER(N22),IF(N22&lt;=Tests_Tolerance*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="23" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P22" s="130" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="128" t="s">
         <v>546</v>
       </c>
-      <c r="D23" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F23)</f>
-        <v>=SACCR_NormCDF(1.96)</v>
-      </c>
-      <c r="E23" s="125">
-        <v>0.97500210485177952</v>
-      </c>
-      <c r="F23" s="125" cm="1">
-        <f t="array" ref="F23">SACCR_NormCDF(1.96)</f>
-        <v>0.97500210485177952</v>
-      </c>
-      <c r="G23" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H23" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="D23" s="24" t="s">
+        <v>880</v>
+      </c>
+      <c r="E23" s="129">
+        <v>1.96</v>
+      </c>
+      <c r="L23" s="125">
+        <f>_xlfn.NORM.S.DIST($E23,TRUE)</f>
+        <v>0.9750021048517795</v>
+      </c>
+      <c r="M23" s="125" cm="1">
+        <f t="array" ref="M23">SACCR_NormCDF($E23)</f>
+        <v>0.9750021048517795</v>
+      </c>
+      <c r="N23" s="126">
+        <f>IFERROR(ABS(M23-L23),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O23" s="127" t="str">
+        <f>IF(ISNUMBER(N23),IF(N23&lt;=Tests_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="24" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P23" s="130" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="128" t="s">
         <v>548</v>
       </c>
-      <c r="D24" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F24)</f>
-        <v>=SACCR_NormCDF(-8)</v>
-      </c>
-      <c r="E24" s="125">
-        <v>6.2209605742718194E-16</v>
-      </c>
-      <c r="F24" s="125" cm="1">
-        <f t="array" ref="F24">SACCR_NormCDF(-8)</f>
-        <v>6.2209605201427843E-16</v>
-      </c>
-      <c r="G24" s="126">
-        <f t="shared" si="0"/>
-        <v>5.4129035033506995E-24</v>
-      </c>
-      <c r="H24" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="D24" s="24" t="s">
+        <v>880</v>
+      </c>
+      <c r="E24" s="129">
+        <v>-8</v>
+      </c>
+      <c r="L24" s="125">
+        <f>_xlfn.NORM.S.DIST($E24,TRUE)</f>
+        <v>6.220960574271819e-16</v>
+      </c>
+      <c r="M24" s="125" cm="1">
+        <f t="array" ref="M24">SACCR_NormCDF($E24)</f>
+        <v>6.220960520142784e-16</v>
+      </c>
+      <c r="N24" s="126">
+        <f>IFERROR(ABS(M24-L24),"")</f>
+        <v>5.4129035033506995e-24</v>
+      </c>
+      <c r="O24" s="127" t="str">
+        <f>IF(ISNUMBER(N24),IF(N24&lt;=Tests_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="25" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P24" s="130" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="128" t="s">
         <v>550</v>
       </c>
-      <c r="D25" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F25)</f>
-        <v>=SACCR_LambdaCRR(-0.002,0.001,TRUE)</v>
-      </c>
-      <c r="E25" s="125">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="F25" s="125" cm="1">
-        <f t="array" ref="F25">SACCR_LambdaCRR(-0.002,0.001,TRUE)</f>
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="G25" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H25" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="D25" s="24" t="s">
+        <v>882</v>
+      </c>
+      <c r="E25" s="129">
+        <v>-0.002</v>
+      </c>
+      <c r="F25" s="129">
+        <v>0.001</v>
+      </c>
+      <c r="G25" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" s="125">
+        <f>IF($G25,MAX(0.001-MIN($E25,$F25),0),MAX(-(1+0.1)*MIN($E25,$F25),0))</f>
+        <v>0.003</v>
+      </c>
+      <c r="M25" s="125" cm="1">
+        <f t="array" ref="M25">SACCR_LambdaCRR($E25,$F25,$G25)</f>
+        <v>0.003</v>
+      </c>
+      <c r="N25" s="126">
+        <f>IFERROR(ABS(M25-L25),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O25" s="127" t="str">
+        <f>IF(ISNUMBER(N25),IF(N25&lt;=Tests_Tolerance*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="26" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P25" s="130" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="26" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="128" t="s">
         <v>552</v>
       </c>
-      <c r="D26" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F26)</f>
-        <v>=SACCR_LambdaCRR(0.02,0.03,TRUE)</v>
-      </c>
-      <c r="E26" s="125">
+      <c r="D26" s="24" t="s">
+        <v>882</v>
+      </c>
+      <c r="E26" s="129">
+        <v>0.02</v>
+      </c>
+      <c r="F26" s="129">
+        <v>0.03</v>
+      </c>
+      <c r="G26" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" s="125">
+        <f>IF($G26,MAX(0.001-MIN($E26,$F26),0),MAX(-(1+0.1)*MIN($E26,$F26),0))</f>
         <v>0</v>
       </c>
-      <c r="F26" s="125" cm="1">
-        <f t="array" ref="F26">SACCR_LambdaCRR(0.02,0.03,TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="G26" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H26" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M26" s="125" cm="1">
+        <f t="array" ref="M26">SACCR_LambdaCRR($E26,$F26,$G26)</f>
+        <v>0.0</v>
+      </c>
+      <c r="N26" s="126">
+        <f>IFERROR(ABS(M26-L26),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O26" s="127" t="str">
+        <f>IF(ISNUMBER(N26),IF(N26&lt;=Tests_Tolerance*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="27" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P26" s="130" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="27" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="128" t="s">
         <v>554</v>
       </c>
-      <c r="D27" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F27)</f>
-        <v>=SACCR_LambdaCRR(0.0005,0.01,TRUE)</v>
-      </c>
-      <c r="E27" s="125">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="F27" s="125" cm="1">
-        <f t="array" ref="F27">SACCR_LambdaCRR(0.0005,0.01,TRUE)</f>
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="G27" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H27" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="D27" s="24" t="s">
+        <v>882</v>
+      </c>
+      <c r="E27" s="129">
+        <v>0.0005</v>
+      </c>
+      <c r="F27" s="129">
+        <v>0.01</v>
+      </c>
+      <c r="G27" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" s="125">
+        <f>IF($G27,MAX(0.001-MIN($E27,$F27),0),MAX(-(1+0.1)*MIN($E27,$F27),0))</f>
+        <v>0.0005</v>
+      </c>
+      <c r="M27" s="125" cm="1">
+        <f t="array" ref="M27">SACCR_LambdaCRR($E27,$F27,$G27)</f>
+        <v>0.0005</v>
+      </c>
+      <c r="N27" s="126">
+        <f>IFERROR(ABS(M27-L27),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O27" s="127" t="str">
+        <f>IF(ISNUMBER(N27),IF(N27&lt;=Tests_Tolerance*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="28" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P27" s="130" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C28" s="128" t="s">
         <v>556</v>
       </c>
-      <c r="D28" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F28)</f>
-        <v>=SACCR_LambdaCRR(-5,-4,FALSE)</v>
-      </c>
-      <c r="E28" s="125">
+      <c r="D28" s="24" t="s">
+        <v>882</v>
+      </c>
+      <c r="E28" s="129">
+        <v>-5</v>
+      </c>
+      <c r="F28" s="129">
+        <v>-4</v>
+      </c>
+      <c r="G28" s="129" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" s="125">
+        <f>IF($G28,MAX(0.001-MIN($E28,$F28),0),MAX(-(1+0.1)*MIN($E28,$F28),0))</f>
         <v>5.5</v>
       </c>
-      <c r="F28" s="125" cm="1">
-        <f t="array" ref="F28">SACCR_LambdaCRR(-5,-4,FALSE)</f>
+      <c r="M28" s="125" cm="1">
+        <f t="array" ref="M28">SACCR_LambdaCRR($E28,$F28,$G28)</f>
         <v>5.5</v>
       </c>
-      <c r="G28" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H28" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="N28" s="126">
+        <f>IFERROR(ABS(M28-L28),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O28" s="127" t="str">
+        <f>IF(ISNUMBER(N28),IF(N28&lt;=Tests_Tolerance*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
-    </row>
-    <row r="29" spans="3:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P28" s="130" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C29" s="128" t="s">
         <v>558</v>
       </c>
-      <c r="D29" s="24" t="str">
-        <f>_xlfn.FORMULATEXT(F29)</f>
-        <v>=SACCR_LambdaCRR(40,35,FALSE)</v>
-      </c>
-      <c r="E29" s="125">
+      <c r="D29" s="24" t="s">
+        <v>882</v>
+      </c>
+      <c r="E29" s="129">
+        <v>40</v>
+      </c>
+      <c r="F29" s="129">
+        <v>35</v>
+      </c>
+      <c r="G29" s="129" t="b">
         <v>0</v>
       </c>
-      <c r="F29" s="125" cm="1">
-        <f t="array" ref="F29">SACCR_LambdaCRR(40,35,FALSE)</f>
+      <c r="L29" s="125">
+        <f>IF($G29,MAX(0.001-MIN($E29,$F29),0),MAX(-(1+0.1)*MIN($E29,$F29),0))</f>
         <v>0</v>
       </c>
-      <c r="G29" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H29" s="127" t="str">
-        <f t="shared" si="1"/>
+      <c r="M29" s="125" cm="1">
+        <f t="array" ref="M29">SACCR_LambdaCRR($E29,$F29,$G29)</f>
+        <v>0.0</v>
+      </c>
+      <c r="N29" s="126">
+        <f>IFERROR(ABS(M29-L29),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O29" s="127" t="str">
+        <f>IF(ISNUMBER(N29),IF(N29&lt;=Tests_Tolerance*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
+      <c r="P29" s="130" t="s">
+        <v>883</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%." sqref="D5">
+      <formula1>0.0000000000000001</formula1>
+      <formula2>0.01</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
 </worksheet>

</xml_diff>

<commit_message>
Rename the Tests sheet to FormulaTest
The sheet tests the SACCR_* worksheet functions, and "Tests" did not
say which tests next to TestCatalogue and the VBA test suites. The sheet
is now FormulaTest with the title "Formula tests"; the tolerance name
becomes FormulaTest_Tolerance and the 22 Result formulas use it. The
README sheet list (C46) and description (D11) and the Basel_vs_CRR
reference (J18) name the new sheet. The code name stays shTests, so the
document module and existing development workbooks are unaffected.
Workbook guide and the CHANGELOG entry updated.

Validated: python tools/check.py, all gates pass; no VBA refers to the
sheet by name; LibreOffice opens the sheet as FormulaTest and, with the
cached values removed, a Result formula evaluates through
FormulaTest_Tolerance. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -17,7 +17,7 @@
     <sheet name="TradeCalc" sheetId="8" r:id="rId8"/>
     <sheet name="Checks" sheetId="9" r:id="rId9"/>
     <sheet name="TestCatalogue" sheetId="10" r:id="rId10"/>
-    <sheet name="Tests" sheetId="11" r:id="rId11"/>
+    <sheet name="FormulaTest" sheetId="11" r:id="rId11"/>
     <sheet name="Basel_vs_CRR" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
@@ -28,6 +28,7 @@
     <definedName name="BasisFactor">Params!$E$17</definedName>
     <definedName name="BusinessDaysPerYear">Params!$E$11</definedName>
     <definedName name="DaysPerYear">Params!$E$10</definedName>
+    <definedName name="FormulaTest_Tolerance">FormulaTest!$D$5</definedName>
     <definedName name="FX_Table">Params!$C$57:$E$62</definedName>
     <definedName name="IRBucketOffset">Params!$E$22</definedName>
     <definedName name="IRCorrBucket12">Params!$E$19</definedName>
@@ -48,7 +49,6 @@
     <definedName name="SACCR_RunInputs" hidden="1">""</definedName>
     <definedName name="SDFloorBD">Params!$E$13</definedName>
     <definedName name="SF_Table">Params!$C$28:$K$54</definedName>
-    <definedName name="Tests_Tolerance">Tests!$D$5</definedName>
     <definedName name="Trades_Header">Trades!$C$4</definedName>
     <definedName name="VolatilityFactor">Params!$E$18</definedName>
   </definedNames>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="898">
   <si>
     <t>SA-CCR Calculator</t>
   </si>
@@ -136,7 +136,7 @@
     <t>6. Review</t>
   </si>
   <si>
-    <t>Checks lists every excluded trade and warning. TestCatalogue compares the engine with published / hand-calculated reference values per regime; Tests unit-tests the formula functions.</t>
+    <t>Checks lists every excluded trade and warning. TestCatalogue compares the engine with published / hand-calculated reference values per regime; FormulaTest unit-tests the formula functions.</t>
   </si>
   <si>
     <t>7. Regime</t>
@@ -2338,7 +2338,7 @@
     <t>Common table on Params.</t>
   </si>
   <si>
-    <t>Tests sheet</t>
+    <t>FormulaTest sheet</t>
   </si>
   <si>
     <t>Credit supervisory factors</t>
@@ -2792,6 +2792,12 @@
   </si>
   <si>
     <t>Tolerance: a test passes when |Function - Expected| &lt;= tolerance x max(1, |Expected|)</t>
+  </si>
+  <si>
+    <t>FormulaTest</t>
+  </si>
+  <si>
+    <t>Formula tests</t>
   </si>
 </sst>
 </file>
@@ -5000,7 +5006,7 @@
     </row>
     <row r="46" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C46" s="25" t="s">
-        <v>70</v>
+        <v>896</v>
       </c>
       <c r="D46" s="34" t="s">
         <v>71</v>
@@ -6987,7 +6993,7 @@
     </row>
     <row r="2" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="30" t="s">
-        <v>70</v>
+        <v>897</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="32"/>
@@ -7107,7 +7113,7 @@
         <v>0.0</v>
       </c>
       <c r="O8" s="127" t="str">
-        <f>IF(ISNUMBER(N8),IF(N8&lt;=Tests_Tolerance*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N8),IF(N8&lt;=FormulaTest_Tolerance*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P8" s="130" t="s">
@@ -7140,7 +7146,7 @@
         <v>0.0</v>
       </c>
       <c r="O9" s="127" t="str">
-        <f>IF(ISNUMBER(N9),IF(N9&lt;=Tests_Tolerance*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N9),IF(N9&lt;=FormulaTest_Tolerance*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P9" s="130" t="s">
@@ -7177,7 +7183,7 @@
         <v>0.0</v>
       </c>
       <c r="O10" s="127" t="str">
-        <f>IF(ISNUMBER(N10),IF(N10&lt;=Tests_Tolerance*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N10),IF(N10&lt;=FormulaTest_Tolerance*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P10" s="130" t="s">
@@ -7207,7 +7213,7 @@
         <v>0.0</v>
       </c>
       <c r="O11" s="127" t="str">
-        <f>IF(ISNUMBER(N11),IF(N11&lt;=Tests_Tolerance*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N11),IF(N11&lt;=FormulaTest_Tolerance*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P11" s="130" t="s">
@@ -7238,7 +7244,7 @@
         <v>0.0</v>
       </c>
       <c r="O12" s="127" t="str">
-        <f>IF(ISNUMBER(N12),IF(N12&lt;=Tests_Tolerance*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N12),IF(N12&lt;=FormulaTest_Tolerance*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P12" s="130" t="s">
@@ -7274,7 +7280,7 @@
         <v>0.0</v>
       </c>
       <c r="O13" s="127" t="str">
-        <f>IF(ISNUMBER(N13),IF(N13&lt;=Tests_Tolerance*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N13),IF(N13&lt;=FormulaTest_Tolerance*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P13" s="130" t="s">
@@ -7319,7 +7325,7 @@
         <v>0.0</v>
       </c>
       <c r="O14" s="127" t="str">
-        <f>IF(ISNUMBER(N14),IF(N14&lt;=Tests_Tolerance*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N14),IF(N14&lt;=FormulaTest_Tolerance*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P14" s="130" t="s">
@@ -7364,7 +7370,7 @@
         <v>0.0</v>
       </c>
       <c r="O15" s="127" t="str">
-        <f>IF(ISNUMBER(N15),IF(N15&lt;=Tests_Tolerance*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N15),IF(N15&lt;=FormulaTest_Tolerance*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P15" s="130" t="s">
@@ -7412,7 +7418,7 @@
         <v>0.0</v>
       </c>
       <c r="O16" s="127" t="str">
-        <f>IF(ISNUMBER(N16),IF(N16&lt;=Tests_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N16),IF(N16&lt;=FormulaTest_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P16" s="130" t="s">
@@ -7448,7 +7454,7 @@
         <v>8.881784197001252e-16</v>
       </c>
       <c r="O17" s="127" t="str">
-        <f>IF(ISNUMBER(N17),IF(N17&lt;=Tests_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N17),IF(N17&lt;=FormulaTest_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P17" s="130" t="s">
@@ -7484,7 +7490,7 @@
         <v>0.0</v>
       </c>
       <c r="O18" s="127" t="str">
-        <f>IF(ISNUMBER(N18),IF(N18&lt;=Tests_Tolerance*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N18),IF(N18&lt;=FormulaTest_Tolerance*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P18" s="130" t="s">
@@ -7529,7 +7535,7 @@
         <v>0.0</v>
       </c>
       <c r="O19" s="127" t="str">
-        <f>IF(ISNUMBER(N19),IF(N19&lt;=Tests_Tolerance*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N19),IF(N19&lt;=FormulaTest_Tolerance*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P19" s="130" t="s">
@@ -7562,7 +7568,7 @@
         <v>0.0</v>
       </c>
       <c r="O20" s="127" t="str">
-        <f>IF(ISNUMBER(N20),IF(N20&lt;=Tests_Tolerance*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N20),IF(N20&lt;=FormulaTest_Tolerance*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P20" s="130" t="s">
@@ -7595,7 +7601,7 @@
         <v>0.0</v>
       </c>
       <c r="O21" s="127" t="str">
-        <f>IF(ISNUMBER(N21),IF(N21&lt;=Tests_Tolerance*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N21),IF(N21&lt;=FormulaTest_Tolerance*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P21" s="130" t="s">
@@ -7640,7 +7646,7 @@
         <v>0.0</v>
       </c>
       <c r="O22" s="127" t="str">
-        <f>IF(ISNUMBER(N22),IF(N22&lt;=Tests_Tolerance*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N22),IF(N22&lt;=FormulaTest_Tolerance*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P22" s="130" t="s">
@@ -7670,7 +7676,7 @@
         <v>0.0</v>
       </c>
       <c r="O23" s="127" t="str">
-        <f>IF(ISNUMBER(N23),IF(N23&lt;=Tests_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N23),IF(N23&lt;=FormulaTest_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P23" s="130" t="s">
@@ -7700,7 +7706,7 @@
         <v>5.4129035033506995e-24</v>
       </c>
       <c r="O24" s="127" t="str">
-        <f>IF(ISNUMBER(N24),IF(N24&lt;=Tests_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N24),IF(N24&lt;=FormulaTest_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P24" s="130" t="s">
@@ -7736,7 +7742,7 @@
         <v>0.0</v>
       </c>
       <c r="O25" s="127" t="str">
-        <f>IF(ISNUMBER(N25),IF(N25&lt;=Tests_Tolerance*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N25),IF(N25&lt;=FormulaTest_Tolerance*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P25" s="130" t="s">
@@ -7772,7 +7778,7 @@
         <v>0.0</v>
       </c>
       <c r="O26" s="127" t="str">
-        <f>IF(ISNUMBER(N26),IF(N26&lt;=Tests_Tolerance*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N26),IF(N26&lt;=FormulaTest_Tolerance*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P26" s="130" t="s">
@@ -7808,7 +7814,7 @@
         <v>0.0</v>
       </c>
       <c r="O27" s="127" t="str">
-        <f>IF(ISNUMBER(N27),IF(N27&lt;=Tests_Tolerance*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N27),IF(N27&lt;=FormulaTest_Tolerance*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P27" s="130" t="s">
@@ -7844,7 +7850,7 @@
         <v>0.0</v>
       </c>
       <c r="O28" s="127" t="str">
-        <f>IF(ISNUMBER(N28),IF(N28&lt;=Tests_Tolerance*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N28),IF(N28&lt;=FormulaTest_Tolerance*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P28" s="130" t="s">
@@ -7880,7 +7886,7 @@
         <v>0.0</v>
       </c>
       <c r="O29" s="127" t="str">
-        <f>IF(ISNUMBER(N29),IF(N29&lt;=Tests_Tolerance*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N29),IF(N29&lt;=FormulaTest_Tolerance*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P29" s="130" t="s">

</xml_diff>

<commit_message>
FormulaTest: data validation on every input cell
The 70 input cells of the formula tests had no validation, unlike the
input sheets. Each now has the input sheets' pattern: an input message
with the argument's meaning, range and rule, and a Stop alert. Ranges
are those the function accepts: dates and maturities in years, E after
S and after today, MPOR whole business days 1-250, option price and
strike above 0 after the lambda shift, expiry and volatility above 0,
attachment 0 to below 1 and detachment above it, correlations 0-1,
add-on, threshold and MTA 0 or more, TRUE/FALSE lists for the flags,
and any number where the rule allows a sign (V, C, NICA, bucket
notionals, entity add-ons, lambda P and K).

Validated: python tools/check.py, all gates pass; each input cell is
covered by exactly one rule (70 cells, 30 rules) and every shipped input
satisfies its rule; the workbook opens in LibreOffice and openpyxl reads
the 31 validations. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -7894,10 +7894,106 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="31">
     <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%." sqref="D5">
       <formula1>0.0000000000000001</formula1>
       <formula2>0.01</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E8:E10">
+      <formula1>-50</formula1>
+      <formula2>50</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid end date" error="Enter a number of years after the start date and after 0, at most 50." promptTitle="End date E (years)" prompt="Years from today to the end of the period referenced: after the start date and after today, at most 50 (CRE52.34)." sqref="F8:F10">
+      <formula1>AND(ISNUMBER(F8),F8&gt;MAX(E8,0),F8&lt;=50)</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid floor" error="Enter a number of years from 0 to 1." promptTitle="SD floor (years)" prompt="Floor on the supervisory duration, in years: 10 business days = 10/250 (CRE52.34)." sqref="G10">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid maturity" error="Enter a number of years from 0 to 50." promptTitle="Maturity M (years)" prompt="Remaining maturity in years. The unmargined factor floors it at 10 business days and caps it at 1 year (CRE52.48; CRR Art. 279c(1)(a))." sqref="E11:E13">
+      <formula1>0</formula1>
+      <formula2>50</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined factor 1.5 x sqrt(MPOR / 250) (CRE52.52; CRR Art. 279c(1)(b)). FALSE = unmargined factor from M." sqref="F13">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid MPOR" error="Enter a whole number of business days from 1 to 250." promptTitle="MPOR (business days)" prompt="Margin period of risk in business days, used when margined (CRE52.50-52; CRR Art. 285)." sqref="G13">
+      <formula1>1</formula1>
+      <formula2>250</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid price" error="Enter a number; P plus lambda (Input 7) must be above 0." promptTitle="Price P" prompt="Price of the underlying (forward rate for IR options). P plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="E14:E16">
+      <formula1>AND(ISNUMBER(E14),E14+$K14&gt;0)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid strike" error="Enter a number; K plus lambda (Input 7) must be above 0." promptTitle="Strike K" prompt="Strike of the option. K plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="F14:F16">
+      <formula1>AND(ISNUMBER(F14),F14+$K14&gt;0)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid expiry" error="Enter a number of years above 0, at most 100." promptTitle="Expiry T (years)" prompt="Latest contractual exercise date, in years from today, above 0 (CRE52.40; CRR Art. 279a(1)(a))." sqref="G14:G16">
+      <formula1>AND(ISNUMBER(G14),G14&gt;0,G14&lt;=100)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid volatility" error="Enter a decimal above 0, at most 5." promptTitle="Supervisory volatility" prompt="Supervisory option volatility as a decimal (0.5 = 50%), above 0 and at most 5 (CRE52.72; CRR Art. 279a)." sqref="H14:H16">
+      <formula1>AND(ISNUMBER(H14),H14&gt;0,H14&lt;=5)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Call" prompt="TRUE = call option; FALSE = put option (CRE52.40)." sqref="I14:I16">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Bought" prompt="TRUE = bought option (long); FALSE = sold option (short) (CRE52.40)." sqref="J14:J16">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Lambda shift" prompt="Shift added to P and K so that both are above 0 (CRE52.40 FAQ; CRR-RTS Art. 5). 0 or more." sqref="K16">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid attachment" error="Enter a decimal from 0 to below 1, e.g. 0.03 for 3%." promptTitle="Attachment A" prompt="Attachment point of the tranche, from 0 to below 1 (CRE52.41)." sqref="E17">
+      <formula1>0</formula1>
+      <formula2>0.9999</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid detachment" error="Enter a decimal above the attachment point and at most 1." promptTitle="Detachment D" prompt="Detachment point, above the attachment and at most 1 (CRE52.41)." sqref="F17">
+      <formula1>AND(ISNUMBER(F17),F17&gt;E17,F17&lt;=1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Long" prompt="TRUE = long in the tranche (positive delta); FALSE = short (CRE52.41)." sqref="G17">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Bucket effective notional" prompt="Signed effective notional D of maturity bucket 1, 2 or 3 (under 1 year, 1 to 5 years, over 5 years) (CRE52.57)." sqref="E18:G18">
+      <formula1>ISNUMBER(E18)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Entity add-on" prompt="Add-on of entity or commodity type k, signed by direction (CRE52.61; CRR Art. 280c)." sqref="E19:G19">
+      <formula1>ISNUMBER(E19)</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid correlation" error="Enter a decimal from 0 to 1." promptTitle="Correlation" prompt="Correlation of entity k, as a decimal from 0 to 1: credit 0.5 single name, 0.8 index (CRE52.61)." sqref="H19:J19">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V - C" prompt="Net market value of the netting set less collateral, signed (CRE52.23; CRR Art. 278(3))." sqref="E20:E21">
+      <formula1>ISNUMBER(E20)</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Aggregate add-on" prompt="Aggregate add-on of the netting set, 0 or more; 0 gives a multiplier of 1 (CRE52.23)." sqref="F20:F21">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V" prompt="Net market value of the trades in the netting set, signed (CRE52.10; CRR Art. 275)." sqref="E22">
+      <formula1>ISNUMBER(E22)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="C" prompt="Net collateral held after haircuts; negative if posted (CRE52.10; CRR Art. 275)." sqref="F22">
+      <formula1>ISNUMBER(F22)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined RC max(V - C, TH + MTA - NICA, 0) (CRE52.18); FALSE = max(V - C, 0) (CRE52.10)." sqref="G22">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Threshold TH" prompt="Threshold of the margin agreement, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="H22">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Minimum transfer amount" prompt="Minimum transfer amount MTA, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="I22">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="NICA" prompt="Net independent collateral amount, signed; negative if posted (CRE52.13; CRR Art. 275(2))." sqref="J22">
+      <formula1>ISNUMBER(J22)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="x" prompt="Point at which the standard normal distribution function is evaluated." sqref="E23:E24">
+      <formula1>ISNUMBER(E23)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Price or strike" prompt="Price P (Input 1) or strike K (Input 2) of the option; negative values allowed (CRR-RTS Art. 5(2))." sqref="E25:F29">
+      <formula1>ISNUMBER(E25)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Interest rate" prompt="TRUE = interest-rate option (threshold 0.10%); FALSE = commodity option (threshold 0.1) (CRR-RTS Art. 5(2))." sqref="G25:G29">
+      <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
FormulaTest: tolerance accepts any value above 0%
The tolerance validation was "decimal between 1E-16 and 1%", so a
smaller value such as 0.0000000000000000000001% was refused with a
message saying any percentage above 0% is accepted (found in Excel by
the owner). The rule is now D5 > 0 and D5 <= 1%, as the message says,
and the input message notes that below about 1e-16 (double precision)
only an exact match passes.

Validated: python tools/check.py, all gates pass. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -7895,9 +7895,8 @@
     </row>
   </sheetData>
   <dataValidations count="31">
-    <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%." sqref="D5">
-      <formula1>0.0000000000000001</formula1>
-      <formula2>0.01</formula2>
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%. Below about 0.00000000000001% (1e-16, double precision) only an exact match passes." sqref="D5">
+      <formula1>AND(ISNUMBER(D5),D5&gt;0,D5&lt;=0.01)</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E8:E10">
       <formula1>-50</formula1>

</xml_diff>

<commit_message>
FormulaTest: rename the Tests sheet and validate its inputs (#164)
The Tests sheet is FormulaTest (title "Formula tests"); the tolerance
name is FormulaTest_Tolerance; README and Basel_vs_CRR references
updated; code name shTests kept. The 70 input cells have data validation
in the input sheets' pattern, with the ranges the functions accept, and
the tolerance accepts any value above 0% and at most 1%.

Validated: python tools/check.py, all gates pass; owner verified in
Excel (sheet, validation, tolerance, 22 results); the tolerance rule
found there is fixed in the last commit.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -17,7 +17,7 @@
     <sheet name="TradeCalc" sheetId="8" r:id="rId8"/>
     <sheet name="Checks" sheetId="9" r:id="rId9"/>
     <sheet name="TestCatalogue" sheetId="10" r:id="rId10"/>
-    <sheet name="Tests" sheetId="11" r:id="rId11"/>
+    <sheet name="FormulaTest" sheetId="11" r:id="rId11"/>
     <sheet name="Basel_vs_CRR" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
@@ -28,6 +28,7 @@
     <definedName name="BasisFactor">Params!$E$17</definedName>
     <definedName name="BusinessDaysPerYear">Params!$E$11</definedName>
     <definedName name="DaysPerYear">Params!$E$10</definedName>
+    <definedName name="FormulaTest_Tolerance">FormulaTest!$D$5</definedName>
     <definedName name="FX_Table">Params!$C$57:$E$62</definedName>
     <definedName name="IRBucketOffset">Params!$E$22</definedName>
     <definedName name="IRCorrBucket12">Params!$E$19</definedName>
@@ -48,7 +49,6 @@
     <definedName name="SACCR_RunInputs" hidden="1">""</definedName>
     <definedName name="SDFloorBD">Params!$E$13</definedName>
     <definedName name="SF_Table">Params!$C$28:$K$54</definedName>
-    <definedName name="Tests_Tolerance">Tests!$D$5</definedName>
     <definedName name="Trades_Header">Trades!$C$4</definedName>
     <definedName name="VolatilityFactor">Params!$E$18</definedName>
   </definedNames>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="898">
   <si>
     <t>SA-CCR Calculator</t>
   </si>
@@ -136,7 +136,7 @@
     <t>6. Review</t>
   </si>
   <si>
-    <t>Checks lists every excluded trade and warning. TestCatalogue compares the engine with published / hand-calculated reference values per regime; Tests unit-tests the formula functions.</t>
+    <t>Checks lists every excluded trade and warning. TestCatalogue compares the engine with published / hand-calculated reference values per regime; FormulaTest unit-tests the formula functions.</t>
   </si>
   <si>
     <t>7. Regime</t>
@@ -2338,7 +2338,7 @@
     <t>Common table on Params.</t>
   </si>
   <si>
-    <t>Tests sheet</t>
+    <t>FormulaTest sheet</t>
   </si>
   <si>
     <t>Credit supervisory factors</t>
@@ -2792,6 +2792,12 @@
   </si>
   <si>
     <t>Tolerance: a test passes when |Function - Expected| &lt;= tolerance x max(1, |Expected|)</t>
+  </si>
+  <si>
+    <t>FormulaTest</t>
+  </si>
+  <si>
+    <t>Formula tests</t>
   </si>
 </sst>
 </file>
@@ -5000,7 +5006,7 @@
     </row>
     <row r="46" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C46" s="25" t="s">
-        <v>70</v>
+        <v>896</v>
       </c>
       <c r="D46" s="34" t="s">
         <v>71</v>
@@ -6987,7 +6993,7 @@
     </row>
     <row r="2" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="30" t="s">
-        <v>70</v>
+        <v>897</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="32"/>
@@ -7107,7 +7113,7 @@
         <v>0.0</v>
       </c>
       <c r="O8" s="127" t="str">
-        <f>IF(ISNUMBER(N8),IF(N8&lt;=Tests_Tolerance*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N8),IF(N8&lt;=FormulaTest_Tolerance*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P8" s="130" t="s">
@@ -7140,7 +7146,7 @@
         <v>0.0</v>
       </c>
       <c r="O9" s="127" t="str">
-        <f>IF(ISNUMBER(N9),IF(N9&lt;=Tests_Tolerance*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N9),IF(N9&lt;=FormulaTest_Tolerance*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P9" s="130" t="s">
@@ -7177,7 +7183,7 @@
         <v>0.0</v>
       </c>
       <c r="O10" s="127" t="str">
-        <f>IF(ISNUMBER(N10),IF(N10&lt;=Tests_Tolerance*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N10),IF(N10&lt;=FormulaTest_Tolerance*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P10" s="130" t="s">
@@ -7207,7 +7213,7 @@
         <v>0.0</v>
       </c>
       <c r="O11" s="127" t="str">
-        <f>IF(ISNUMBER(N11),IF(N11&lt;=Tests_Tolerance*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N11),IF(N11&lt;=FormulaTest_Tolerance*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P11" s="130" t="s">
@@ -7238,7 +7244,7 @@
         <v>0.0</v>
       </c>
       <c r="O12" s="127" t="str">
-        <f>IF(ISNUMBER(N12),IF(N12&lt;=Tests_Tolerance*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N12),IF(N12&lt;=FormulaTest_Tolerance*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P12" s="130" t="s">
@@ -7274,7 +7280,7 @@
         <v>0.0</v>
       </c>
       <c r="O13" s="127" t="str">
-        <f>IF(ISNUMBER(N13),IF(N13&lt;=Tests_Tolerance*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N13),IF(N13&lt;=FormulaTest_Tolerance*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P13" s="130" t="s">
@@ -7319,7 +7325,7 @@
         <v>0.0</v>
       </c>
       <c r="O14" s="127" t="str">
-        <f>IF(ISNUMBER(N14),IF(N14&lt;=Tests_Tolerance*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N14),IF(N14&lt;=FormulaTest_Tolerance*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P14" s="130" t="s">
@@ -7364,7 +7370,7 @@
         <v>0.0</v>
       </c>
       <c r="O15" s="127" t="str">
-        <f>IF(ISNUMBER(N15),IF(N15&lt;=Tests_Tolerance*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N15),IF(N15&lt;=FormulaTest_Tolerance*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P15" s="130" t="s">
@@ -7412,7 +7418,7 @@
         <v>0.0</v>
       </c>
       <c r="O16" s="127" t="str">
-        <f>IF(ISNUMBER(N16),IF(N16&lt;=Tests_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N16),IF(N16&lt;=FormulaTest_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P16" s="130" t="s">
@@ -7448,7 +7454,7 @@
         <v>8.881784197001252e-16</v>
       </c>
       <c r="O17" s="127" t="str">
-        <f>IF(ISNUMBER(N17),IF(N17&lt;=Tests_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N17),IF(N17&lt;=FormulaTest_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P17" s="130" t="s">
@@ -7484,7 +7490,7 @@
         <v>0.0</v>
       </c>
       <c r="O18" s="127" t="str">
-        <f>IF(ISNUMBER(N18),IF(N18&lt;=Tests_Tolerance*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N18),IF(N18&lt;=FormulaTest_Tolerance*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P18" s="130" t="s">
@@ -7529,7 +7535,7 @@
         <v>0.0</v>
       </c>
       <c r="O19" s="127" t="str">
-        <f>IF(ISNUMBER(N19),IF(N19&lt;=Tests_Tolerance*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N19),IF(N19&lt;=FormulaTest_Tolerance*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P19" s="130" t="s">
@@ -7562,7 +7568,7 @@
         <v>0.0</v>
       </c>
       <c r="O20" s="127" t="str">
-        <f>IF(ISNUMBER(N20),IF(N20&lt;=Tests_Tolerance*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N20),IF(N20&lt;=FormulaTest_Tolerance*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P20" s="130" t="s">
@@ -7595,7 +7601,7 @@
         <v>0.0</v>
       </c>
       <c r="O21" s="127" t="str">
-        <f>IF(ISNUMBER(N21),IF(N21&lt;=Tests_Tolerance*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N21),IF(N21&lt;=FormulaTest_Tolerance*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P21" s="130" t="s">
@@ -7640,7 +7646,7 @@
         <v>0.0</v>
       </c>
       <c r="O22" s="127" t="str">
-        <f>IF(ISNUMBER(N22),IF(N22&lt;=Tests_Tolerance*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N22),IF(N22&lt;=FormulaTest_Tolerance*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P22" s="130" t="s">
@@ -7670,7 +7676,7 @@
         <v>0.0</v>
       </c>
       <c r="O23" s="127" t="str">
-        <f>IF(ISNUMBER(N23),IF(N23&lt;=Tests_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N23),IF(N23&lt;=FormulaTest_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P23" s="130" t="s">
@@ -7700,7 +7706,7 @@
         <v>5.4129035033506995e-24</v>
       </c>
       <c r="O24" s="127" t="str">
-        <f>IF(ISNUMBER(N24),IF(N24&lt;=Tests_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N24),IF(N24&lt;=FormulaTest_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P24" s="130" t="s">
@@ -7736,7 +7742,7 @@
         <v>0.0</v>
       </c>
       <c r="O25" s="127" t="str">
-        <f>IF(ISNUMBER(N25),IF(N25&lt;=Tests_Tolerance*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N25),IF(N25&lt;=FormulaTest_Tolerance*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P25" s="130" t="s">
@@ -7772,7 +7778,7 @@
         <v>0.0</v>
       </c>
       <c r="O26" s="127" t="str">
-        <f>IF(ISNUMBER(N26),IF(N26&lt;=Tests_Tolerance*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N26),IF(N26&lt;=FormulaTest_Tolerance*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P26" s="130" t="s">
@@ -7808,7 +7814,7 @@
         <v>0.0</v>
       </c>
       <c r="O27" s="127" t="str">
-        <f>IF(ISNUMBER(N27),IF(N27&lt;=Tests_Tolerance*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N27),IF(N27&lt;=FormulaTest_Tolerance*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P27" s="130" t="s">
@@ -7844,7 +7850,7 @@
         <v>0.0</v>
       </c>
       <c r="O28" s="127" t="str">
-        <f>IF(ISNUMBER(N28),IF(N28&lt;=Tests_Tolerance*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N28),IF(N28&lt;=FormulaTest_Tolerance*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P28" s="130" t="s">
@@ -7880,7 +7886,7 @@
         <v>0.0</v>
       </c>
       <c r="O29" s="127" t="str">
-        <f>IF(ISNUMBER(N29),IF(N29&lt;=Tests_Tolerance*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N29),IF(N29&lt;=FormulaTest_Tolerance*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P29" s="130" t="s">
@@ -7888,10 +7894,105 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="decimal" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%." sqref="D5">
-      <formula1>0.0000000000000001</formula1>
-      <formula2>0.01</formula2>
+  <dataValidations count="31">
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%. Below about 0.00000000000001% (1e-16, double precision) only an exact match passes." sqref="D5">
+      <formula1>AND(ISNUMBER(D5),D5&gt;0,D5&lt;=0.01)</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E8:E10">
+      <formula1>-50</formula1>
+      <formula2>50</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid end date" error="Enter a number of years after the start date and after 0, at most 50." promptTitle="End date E (years)" prompt="Years from today to the end of the period referenced: after the start date and after today, at most 50 (CRE52.34)." sqref="F8:F10">
+      <formula1>AND(ISNUMBER(F8),F8&gt;MAX(E8,0),F8&lt;=50)</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid floor" error="Enter a number of years from 0 to 1." promptTitle="SD floor (years)" prompt="Floor on the supervisory duration, in years: 10 business days = 10/250 (CRE52.34)." sqref="G10">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid maturity" error="Enter a number of years from 0 to 50." promptTitle="Maturity M (years)" prompt="Remaining maturity in years. The unmargined factor floors it at 10 business days and caps it at 1 year (CRE52.48; CRR Art. 279c(1)(a))." sqref="E11:E13">
+      <formula1>0</formula1>
+      <formula2>50</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined factor 1.5 x sqrt(MPOR / 250) (CRE52.52; CRR Art. 279c(1)(b)). FALSE = unmargined factor from M." sqref="F13">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid MPOR" error="Enter a whole number of business days from 1 to 250." promptTitle="MPOR (business days)" prompt="Margin period of risk in business days, used when margined (CRE52.50-52; CRR Art. 285)." sqref="G13">
+      <formula1>1</formula1>
+      <formula2>250</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid price" error="Enter a number; P plus lambda (Input 7) must be above 0." promptTitle="Price P" prompt="Price of the underlying (forward rate for IR options). P plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="E14:E16">
+      <formula1>AND(ISNUMBER(E14),E14+$K14&gt;0)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid strike" error="Enter a number; K plus lambda (Input 7) must be above 0." promptTitle="Strike K" prompt="Strike of the option. K plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="F14:F16">
+      <formula1>AND(ISNUMBER(F14),F14+$K14&gt;0)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid expiry" error="Enter a number of years above 0, at most 100." promptTitle="Expiry T (years)" prompt="Latest contractual exercise date, in years from today, above 0 (CRE52.40; CRR Art. 279a(1)(a))." sqref="G14:G16">
+      <formula1>AND(ISNUMBER(G14),G14&gt;0,G14&lt;=100)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid volatility" error="Enter a decimal above 0, at most 5." promptTitle="Supervisory volatility" prompt="Supervisory option volatility as a decimal (0.5 = 50%), above 0 and at most 5 (CRE52.72; CRR Art. 279a)." sqref="H14:H16">
+      <formula1>AND(ISNUMBER(H14),H14&gt;0,H14&lt;=5)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Call" prompt="TRUE = call option; FALSE = put option (CRE52.40)." sqref="I14:I16">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Bought" prompt="TRUE = bought option (long); FALSE = sold option (short) (CRE52.40)." sqref="J14:J16">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Lambda shift" prompt="Shift added to P and K so that both are above 0 (CRE52.40 FAQ; CRR-RTS Art. 5). 0 or more." sqref="K16">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid attachment" error="Enter a decimal from 0 to below 1, e.g. 0.03 for 3%." promptTitle="Attachment A" prompt="Attachment point of the tranche, from 0 to below 1 (CRE52.41)." sqref="E17">
+      <formula1>0</formula1>
+      <formula2>0.9999</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid detachment" error="Enter a decimal above the attachment point and at most 1." promptTitle="Detachment D" prompt="Detachment point, above the attachment and at most 1 (CRE52.41)." sqref="F17">
+      <formula1>AND(ISNUMBER(F17),F17&gt;E17,F17&lt;=1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Long" prompt="TRUE = long in the tranche (positive delta); FALSE = short (CRE52.41)." sqref="G17">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Bucket effective notional" prompt="Signed effective notional D of maturity bucket 1, 2 or 3 (under 1 year, 1 to 5 years, over 5 years) (CRE52.57)." sqref="E18:G18">
+      <formula1>ISNUMBER(E18)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Entity add-on" prompt="Add-on of entity or commodity type k, signed by direction (CRE52.61; CRR Art. 280c)." sqref="E19:G19">
+      <formula1>ISNUMBER(E19)</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid correlation" error="Enter a decimal from 0 to 1." promptTitle="Correlation" prompt="Correlation of entity k, as a decimal from 0 to 1: credit 0.5 single name, 0.8 index (CRE52.61)." sqref="H19:J19">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V - C" prompt="Net market value of the netting set less collateral, signed (CRE52.23; CRR Art. 278(3))." sqref="E20:E21">
+      <formula1>ISNUMBER(E20)</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Aggregate add-on" prompt="Aggregate add-on of the netting set, 0 or more; 0 gives a multiplier of 1 (CRE52.23)." sqref="F20:F21">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V" prompt="Net market value of the trades in the netting set, signed (CRE52.10; CRR Art. 275)." sqref="E22">
+      <formula1>ISNUMBER(E22)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="C" prompt="Net collateral held after haircuts; negative if posted (CRE52.10; CRR Art. 275)." sqref="F22">
+      <formula1>ISNUMBER(F22)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined RC max(V - C, TH + MTA - NICA, 0) (CRE52.18); FALSE = max(V - C, 0) (CRE52.10)." sqref="G22">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Threshold TH" prompt="Threshold of the margin agreement, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="H22">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Minimum transfer amount" prompt="Minimum transfer amount MTA, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="I22">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="NICA" prompt="Net independent collateral amount, signed; negative if posted (CRE52.13; CRR Art. 275(2))." sqref="J22">
+      <formula1>ISNUMBER(J22)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="x" prompt="Point at which the standard normal distribution function is evaluated." sqref="E23:E24">
+      <formula1>ISNUMBER(E23)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Price or strike" prompt="Price P (Input 1) or strike K (Input 2) of the option; negative values allowed (CRR-RTS Art. 5(2))." sqref="E25:F29">
+      <formula1>ISNUMBER(E25)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Interest rate" prompt="TRUE = interest-rate option (threshold 0.10%); FALSE = commodity option (threshold 0.1) (CRR-RTS Art. 5(2))." sqref="G25:G29">
+      <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
FormulaTest: tolerance value on its label's row, column E
The tolerance value sat in D5 and cut its label in C5. It moves to E5,
so the label shows in full across C:D; the workbook name
FormulaTest_Tolerance and the validation move with it. Workbook guide
and CHANGELOG updated.

Validated: python tools/check.py, all gates pass; LibreOffice with the
cached values removed reads the tolerance through the name (a function
value 7.9e-6 relative off passes, 1.4e-5 fails). Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -28,7 +28,7 @@
     <definedName name="BasisFactor">Params!$E$17</definedName>
     <definedName name="BusinessDaysPerYear">Params!$E$11</definedName>
     <definedName name="DaysPerYear">Params!$E$10</definedName>
-    <definedName name="FormulaTest_Tolerance">FormulaTest!$D$5</definedName>
+    <definedName name="FormulaTest_Tolerance">FormulaTest!$E$5</definedName>
     <definedName name="FX_Table">Params!$C$57:$E$62</definedName>
     <definedName name="IRBucketOffset">Params!$E$22</definedName>
     <definedName name="IRCorrBucket12">Params!$E$19</definedName>
@@ -7034,7 +7034,7 @@
       <c r="C5" s="128" t="s">
         <v>895</v>
       </c>
-      <c r="D5" s="131">
+      <c r="E5" s="131">
         <v>1.0000000000000001E-5</v>
       </c>
     </row>
@@ -7895,8 +7895,8 @@
     </row>
   </sheetData>
   <dataValidations count="31">
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%. Below about 0.00000000000001% (1e-16, double precision) only an exact match passes." sqref="D5">
-      <formula1>AND(ISNUMBER(D5),D5&gt;0,D5&lt;=0.01)</formula1>
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%. Below about 0.00000000000001% (1e-16, double precision) only an exact match passes." sqref="E5">
+      <formula1>AND(ISNUMBER(E5),E5&gt;0,E5&lt;=0.01)</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E8:E10">
       <formula1>-50</formula1>

</xml_diff>

<commit_message>
FormulaTest: remove the empty row 3
Row 3 of the formula tests was empty. It is removed, so the description
is in C3, the tolerance in E4 (FormulaTest_Tolerance), the title in C5,
the column headers on row 6 and the tests on rows 7 to 28, as on the
output sheets. Every formula, array anchor, validation range and rule,
the selection and the workbook name move up one row with their cells.
Workbook guide and CHANGELOG name E4.

Validated: python tools/check.py, all gates pass; every cell is one row
higher with its references shifted (cell sets compared before and
after); LibreOffice with the cached values removed recalculates the 22
Expected values unchanged and reads the tolerance from E4 (7.9e-6
relative passes, 1.4e-5 fails); 31 validations kept. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -28,7 +28,7 @@
     <definedName name="BasisFactor">Params!$E$17</definedName>
     <definedName name="BusinessDaysPerYear">Params!$E$11</definedName>
     <definedName name="DaysPerYear">Params!$E$10</definedName>
-    <definedName name="FormulaTest_Tolerance">FormulaTest!$E$5</definedName>
+    <definedName name="FormulaTest_Tolerance">FormulaTest!$E$4</definedName>
     <definedName name="FX_Table">Params!$C$57:$E$62</definedName>
     <definedName name="IRBucketOffset">Params!$E$22</definedName>
     <definedName name="IRCorrBucket12">Params!$E$19</definedName>
@@ -6948,7 +6948,7 @@
     <tabColor rgb="FF548235"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AB29"/>
+  <dimension ref="B1:AB28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="4" customWidth="1"/>
@@ -7022,91 +7022,121 @@
       <c r="AA2" s="68"/>
       <c r="AB2" s="68"/>
     </row>
-    <row r="3" ht="21" x14ac:dyDescent="0.25">
-      <c r="C3" s="1"/>
-    </row>
-    <row r="4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="2" t="s">
+    <row r="3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="2" t="s">
         <v>508</v>
       </c>
     </row>
+    <row r="4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="128" t="s">
+        <v>895</v>
+      </c>
+      <c r="E4" s="131">
+        <v>1.0000000000000001E-5</v>
+      </c>
+    </row>
     <row r="5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="128" t="s">
-        <v>895</v>
-      </c>
-      <c r="E5" s="131">
-        <v>1.0000000000000001E-5</v>
-      </c>
-    </row>
-    <row r="6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="48" t="s">
+      <c r="C5" s="48" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="54" t="s">
+    <row r="6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="54" t="s">
         <v>510</v>
       </c>
-      <c r="D7" s="54" t="s">
+      <c r="D6" s="54" t="s">
         <v>884</v>
       </c>
-      <c r="E7" s="55" t="s">
+      <c r="E6" s="55" t="s">
         <v>885</v>
       </c>
-      <c r="F7" s="55" t="s">
+      <c r="F6" s="55" t="s">
         <v>886</v>
       </c>
-      <c r="G7" s="55" t="s">
+      <c r="G6" s="55" t="s">
         <v>887</v>
       </c>
-      <c r="H7" s="55" t="s">
+      <c r="H6" s="55" t="s">
         <v>888</v>
       </c>
-      <c r="I7" s="55" t="s">
+      <c r="I6" s="55" t="s">
         <v>889</v>
       </c>
-      <c r="J7" s="55" t="s">
+      <c r="J6" s="55" t="s">
         <v>890</v>
       </c>
-      <c r="K7" s="55" t="s">
+      <c r="K6" s="55" t="s">
         <v>891</v>
       </c>
-      <c r="L7" s="55" t="s">
+      <c r="L6" s="55" t="s">
         <v>892</v>
       </c>
-      <c r="M7" s="55" t="s">
+      <c r="M6" s="55" t="s">
         <v>893</v>
       </c>
-      <c r="N7" s="55" t="s">
+      <c r="N6" s="55" t="s">
         <v>514</v>
       </c>
-      <c r="O7" s="55" t="s">
+      <c r="O6" s="55" t="s">
         <v>515</v>
       </c>
-      <c r="P7" s="54" t="s">
+      <c r="P6" s="54" t="s">
         <v>894</v>
+      </c>
+    </row>
+    <row r="7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="128" t="s">
+        <v>516</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>859</v>
+      </c>
+      <c r="E7" s="129">
+        <v>0</v>
+      </c>
+      <c r="F7" s="129">
+        <v>10</v>
+      </c>
+      <c r="L7" s="125">
+        <f>(EXP(-0.05*MAX($E7,0))-EXP(-0.05*$F7))/0.05</f>
+        <v>7.8693868057473315</v>
+      </c>
+      <c r="M7" s="125" cm="1">
+        <f t="array" ref="M7">SACCR_SupervisoryDuration($E7,$F7)</f>
+        <v>7.8693868057473315</v>
+      </c>
+      <c r="N7" s="126">
+        <f>IFERROR(ABS(M7-L7),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O7" s="127" t="str">
+        <f>IF(ISNUMBER(N7),IF(N7&lt;=FormulaTest_Tolerance*MAX(1,ABS(L7)),"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P7" s="130" t="s">
+        <v>860</v>
       </c>
     </row>
     <row r="8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="128" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>859</v>
       </c>
       <c r="E8" s="129">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="129">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L8" s="125">
         <f>(EXP(-0.05*MAX($E8,0))-EXP(-0.05*$F8))/0.05</f>
-        <v>7.8693868057473315</v>
+        <v>7.485592282404547</v>
       </c>
       <c r="M8" s="125" cm="1">
         <f t="array" ref="M8">SACCR_SupervisoryDuration($E8,$F8)</f>
-        <v>7.8693868057473315</v>
+        <v>7.485592282404547</v>
       </c>
       <c r="N8" s="126">
         <f>IFERROR(ABS(M8-L8),"")</f>
@@ -7122,24 +7152,28 @@
     </row>
     <row r="9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="128" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>859</v>
+        <v>861</v>
       </c>
       <c r="E9" s="129">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="129">
-        <v>11</v>
+        <v>0.01</v>
+      </c>
+      <c r="G9" s="129">
+        <f>10/250</f>
+        <v>0.04</v>
       </c>
       <c r="L9" s="125">
-        <f>(EXP(-0.05*MAX($E9,0))-EXP(-0.05*$F9))/0.05</f>
-        <v>7.485592282404547</v>
+        <f>MAX((EXP(-0.05*MAX($E9,0))-EXP(-0.05*$F9))/0.05,$G9)</f>
+        <v>0.04</v>
       </c>
       <c r="M9" s="125" cm="1">
-        <f t="array" ref="M9">SACCR_SupervisoryDuration($E9,$F9)</f>
-        <v>7.485592282404547</v>
+        <f t="array" ref="M9">SACCR_SupervisoryDuration($E9,$F9,$G9)</f>
+        <v>0.04</v>
       </c>
       <c r="N9" s="126">
         <f>IFERROR(ABS(M9-L9),"")</f>
@@ -7155,28 +7189,21 @@
     </row>
     <row r="10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="128" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="E10" s="129">
-        <v>0</v>
-      </c>
-      <c r="F10" s="129">
-        <v>0.01</v>
-      </c>
-      <c r="G10" s="129">
-        <f>10/250</f>
-        <v>0.04</v>
+        <v>0.75</v>
       </c>
       <c r="L10" s="125">
-        <f>MAX((EXP(-0.05*MAX($E10,0))-EXP(-0.05*$F10))/0.05,$G10)</f>
-        <v>0.04</v>
+        <f>SQRT(MIN(MAX($E10,10/250),1))</f>
+        <v>0.8660254037844386</v>
       </c>
       <c r="M10" s="125" cm="1">
-        <f t="array" ref="M10">SACCR_SupervisoryDuration($E10,$F10,$G10)</f>
-        <v>0.04</v>
+        <f t="array" ref="M10">SACCR_MaturityFactor($E10)</f>
+        <v>0.8660254037844386</v>
       </c>
       <c r="N10" s="126">
         <f>IFERROR(ABS(M10-L10),"")</f>
@@ -7187,26 +7214,27 @@
         <v>PASS</v>
       </c>
       <c r="P10" s="130" t="s">
-        <v>860</v>
+        <v>863</v>
       </c>
     </row>
     <row r="11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="128" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D11" s="24" t="s">
         <v>862</v>
       </c>
       <c r="E11" s="129">
-        <v>0.75</v>
+        <f>3/365</f>
+        <v>0.00821917808219178</v>
       </c>
       <c r="L11" s="125">
         <f>SQRT(MIN(MAX($E11,10/250),1))</f>
-        <v>0.8660254037844386</v>
+        <v>0.2</v>
       </c>
       <c r="M11" s="125" cm="1">
         <f t="array" ref="M11">SACCR_MaturityFactor($E11)</f>
-        <v>0.8660254037844386</v>
+        <v>0.2</v>
       </c>
       <c r="N11" s="126">
         <f>IFERROR(ABS(M11-L11),"")</f>
@@ -7222,22 +7250,27 @@
     </row>
     <row r="12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="128" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="E12" s="129">
-        <f>3/365</f>
-        <v>0.00821917808219178</v>
+        <v>0</v>
+      </c>
+      <c r="F12" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="129">
+        <v>10</v>
       </c>
       <c r="L12" s="125">
-        <f>SQRT(MIN(MAX($E12,10/250),1))</f>
-        <v>0.2</v>
+        <f>IF($F12,1.5*SQRT($G12/250),SQRT(MIN(MAX($E12,10/250),1)))</f>
+        <v>0.30000000000000004</v>
       </c>
       <c r="M12" s="125" cm="1">
-        <f t="array" ref="M12">SACCR_MaturityFactor($E12)</f>
-        <v>0.2</v>
+        <f t="array" ref="M12">SACCR_MaturityFactor($E12,$F12,$G12)</f>
+        <v>0.30000000000000004</v>
       </c>
       <c r="N12" s="126">
         <f>IFERROR(ABS(M12-L12),"")</f>
@@ -7248,32 +7281,41 @@
         <v>PASS</v>
       </c>
       <c r="P12" s="130" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
     </row>
     <row r="13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="128" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>864</v>
+        <v>866</v>
       </c>
       <c r="E13" s="129">
+        <v>0.06</v>
+      </c>
+      <c r="F13" s="129">
+        <v>0.05</v>
+      </c>
+      <c r="G13" s="129">
+        <v>1</v>
+      </c>
+      <c r="H13" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="I13" s="129" t="b">
         <v>0</v>
       </c>
-      <c r="F13" s="129" t="b">
+      <c r="J13" s="129" t="b">
         <v>1</v>
       </c>
-      <c r="G13" s="129">
-        <v>10</v>
-      </c>
       <c r="L13" s="125">
-        <f>IF($F13,1.5*SQRT($G13/250),SQRT(MIN(MAX($E13,10/250),1)))</f>
-        <v>0.30000000000000004</v>
+        <f>IF($I13,_xlfn.NORM.S.DIST((LN(($E13+$K13)/($F13+$K13))+$H13^2*$G13/2)/($H13*SQRT($G13)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E13+$K13)/($F13+$K13))+$H13^2*$G13/2)/($H13*SQRT($G13)),TRUE))*IF($J13,1,-1)</f>
+        <v>-0.2693952177105327</v>
       </c>
       <c r="M13" s="125" cm="1">
-        <f t="array" ref="M13">SACCR_MaturityFactor($E13,$F13,$G13)</f>
-        <v>0.30000000000000004</v>
+        <f t="array" ref="M13">SACCR_OptionDelta($E13,$F13,$G13,$H13,$I13,$J13)</f>
+        <v>-0.2693952177105327</v>
       </c>
       <c r="N13" s="126">
         <f>IFERROR(ABS(M13-L13),"")</f>
@@ -7284,41 +7326,41 @@
         <v>PASS</v>
       </c>
       <c r="P13" s="130" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
     </row>
     <row r="14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="128" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D14" s="24" t="s">
         <v>866</v>
       </c>
       <c r="E14" s="129">
-        <v>0.06</v>
+        <v>100</v>
       </c>
       <c r="F14" s="129">
-        <v>0.05</v>
+        <v>110</v>
       </c>
       <c r="G14" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="H14" s="129">
+        <v>0.32</v>
+      </c>
+      <c r="I14" s="129" t="b">
         <v>1</v>
       </c>
-      <c r="H14" s="129">
-        <v>0.5</v>
-      </c>
-      <c r="I14" s="129" t="b">
+      <c r="J14" s="129" t="b">
         <v>0</v>
-      </c>
-      <c r="J14" s="129" t="b">
-        <v>1</v>
       </c>
       <c r="L14" s="125">
         <f>IF($I14,_xlfn.NORM.S.DIST((LN(($E14+$K14)/($F14+$K14))+$H14^2*$G14/2)/($H14*SQRT($G14)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E14+$K14)/($F14+$K14))+$H14^2*$G14/2)/($H14*SQRT($G14)),TRUE))*IF($J14,1,-1)</f>
-        <v>-0.2693952177105327</v>
+        <v>-0.37901134582780294</v>
       </c>
       <c r="M14" s="125" cm="1">
         <f t="array" ref="M14">SACCR_OptionDelta($E14,$F14,$G14,$H14,$I14,$J14)</f>
-        <v>-0.2693952177105327</v>
+        <v>-0.37901134582780294</v>
       </c>
       <c r="N14" s="126">
         <f>IFERROR(ABS(M14-L14),"")</f>
@@ -7334,36 +7376,39 @@
     </row>
     <row r="15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="128" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>866</v>
+        <v>868</v>
       </c>
       <c r="E15" s="129">
-        <v>100</v>
+        <v>-0.002</v>
       </c>
       <c r="F15" s="129">
-        <v>110</v>
+        <v>0.001</v>
       </c>
       <c r="G15" s="129">
+        <v>2</v>
+      </c>
+      <c r="H15" s="129">
         <v>0.5</v>
-      </c>
-      <c r="H15" s="129">
-        <v>0.32</v>
       </c>
       <c r="I15" s="129" t="b">
         <v>1</v>
       </c>
       <c r="J15" s="129" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K15" s="129">
+        <v>0.01</v>
       </c>
       <c r="L15" s="125">
         <f>IF($I15,_xlfn.NORM.S.DIST((LN(($E15+$K15)/($F15+$K15))+$H15^2*$G15/2)/($H15*SQRT($G15)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E15+$K15)/($F15+$K15))+$H15^2*$G15/2)/($H15*SQRT($G15)),TRUE))*IF($J15,1,-1)</f>
-        <v>-0.37901134582780294</v>
+        <v>0.46143935794124913</v>
       </c>
       <c r="M15" s="125" cm="1">
-        <f t="array" ref="M15">SACCR_OptionDelta($E15,$F15,$G15,$H15,$I15,$J15)</f>
-        <v>-0.37901134582780294</v>
+        <f t="array" ref="M15">SACCR_OptionDelta($E15,$F15,$G15,$H15,$I15,$J15,$K15)</f>
+        <v>0.46143935794124913</v>
       </c>
       <c r="N15" s="126">
         <f>IFERROR(ABS(M15-L15),"")</f>
@@ -7374,116 +7419,113 @@
         <v>PASS</v>
       </c>
       <c r="P15" s="130" t="s">
-        <v>867</v>
+        <v>869</v>
       </c>
     </row>
     <row r="16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="128" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>868</v>
+        <v>870</v>
       </c>
       <c r="E16" s="129">
-        <v>-0.002</v>
+        <v>0.03</v>
       </c>
       <c r="F16" s="129">
-        <v>0.001</v>
-      </c>
-      <c r="G16" s="129">
-        <v>2</v>
-      </c>
-      <c r="H16" s="129">
-        <v>0.5</v>
-      </c>
-      <c r="I16" s="129" t="b">
+        <v>0.06</v>
+      </c>
+      <c r="G16" s="129" t="b">
         <v>1</v>
       </c>
-      <c r="J16" s="129" t="b">
-        <v>1</v>
-      </c>
-      <c r="K16" s="129">
-        <v>0.01</v>
-      </c>
       <c r="L16" s="125">
-        <f>IF($I16,_xlfn.NORM.S.DIST((LN(($E16+$K16)/($F16+$K16))+$H16^2*$G16/2)/($H16*SQRT($G16)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E16+$K16)/($F16+$K16))+$H16^2*$G16/2)/($H16*SQRT($G16)),TRUE))*IF($J16,1,-1)</f>
-        <v>0.46143935794124913</v>
+        <f>15/((1+14*$E16)*(1+14*$F16))*IF($G16,1,-1)</f>
+        <v>5.740967544396817</v>
       </c>
       <c r="M16" s="125" cm="1">
-        <f t="array" ref="M16">SACCR_OptionDelta($E16,$F16,$G16,$H16,$I16,$J16,$K16)</f>
-        <v>0.46143935794124913</v>
+        <f t="array" ref="M16">SACCR_CDODelta($E16,$F16,$G16)</f>
+        <v>5.740967544396816</v>
       </c>
       <c r="N16" s="126">
         <f>IFERROR(ABS(M16-L16),"")</f>
-        <v>0.0</v>
+        <v>8.881784197001252e-16</v>
       </c>
       <c r="O16" s="127" t="str">
         <f>IF(ISNUMBER(N16),IF(N16&lt;=FormulaTest_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P16" s="130" t="s">
-        <v>869</v>
+        <v>871</v>
       </c>
     </row>
     <row r="17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="128" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="D17" s="24" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
       <c r="E17" s="129">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F17" s="129">
-        <v>0.06</v>
-      </c>
-      <c r="G17" s="129" t="b">
-        <v>1</v>
+        <v>-36253.8493844036</v>
+      </c>
+      <c r="G17" s="129">
+        <v>78693.8680574733</v>
       </c>
       <c r="L17" s="125">
-        <f>15/((1+14*$E17)*(1+14*$F17))*IF($G17,1,-1)</f>
-        <v>5.740967544396817</v>
+        <f>SQRT(MAX($E17^2+$F17^2+$G17^2+1.4*$E17*$F17+1.4*$F17*$G17+0.6*$E17*$G17,0))</f>
+        <v>59269.963463710395</v>
       </c>
       <c r="M17" s="125" cm="1">
-        <f t="array" ref="M17">SACCR_CDODelta($E17,$F17,$G17)</f>
-        <v>5.740967544396816</v>
+        <f t="array" ref="M17">SACCR_IREffectiveNotional($E17,$F17,$G17)</f>
+        <v>59269.963463710395</v>
       </c>
       <c r="N17" s="126">
         <f>IFERROR(ABS(M17-L17),"")</f>
-        <v>8.881784197001252e-16</v>
+        <v>0.0</v>
       </c>
       <c r="O17" s="127" t="str">
         <f>IF(ISNUMBER(N17),IF(N17&lt;=FormulaTest_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P17" s="130" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
     </row>
     <row r="18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="128" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="D18" s="24" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="E18" s="129">
-        <v>0</v>
+        <v>105.861937916956</v>
       </c>
       <c r="F18" s="129">
-        <v>-36253.8493844036</v>
+        <v>-279.916321663744</v>
       </c>
       <c r="G18" s="129">
-        <v>78693.8680574733</v>
+        <v>168.111404865732</v>
+      </c>
+      <c r="H18" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="I18" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="J18" s="129">
+        <v>0.8</v>
       </c>
       <c r="L18" s="125">
-        <f>SQRT(MAX($E18^2+$F18^2+$G18^2+1.4*$E18*$F18+1.4*$F18*$G18+0.6*$E18*$G18,0))</f>
-        <v>59269.963463710395</v>
+        <f>SQRT(SUMPRODUCT($E18:$G18,$H18:$J18)^2+SUMPRODUCT((1-$H18:$J18^2)*$E18:$G18^2))</f>
+        <v>282.12883185966604</v>
       </c>
       <c r="M18" s="125" cm="1">
-        <f t="array" ref="M18">SACCR_IREffectiveNotional($E18,$F18,$G18)</f>
-        <v>59269.963463710395</v>
+        <f t="array" ref="M18">SACCR_FactorAggregation($E18:$G18,$H18:$J18)</f>
+        <v>282.12883185966604</v>
       </c>
       <c r="N18" s="126">
         <f>IFERROR(ABS(M18-L18),"")</f>
@@ -7494,41 +7536,29 @@
         <v>PASS</v>
       </c>
       <c r="P18" s="130" t="s">
-        <v>873</v>
+        <v>875</v>
       </c>
     </row>
     <row r="19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="128" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="E19" s="129">
-        <v>105.861937916956</v>
+        <v>-20</v>
       </c>
       <c r="F19" s="129">
-        <v>-279.916321663744</v>
-      </c>
-      <c r="G19" s="129">
-        <v>168.111404865732</v>
-      </c>
-      <c r="H19" s="129">
-        <v>0.5</v>
-      </c>
-      <c r="I19" s="129">
-        <v>0.5</v>
-      </c>
-      <c r="J19" s="129">
-        <v>0.8</v>
+        <v>282</v>
       </c>
       <c r="L19" s="125">
-        <f>SQRT(SUMPRODUCT($E19:$G19,$H19:$J19)^2+SUMPRODUCT((1-$H19:$J19^2)*$E19:$G19^2))</f>
-        <v>282.12883185966604</v>
+        <f>IF($F19&lt;=0,1,MIN(1,0.05+0.95*EXP($E19/(2*0.95*$F19))))</f>
+        <v>0.9651926811871945</v>
       </c>
       <c r="M19" s="125" cm="1">
-        <f t="array" ref="M19">SACCR_FactorAggregation($E19:$G19,$H19:$J19)</f>
-        <v>282.12883185966604</v>
+        <f t="array" ref="M19">SACCR_Multiplier($E19,$F19)</f>
+        <v>0.9651926811871945</v>
       </c>
       <c r="N19" s="126">
         <f>IFERROR(ABS(M19-L19),"")</f>
@@ -7539,29 +7569,29 @@
         <v>PASS</v>
       </c>
       <c r="P19" s="130" t="s">
-        <v>875</v>
+        <v>877</v>
       </c>
     </row>
     <row r="20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="128" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D20" s="24" t="s">
         <v>876</v>
       </c>
       <c r="E20" s="129">
-        <v>-20</v>
+        <v>10</v>
       </c>
       <c r="F20" s="129">
         <v>282</v>
       </c>
       <c r="L20" s="125">
         <f>IF($F20&lt;=0,1,MIN(1,0.05+0.95*EXP($E20/(2*0.95*$F20))))</f>
-        <v>0.9651926811871945</v>
+        <v>1</v>
       </c>
       <c r="M20" s="125" cm="1">
         <f t="array" ref="M20">SACCR_Multiplier($E20,$F20)</f>
-        <v>0.9651926811871945</v>
+        <v>1.0</v>
       </c>
       <c r="N20" s="126">
         <f>IFERROR(ABS(M20-L20),"")</f>
@@ -7577,24 +7607,36 @@
     </row>
     <row r="21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="128" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D21" s="24" t="s">
-        <v>876</v>
+        <v>878</v>
       </c>
       <c r="E21" s="129">
+        <v>5</v>
+      </c>
+      <c r="F21" s="129">
         <v>10</v>
       </c>
-      <c r="F21" s="129">
-        <v>282</v>
+      <c r="G21" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="129">
+        <v>0</v>
+      </c>
+      <c r="I21" s="129">
+        <v>10</v>
+      </c>
+      <c r="J21" s="129">
+        <v>2</v>
       </c>
       <c r="L21" s="125">
-        <f>IF($F21&lt;=0,1,MIN(1,0.05+0.95*EXP($E21/(2*0.95*$F21))))</f>
-        <v>1</v>
+        <f>IF($G21,MAX($E21-$F21,$H21+$I21-$J21,0),MAX($E21-$F21,0))</f>
+        <v>8</v>
       </c>
       <c r="M21" s="125" cm="1">
-        <f t="array" ref="M21">SACCR_Multiplier($E21,$F21)</f>
-        <v>1.0</v>
+        <f t="array" ref="M21">SACCR_ReplacementCost($E21,$F21,$G21,$H21,$I21,$J21)</f>
+        <v>8.0</v>
       </c>
       <c r="N21" s="126">
         <f>IFERROR(ABS(M21-L21),"")</f>
@@ -7605,41 +7647,26 @@
         <v>PASS</v>
       </c>
       <c r="P21" s="130" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
     </row>
     <row r="22" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="128" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D22" s="24" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="E22" s="129">
-        <v>5</v>
-      </c>
-      <c r="F22" s="129">
-        <v>10</v>
-      </c>
-      <c r="G22" s="129" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="129">
-        <v>0</v>
-      </c>
-      <c r="I22" s="129">
-        <v>10</v>
-      </c>
-      <c r="J22" s="129">
-        <v>2</v>
+        <v>1.96</v>
       </c>
       <c r="L22" s="125">
-        <f>IF($G22,MAX($E22-$F22,$H22+$I22-$J22,0),MAX($E22-$F22,0))</f>
-        <v>8</v>
+        <f>_xlfn.NORM.S.DIST($E22,TRUE)</f>
+        <v>0.9750021048517795</v>
       </c>
       <c r="M22" s="125" cm="1">
-        <f t="array" ref="M22">SACCR_ReplacementCost($E22,$F22,$G22,$H22,$I22,$J22)</f>
-        <v>8.0</v>
+        <f t="array" ref="M22">SACCR_NormCDF($E22)</f>
+        <v>0.9750021048517795</v>
       </c>
       <c r="N22" s="126">
         <f>IFERROR(ABS(M22-L22),"")</f>
@@ -7650,30 +7677,30 @@
         <v>PASS</v>
       </c>
       <c r="P22" s="130" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
     </row>
     <row r="23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="128" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D23" s="24" t="s">
         <v>880</v>
       </c>
       <c r="E23" s="129">
-        <v>1.96</v>
+        <v>-8</v>
       </c>
       <c r="L23" s="125">
         <f>_xlfn.NORM.S.DIST($E23,TRUE)</f>
-        <v>0.9750021048517795</v>
+        <v>6.220960574271819e-16</v>
       </c>
       <c r="M23" s="125" cm="1">
         <f t="array" ref="M23">SACCR_NormCDF($E23)</f>
-        <v>0.9750021048517795</v>
+        <v>6.220960520142784e-16</v>
       </c>
       <c r="N23" s="126">
         <f>IFERROR(ABS(M23-L23),"")</f>
-        <v>0.0</v>
+        <v>5.4129035033506995e-24</v>
       </c>
       <c r="O23" s="127" t="str">
         <f>IF(ISNUMBER(N23),IF(N23&lt;=FormulaTest_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
@@ -7685,57 +7712,63 @@
     </row>
     <row r="24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="128" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D24" s="24" t="s">
-        <v>880</v>
+        <v>882</v>
       </c>
       <c r="E24" s="129">
-        <v>-8</v>
+        <v>-0.002</v>
+      </c>
+      <c r="F24" s="129">
+        <v>0.001</v>
+      </c>
+      <c r="G24" s="129" t="b">
+        <v>1</v>
       </c>
       <c r="L24" s="125">
-        <f>_xlfn.NORM.S.DIST($E24,TRUE)</f>
-        <v>6.220960574271819e-16</v>
+        <f>IF($G24,MAX(0.001-MIN($E24,$F24),0),MAX(-(1+0.1)*MIN($E24,$F24),0))</f>
+        <v>0.003</v>
       </c>
       <c r="M24" s="125" cm="1">
-        <f t="array" ref="M24">SACCR_NormCDF($E24)</f>
-        <v>6.220960520142784e-16</v>
+        <f t="array" ref="M24">SACCR_LambdaCRR($E24,$F24,$G24)</f>
+        <v>0.003</v>
       </c>
       <c r="N24" s="126">
         <f>IFERROR(ABS(M24-L24),"")</f>
-        <v>5.4129035033506995e-24</v>
+        <v>0.0</v>
       </c>
       <c r="O24" s="127" t="str">
         <f>IF(ISNUMBER(N24),IF(N24&lt;=FormulaTest_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P24" s="130" t="s">
-        <v>881</v>
+        <v>883</v>
       </c>
     </row>
     <row r="25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="128" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D25" s="24" t="s">
         <v>882</v>
       </c>
       <c r="E25" s="129">
-        <v>-0.002</v>
+        <v>0.02</v>
       </c>
       <c r="F25" s="129">
-        <v>0.001</v>
+        <v>0.03</v>
       </c>
       <c r="G25" s="129" t="b">
         <v>1</v>
       </c>
       <c r="L25" s="125">
         <f>IF($G25,MAX(0.001-MIN($E25,$F25),0),MAX(-(1+0.1)*MIN($E25,$F25),0))</f>
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="M25" s="125" cm="1">
         <f t="array" ref="M25">SACCR_LambdaCRR($E25,$F25,$G25)</f>
-        <v>0.003</v>
+        <v>0.0</v>
       </c>
       <c r="N25" s="126">
         <f>IFERROR(ABS(M25-L25),"")</f>
@@ -7751,27 +7784,27 @@
     </row>
     <row r="26" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="128" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="D26" s="24" t="s">
         <v>882</v>
       </c>
       <c r="E26" s="129">
-        <v>0.02</v>
+        <v>0.0005</v>
       </c>
       <c r="F26" s="129">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="G26" s="129" t="b">
         <v>1</v>
       </c>
       <c r="L26" s="125">
         <f>IF($G26,MAX(0.001-MIN($E26,$F26),0),MAX(-(1+0.1)*MIN($E26,$F26),0))</f>
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="M26" s="125" cm="1">
         <f t="array" ref="M26">SACCR_LambdaCRR($E26,$F26,$G26)</f>
-        <v>0.0</v>
+        <v>0.0005</v>
       </c>
       <c r="N26" s="126">
         <f>IFERROR(ABS(M26-L26),"")</f>
@@ -7787,27 +7820,27 @@
     </row>
     <row r="27" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="128" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D27" s="24" t="s">
         <v>882</v>
       </c>
       <c r="E27" s="129">
-        <v>0.0005</v>
+        <v>-5</v>
       </c>
       <c r="F27" s="129">
-        <v>0.01</v>
+        <v>-4</v>
       </c>
       <c r="G27" s="129" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L27" s="125">
         <f>IF($G27,MAX(0.001-MIN($E27,$F27),0),MAX(-(1+0.1)*MIN($E27,$F27),0))</f>
-        <v>0.0005</v>
+        <v>5.5</v>
       </c>
       <c r="M27" s="125" cm="1">
         <f t="array" ref="M27">SACCR_LambdaCRR($E27,$F27,$G27)</f>
-        <v>0.0005</v>
+        <v>5.5</v>
       </c>
       <c r="N27" s="126">
         <f>IFERROR(ABS(M27-L27),"")</f>
@@ -7823,27 +7856,27 @@
     </row>
     <row r="28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C28" s="128" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="D28" s="24" t="s">
         <v>882</v>
       </c>
       <c r="E28" s="129">
-        <v>-5</v>
+        <v>40</v>
       </c>
       <c r="F28" s="129">
-        <v>-4</v>
+        <v>35</v>
       </c>
       <c r="G28" s="129" t="b">
         <v>0</v>
       </c>
       <c r="L28" s="125">
         <f>IF($G28,MAX(0.001-MIN($E28,$F28),0),MAX(-(1+0.1)*MIN($E28,$F28),0))</f>
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="M28" s="125" cm="1">
         <f t="array" ref="M28">SACCR_LambdaCRR($E28,$F28,$G28)</f>
-        <v>5.5</v>
+        <v>0.0</v>
       </c>
       <c r="N28" s="126">
         <f>IFERROR(ABS(M28-L28),"")</f>
@@ -7857,141 +7890,105 @@
         <v>883</v>
       </c>
     </row>
-    <row r="29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C29" s="128" t="s">
-        <v>558</v>
-      </c>
-      <c r="D29" s="24" t="s">
-        <v>882</v>
-      </c>
-      <c r="E29" s="129">
-        <v>40</v>
-      </c>
-      <c r="F29" s="129">
-        <v>35</v>
-      </c>
-      <c r="G29" s="129" t="b">
-        <v>0</v>
-      </c>
-      <c r="L29" s="125">
-        <f>IF($G29,MAX(0.001-MIN($E29,$F29),0),MAX(-(1+0.1)*MIN($E29,$F29),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M29" s="125" cm="1">
-        <f t="array" ref="M29">SACCR_LambdaCRR($E29,$F29,$G29)</f>
-        <v>0.0</v>
-      </c>
-      <c r="N29" s="126">
-        <f>IFERROR(ABS(M29-L29),"")</f>
-        <v>0.0</v>
-      </c>
-      <c r="O29" s="127" t="str">
-        <f>IF(ISNUMBER(N29),IF(N29&lt;=FormulaTest_Tolerance*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P29" s="130" t="s">
-        <v>883</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="31">
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%. Below about 0.00000000000001% (1e-16, double precision) only an exact match passes." sqref="E5">
-      <formula1>AND(ISNUMBER(E5),E5&gt;0,E5&lt;=0.01)</formula1>
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%. Below about 0.00000000000001% (1e-16, double precision) only an exact match passes." sqref="E4">
+      <formula1>AND(ISNUMBER(E4),E4&gt;0,E4&lt;=0.01)</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E8:E10">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E7:E9">
       <formula1>-50</formula1>
       <formula2>50</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid end date" error="Enter a number of years after the start date and after 0, at most 50." promptTitle="End date E (years)" prompt="Years from today to the end of the period referenced: after the start date and after today, at most 50 (CRE52.34)." sqref="F8:F10">
-      <formula1>AND(ISNUMBER(F8),F8&gt;MAX(E8,0),F8&lt;=50)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid end date" error="Enter a number of years after the start date and after 0, at most 50." promptTitle="End date E (years)" prompt="Years from today to the end of the period referenced: after the start date and after today, at most 50 (CRE52.34)." sqref="F7:F9">
+      <formula1>AND(ISNUMBER(F7),F7&gt;MAX(E7,0),F7&lt;=50)</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid floor" error="Enter a number of years from 0 to 1." promptTitle="SD floor (years)" prompt="Floor on the supervisory duration, in years: 10 business days = 10/250 (CRE52.34)." sqref="G10">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid floor" error="Enter a number of years from 0 to 1." promptTitle="SD floor (years)" prompt="Floor on the supervisory duration, in years: 10 business days = 10/250 (CRE52.34)." sqref="G9">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid maturity" error="Enter a number of years from 0 to 50." promptTitle="Maturity M (years)" prompt="Remaining maturity in years. The unmargined factor floors it at 10 business days and caps it at 1 year (CRE52.48; CRR Art. 279c(1)(a))." sqref="E11:E13">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid maturity" error="Enter a number of years from 0 to 50." promptTitle="Maturity M (years)" prompt="Remaining maturity in years. The unmargined factor floors it at 10 business days and caps it at 1 year (CRE52.48; CRR Art. 279c(1)(a))." sqref="E10:E12">
       <formula1>0</formula1>
       <formula2>50</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined factor 1.5 x sqrt(MPOR / 250) (CRE52.52; CRR Art. 279c(1)(b)). FALSE = unmargined factor from M." sqref="F13">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined factor 1.5 x sqrt(MPOR / 250) (CRE52.52; CRR Art. 279c(1)(b)). FALSE = unmargined factor from M." sqref="F12">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid MPOR" error="Enter a whole number of business days from 1 to 250." promptTitle="MPOR (business days)" prompt="Margin period of risk in business days, used when margined (CRE52.50-52; CRR Art. 285)." sqref="G13">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid MPOR" error="Enter a whole number of business days from 1 to 250." promptTitle="MPOR (business days)" prompt="Margin period of risk in business days, used when margined (CRE52.50-52; CRR Art. 285)." sqref="G12">
       <formula1>1</formula1>
       <formula2>250</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid price" error="Enter a number; P plus lambda (Input 7) must be above 0." promptTitle="Price P" prompt="Price of the underlying (forward rate for IR options). P plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="E14:E16">
-      <formula1>AND(ISNUMBER(E14),E14+$K14&gt;0)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid price" error="Enter a number; P plus lambda (Input 7) must be above 0." promptTitle="Price P" prompt="Price of the underlying (forward rate for IR options). P plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="E13:E15">
+      <formula1>AND(ISNUMBER(E13),E13+$K13&gt;0)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid strike" error="Enter a number; K plus lambda (Input 7) must be above 0." promptTitle="Strike K" prompt="Strike of the option. K plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="F14:F16">
-      <formula1>AND(ISNUMBER(F14),F14+$K14&gt;0)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid strike" error="Enter a number; K plus lambda (Input 7) must be above 0." promptTitle="Strike K" prompt="Strike of the option. K plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="F13:F15">
+      <formula1>AND(ISNUMBER(F13),F13+$K13&gt;0)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid expiry" error="Enter a number of years above 0, at most 100." promptTitle="Expiry T (years)" prompt="Latest contractual exercise date, in years from today, above 0 (CRE52.40; CRR Art. 279a(1)(a))." sqref="G14:G16">
-      <formula1>AND(ISNUMBER(G14),G14&gt;0,G14&lt;=100)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid expiry" error="Enter a number of years above 0, at most 100." promptTitle="Expiry T (years)" prompt="Latest contractual exercise date, in years from today, above 0 (CRE52.40; CRR Art. 279a(1)(a))." sqref="G13:G15">
+      <formula1>AND(ISNUMBER(G13),G13&gt;0,G13&lt;=100)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid volatility" error="Enter a decimal above 0, at most 5." promptTitle="Supervisory volatility" prompt="Supervisory option volatility as a decimal (0.5 = 50%), above 0 and at most 5 (CRE52.72; CRR Art. 279a)." sqref="H14:H16">
-      <formula1>AND(ISNUMBER(H14),H14&gt;0,H14&lt;=5)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid volatility" error="Enter a decimal above 0, at most 5." promptTitle="Supervisory volatility" prompt="Supervisory option volatility as a decimal (0.5 = 50%), above 0 and at most 5 (CRE52.72; CRR Art. 279a)." sqref="H13:H15">
+      <formula1>AND(ISNUMBER(H13),H13&gt;0,H13&lt;=5)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Call" prompt="TRUE = call option; FALSE = put option (CRE52.40)." sqref="I14:I16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Call" prompt="TRUE = call option; FALSE = put option (CRE52.40)." sqref="I13:I15">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Bought" prompt="TRUE = bought option (long); FALSE = sold option (short) (CRE52.40)." sqref="J14:J16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Bought" prompt="TRUE = bought option (long); FALSE = sold option (short) (CRE52.40)." sqref="J13:J15">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Lambda shift" prompt="Shift added to P and K so that both are above 0 (CRE52.40 FAQ; CRR-RTS Art. 5). 0 or more." sqref="K16">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Lambda shift" prompt="Shift added to P and K so that both are above 0 (CRE52.40 FAQ; CRR-RTS Art. 5). 0 or more." sqref="K15">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid attachment" error="Enter a decimal from 0 to below 1, e.g. 0.03 for 3%." promptTitle="Attachment A" prompt="Attachment point of the tranche, from 0 to below 1 (CRE52.41)." sqref="E17">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid attachment" error="Enter a decimal from 0 to below 1, e.g. 0.03 for 3%." promptTitle="Attachment A" prompt="Attachment point of the tranche, from 0 to below 1 (CRE52.41)." sqref="E16">
       <formula1>0</formula1>
       <formula2>0.9999</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid detachment" error="Enter a decimal above the attachment point and at most 1." promptTitle="Detachment D" prompt="Detachment point, above the attachment and at most 1 (CRE52.41)." sqref="F17">
-      <formula1>AND(ISNUMBER(F17),F17&gt;E17,F17&lt;=1)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid detachment" error="Enter a decimal above the attachment point and at most 1." promptTitle="Detachment D" prompt="Detachment point, above the attachment and at most 1 (CRE52.41)." sqref="F16">
+      <formula1>AND(ISNUMBER(F16),F16&gt;E16,F16&lt;=1)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Long" prompt="TRUE = long in the tranche (positive delta); FALSE = short (CRE52.41)." sqref="G17">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Long" prompt="TRUE = long in the tranche (positive delta); FALSE = short (CRE52.41)." sqref="G16">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Bucket effective notional" prompt="Signed effective notional D of maturity bucket 1, 2 or 3 (under 1 year, 1 to 5 years, over 5 years) (CRE52.57)." sqref="E18:G18">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Bucket effective notional" prompt="Signed effective notional D of maturity bucket 1, 2 or 3 (under 1 year, 1 to 5 years, over 5 years) (CRE52.57)." sqref="E17:G17">
+      <formula1>ISNUMBER(E17)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Entity add-on" prompt="Add-on of entity or commodity type k, signed by direction (CRE52.61; CRR Art. 280c)." sqref="E18:G18">
       <formula1>ISNUMBER(E18)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Entity add-on" prompt="Add-on of entity or commodity type k, signed by direction (CRE52.61; CRR Art. 280c)." sqref="E19:G19">
-      <formula1>ISNUMBER(E19)</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid correlation" error="Enter a decimal from 0 to 1." promptTitle="Correlation" prompt="Correlation of entity k, as a decimal from 0 to 1: credit 0.5 single name, 0.8 index (CRE52.61)." sqref="H19:J19">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid correlation" error="Enter a decimal from 0 to 1." promptTitle="Correlation" prompt="Correlation of entity k, as a decimal from 0 to 1: credit 0.5 single name, 0.8 index (CRE52.61)." sqref="H18:J18">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V - C" prompt="Net market value of the netting set less collateral, signed (CRE52.23; CRR Art. 278(3))." sqref="E20:E21">
-      <formula1>ISNUMBER(E20)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V - C" prompt="Net market value of the netting set less collateral, signed (CRE52.23; CRR Art. 278(3))." sqref="E19:E20">
+      <formula1>ISNUMBER(E19)</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Aggregate add-on" prompt="Aggregate add-on of the netting set, 0 or more; 0 gives a multiplier of 1 (CRE52.23)." sqref="F20:F21">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Aggregate add-on" prompt="Aggregate add-on of the netting set, 0 or more; 0 gives a multiplier of 1 (CRE52.23)." sqref="F19:F20">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V" prompt="Net market value of the trades in the netting set, signed (CRE52.10; CRR Art. 275)." sqref="E22">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V" prompt="Net market value of the trades in the netting set, signed (CRE52.10; CRR Art. 275)." sqref="E21">
+      <formula1>ISNUMBER(E21)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="C" prompt="Net collateral held after haircuts; negative if posted (CRE52.10; CRR Art. 275)." sqref="F21">
+      <formula1>ISNUMBER(F21)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined RC max(V - C, TH + MTA - NICA, 0) (CRE52.18); FALSE = max(V - C, 0) (CRE52.10)." sqref="G21">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Threshold TH" prompt="Threshold of the margin agreement, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="H21">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Minimum transfer amount" prompt="Minimum transfer amount MTA, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="I21">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="NICA" prompt="Net independent collateral amount, signed; negative if posted (CRE52.13; CRR Art. 275(2))." sqref="J21">
+      <formula1>ISNUMBER(J21)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="x" prompt="Point at which the standard normal distribution function is evaluated." sqref="E22:E23">
       <formula1>ISNUMBER(E22)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="C" prompt="Net collateral held after haircuts; negative if posted (CRE52.10; CRR Art. 275)." sqref="F22">
-      <formula1>ISNUMBER(F22)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Price or strike" prompt="Price P (Input 1) or strike K (Input 2) of the option; negative values allowed (CRR-RTS Art. 5(2))." sqref="E24:F28">
+      <formula1>ISNUMBER(E24)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined RC max(V - C, TH + MTA - NICA, 0) (CRE52.18); FALSE = max(V - C, 0) (CRE52.10)." sqref="G22">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Threshold TH" prompt="Threshold of the margin agreement, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="H22">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Minimum transfer amount" prompt="Minimum transfer amount MTA, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="I22">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="NICA" prompt="Net independent collateral amount, signed; negative if posted (CRE52.13; CRR Art. 275(2))." sqref="J22">
-      <formula1>ISNUMBER(J22)</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="x" prompt="Point at which the standard normal distribution function is evaluated." sqref="E23:E24">
-      <formula1>ISNUMBER(E23)</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Price or strike" prompt="Price P (Input 1) or strike K (Input 2) of the option; negative values allowed (CRR-RTS Art. 5(2))." sqref="E25:F29">
-      <formula1>ISNUMBER(E25)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Interest rate" prompt="TRUE = interest-rate option (threshold 0.10%); FALSE = commodity option (threshold 0.1) (CRR-RTS Art. 5(2))." sqref="G25:G29">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Interest rate" prompt="TRUE = interest-rate option (threshold 0.10%); FALSE = commodity option (threshold 0.1) (CRR-RTS Art. 5(2))." sqref="G24:G28">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
FormulaTest: multiplier Expected returns 1 for positive V - C
For a positive V - C large against the add-on (20 and 0.01, both valid
inputs), the Expected formula of rows 19-20 evaluated EXP of about 1052
and returned #NUM!, so the row showed FAIL; SACCR_Multiplier returns 1
for any positive exponent without evaluating Exp (CRE52.23: the
multiplier is capped at 1). The formula now returns 1 when V - C > 0 or
the add-on is not positive, before the exponential. Found by review on
#166.

Validated: python tools/check.py, all gates pass; LibreOffice with the
cached values removed: shipped inputs unchanged (22 of 22), V - C = 20
with add-on 0.01 gives 1, V - C = -700 gives the 0.05 floor. Excel not
run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -7553,7 +7553,7 @@
         <v>282</v>
       </c>
       <c r="L19" s="125">
-        <f>IF($F19&lt;=0,1,MIN(1,0.05+0.95*EXP($E19/(2*0.95*$F19))))</f>
+        <f>IF(OR($F19&lt;=0,$E19&gt;0),1,MIN(1,0.05+0.95*EXP($E19/(2*0.95*$F19))))</f>
         <v>0.9651926811871945</v>
       </c>
       <c r="M19" s="125" cm="1">
@@ -7586,7 +7586,7 @@
         <v>282</v>
       </c>
       <c r="L20" s="125">
-        <f>IF($F20&lt;=0,1,MIN(1,0.05+0.95*EXP($E20/(2*0.95*$F20))))</f>
+        <f>IF(OR($F20&lt;=0,$E20&gt;0),1,MIN(1,0.05+0.95*EXP($E20/(2*0.95*$F20))))</f>
         <v>1</v>
       </c>
       <c r="M20" s="125" cm="1">

</xml_diff>

<commit_message>
FormulaTest: relative difference in the tolerance's format
The difference column showed |Function - Expected| in scientific
notation while the tolerance is a percentage applied to
max(1, |Expected|), so the two could not be compared by eye. The column
is now Rel. diff = |Function - Expected| / max(1, |Expected|), in the
tolerance's format (0.0000%), and Result compares it with the tolerance
directly: the pass criterion is unchanged. The tolerance label and input
message say so; workbook guide and CHANGELOG updated.

Validated: python tools/check.py, all gates pass; LibreOffice with the
cached values removed: 8.0e-6 relative passes and 1.44e-5 fails at
0.001%, and a difference of 0.54 on 59,270 gives 0.0009% and passes,
as before. Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="898">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="899">
   <si>
     <t>SA-CCR Calculator</t>
   </si>
@@ -2791,13 +2791,16 @@
     <t>Rule</t>
   </si>
   <si>
-    <t>Tolerance: a test passes when |Function - Expected| &lt;= tolerance x max(1, |Expected|)</t>
+    <t>Tolerance: a test passes when its Rel. diff is at most this value</t>
   </si>
   <si>
     <t>FormulaTest</t>
   </si>
   <si>
     <t>Formula tests</t>
+  </si>
+  <si>
+    <t>Rel. diff</t>
   </si>
 </sst>
 </file>
@@ -3224,7 +3227,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3620,6 +3623,9 @@
     </xf>
     <xf numFmtId="169" fontId="8" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7075,7 +7081,7 @@
         <v>893</v>
       </c>
       <c r="N6" s="55" t="s">
-        <v>514</v>
+        <v>898</v>
       </c>
       <c r="O6" s="55" t="s">
         <v>515</v>
@@ -7105,12 +7111,12 @@
         <f t="array" ref="M7">SACCR_SupervisoryDuration($E7,$F7)</f>
         <v>7.8693868057473315</v>
       </c>
-      <c r="N7" s="126">
-        <f>IFERROR(ABS(M7-L7),"")</f>
+      <c r="N7" s="132">
+        <f>IFERROR(ABS(M7-L7)/MAX(1,ABS(L7)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O7" s="127" t="str">
-        <f>IF(ISNUMBER(N7),IF(N7&lt;=FormulaTest_Tolerance*MAX(1,ABS(L7)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N7),IF(N7&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P7" s="130" t="s">
@@ -7138,12 +7144,12 @@
         <f t="array" ref="M8">SACCR_SupervisoryDuration($E8,$F8)</f>
         <v>7.485592282404547</v>
       </c>
-      <c r="N8" s="126">
-        <f>IFERROR(ABS(M8-L8),"")</f>
+      <c r="N8" s="132">
+        <f>IFERROR(ABS(M8-L8)/MAX(1,ABS(L8)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O8" s="127" t="str">
-        <f>IF(ISNUMBER(N8),IF(N8&lt;=FormulaTest_Tolerance*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N8),IF(N8&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P8" s="130" t="s">
@@ -7175,12 +7181,12 @@
         <f t="array" ref="M9">SACCR_SupervisoryDuration($E9,$F9,$G9)</f>
         <v>0.04</v>
       </c>
-      <c r="N9" s="126">
-        <f>IFERROR(ABS(M9-L9),"")</f>
+      <c r="N9" s="132">
+        <f>IFERROR(ABS(M9-L9)/MAX(1,ABS(L9)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O9" s="127" t="str">
-        <f>IF(ISNUMBER(N9),IF(N9&lt;=FormulaTest_Tolerance*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N9),IF(N9&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P9" s="130" t="s">
@@ -7205,12 +7211,12 @@
         <f t="array" ref="M10">SACCR_MaturityFactor($E10)</f>
         <v>0.8660254037844386</v>
       </c>
-      <c r="N10" s="126">
-        <f>IFERROR(ABS(M10-L10),"")</f>
+      <c r="N10" s="132">
+        <f>IFERROR(ABS(M10-L10)/MAX(1,ABS(L10)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O10" s="127" t="str">
-        <f>IF(ISNUMBER(N10),IF(N10&lt;=FormulaTest_Tolerance*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N10),IF(N10&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P10" s="130" t="s">
@@ -7236,12 +7242,12 @@
         <f t="array" ref="M11">SACCR_MaturityFactor($E11)</f>
         <v>0.2</v>
       </c>
-      <c r="N11" s="126">
-        <f>IFERROR(ABS(M11-L11),"")</f>
+      <c r="N11" s="132">
+        <f>IFERROR(ABS(M11-L11)/MAX(1,ABS(L11)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O11" s="127" t="str">
-        <f>IF(ISNUMBER(N11),IF(N11&lt;=FormulaTest_Tolerance*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N11),IF(N11&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P11" s="130" t="s">
@@ -7272,12 +7278,12 @@
         <f t="array" ref="M12">SACCR_MaturityFactor($E12,$F12,$G12)</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="N12" s="126">
-        <f>IFERROR(ABS(M12-L12),"")</f>
+      <c r="N12" s="132">
+        <f>IFERROR(ABS(M12-L12)/MAX(1,ABS(L12)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O12" s="127" t="str">
-        <f>IF(ISNUMBER(N12),IF(N12&lt;=FormulaTest_Tolerance*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N12),IF(N12&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P12" s="130" t="s">
@@ -7317,12 +7323,12 @@
         <f t="array" ref="M13">SACCR_OptionDelta($E13,$F13,$G13,$H13,$I13,$J13)</f>
         <v>-0.2693952177105327</v>
       </c>
-      <c r="N13" s="126">
-        <f>IFERROR(ABS(M13-L13),"")</f>
+      <c r="N13" s="132">
+        <f>IFERROR(ABS(M13-L13)/MAX(1,ABS(L13)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O13" s="127" t="str">
-        <f>IF(ISNUMBER(N13),IF(N13&lt;=FormulaTest_Tolerance*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N13),IF(N13&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P13" s="130" t="s">
@@ -7362,12 +7368,12 @@
         <f t="array" ref="M14">SACCR_OptionDelta($E14,$F14,$G14,$H14,$I14,$J14)</f>
         <v>-0.37901134582780294</v>
       </c>
-      <c r="N14" s="126">
-        <f>IFERROR(ABS(M14-L14),"")</f>
+      <c r="N14" s="132">
+        <f>IFERROR(ABS(M14-L14)/MAX(1,ABS(L14)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O14" s="127" t="str">
-        <f>IF(ISNUMBER(N14),IF(N14&lt;=FormulaTest_Tolerance*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N14),IF(N14&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P14" s="130" t="s">
@@ -7410,12 +7416,12 @@
         <f t="array" ref="M15">SACCR_OptionDelta($E15,$F15,$G15,$H15,$I15,$J15,$K15)</f>
         <v>0.46143935794124913</v>
       </c>
-      <c r="N15" s="126">
-        <f>IFERROR(ABS(M15-L15),"")</f>
+      <c r="N15" s="132">
+        <f>IFERROR(ABS(M15-L15)/MAX(1,ABS(L15)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O15" s="127" t="str">
-        <f>IF(ISNUMBER(N15),IF(N15&lt;=FormulaTest_Tolerance*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N15),IF(N15&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P15" s="130" t="s">
@@ -7446,12 +7452,12 @@
         <f t="array" ref="M16">SACCR_CDODelta($E16,$F16,$G16)</f>
         <v>5.740967544396816</v>
       </c>
-      <c r="N16" s="126">
-        <f>IFERROR(ABS(M16-L16),"")</f>
-        <v>8.881784197001252e-16</v>
+      <c r="N16" s="132">
+        <f>IFERROR(ABS(M16-L16)/MAX(1,ABS(L16)),"")</f>
+        <v>1.5470883833283245e-16</v>
       </c>
       <c r="O16" s="127" t="str">
-        <f>IF(ISNUMBER(N16),IF(N16&lt;=FormulaTest_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N16),IF(N16&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P16" s="130" t="s">
@@ -7482,12 +7488,12 @@
         <f t="array" ref="M17">SACCR_IREffectiveNotional($E17,$F17,$G17)</f>
         <v>59269.963463710395</v>
       </c>
-      <c r="N17" s="126">
-        <f>IFERROR(ABS(M17-L17),"")</f>
+      <c r="N17" s="132">
+        <f>IFERROR(ABS(M17-L17)/MAX(1,ABS(L17)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O17" s="127" t="str">
-        <f>IF(ISNUMBER(N17),IF(N17&lt;=FormulaTest_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N17),IF(N17&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P17" s="130" t="s">
@@ -7527,12 +7533,12 @@
         <f t="array" ref="M18">SACCR_FactorAggregation($E18:$G18,$H18:$J18)</f>
         <v>282.12883185966604</v>
       </c>
-      <c r="N18" s="126">
-        <f>IFERROR(ABS(M18-L18),"")</f>
+      <c r="N18" s="132">
+        <f>IFERROR(ABS(M18-L18)/MAX(1,ABS(L18)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O18" s="127" t="str">
-        <f>IF(ISNUMBER(N18),IF(N18&lt;=FormulaTest_Tolerance*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N18),IF(N18&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P18" s="130" t="s">
@@ -7560,12 +7566,12 @@
         <f t="array" ref="M19">SACCR_Multiplier($E19,$F19)</f>
         <v>0.9651926811871945</v>
       </c>
-      <c r="N19" s="126">
-        <f>IFERROR(ABS(M19-L19),"")</f>
+      <c r="N19" s="132">
+        <f>IFERROR(ABS(M19-L19)/MAX(1,ABS(L19)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O19" s="127" t="str">
-        <f>IF(ISNUMBER(N19),IF(N19&lt;=FormulaTest_Tolerance*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N19),IF(N19&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P19" s="130" t="s">
@@ -7593,12 +7599,12 @@
         <f t="array" ref="M20">SACCR_Multiplier($E20,$F20)</f>
         <v>1.0</v>
       </c>
-      <c r="N20" s="126">
-        <f>IFERROR(ABS(M20-L20),"")</f>
+      <c r="N20" s="132">
+        <f>IFERROR(ABS(M20-L20)/MAX(1,ABS(L20)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O20" s="127" t="str">
-        <f>IF(ISNUMBER(N20),IF(N20&lt;=FormulaTest_Tolerance*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N20),IF(N20&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P20" s="130" t="s">
@@ -7638,12 +7644,12 @@
         <f t="array" ref="M21">SACCR_ReplacementCost($E21,$F21,$G21,$H21,$I21,$J21)</f>
         <v>8.0</v>
       </c>
-      <c r="N21" s="126">
-        <f>IFERROR(ABS(M21-L21),"")</f>
+      <c r="N21" s="132">
+        <f>IFERROR(ABS(M21-L21)/MAX(1,ABS(L21)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O21" s="127" t="str">
-        <f>IF(ISNUMBER(N21),IF(N21&lt;=FormulaTest_Tolerance*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N21),IF(N21&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P21" s="130" t="s">
@@ -7668,12 +7674,12 @@
         <f t="array" ref="M22">SACCR_NormCDF($E22)</f>
         <v>0.9750021048517795</v>
       </c>
-      <c r="N22" s="126">
-        <f>IFERROR(ABS(M22-L22),"")</f>
+      <c r="N22" s="132">
+        <f>IFERROR(ABS(M22-L22)/MAX(1,ABS(L22)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O22" s="127" t="str">
-        <f>IF(ISNUMBER(N22),IF(N22&lt;=FormulaTest_Tolerance*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N22),IF(N22&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P22" s="130" t="s">
@@ -7698,12 +7704,12 @@
         <f t="array" ref="M23">SACCR_NormCDF($E23)</f>
         <v>6.220960520142784e-16</v>
       </c>
-      <c r="N23" s="126">
-        <f>IFERROR(ABS(M23-L23),"")</f>
+      <c r="N23" s="132">
+        <f>IFERROR(ABS(M23-L23)/MAX(1,ABS(L23)),"")</f>
         <v>5.4129035033506995e-24</v>
       </c>
       <c r="O23" s="127" t="str">
-        <f>IF(ISNUMBER(N23),IF(N23&lt;=FormulaTest_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N23),IF(N23&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P23" s="130" t="s">
@@ -7734,12 +7740,12 @@
         <f t="array" ref="M24">SACCR_LambdaCRR($E24,$F24,$G24)</f>
         <v>0.003</v>
       </c>
-      <c r="N24" s="126">
-        <f>IFERROR(ABS(M24-L24),"")</f>
+      <c r="N24" s="132">
+        <f>IFERROR(ABS(M24-L24)/MAX(1,ABS(L24)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O24" s="127" t="str">
-        <f>IF(ISNUMBER(N24),IF(N24&lt;=FormulaTest_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N24),IF(N24&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P24" s="130" t="s">
@@ -7770,12 +7776,12 @@
         <f t="array" ref="M25">SACCR_LambdaCRR($E25,$F25,$G25)</f>
         <v>0.0</v>
       </c>
-      <c r="N25" s="126">
-        <f>IFERROR(ABS(M25-L25),"")</f>
+      <c r="N25" s="132">
+        <f>IFERROR(ABS(M25-L25)/MAX(1,ABS(L25)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O25" s="127" t="str">
-        <f>IF(ISNUMBER(N25),IF(N25&lt;=FormulaTest_Tolerance*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N25),IF(N25&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P25" s="130" t="s">
@@ -7806,12 +7812,12 @@
         <f t="array" ref="M26">SACCR_LambdaCRR($E26,$F26,$G26)</f>
         <v>0.0005</v>
       </c>
-      <c r="N26" s="126">
-        <f>IFERROR(ABS(M26-L26),"")</f>
+      <c r="N26" s="132">
+        <f>IFERROR(ABS(M26-L26)/MAX(1,ABS(L26)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O26" s="127" t="str">
-        <f>IF(ISNUMBER(N26),IF(N26&lt;=FormulaTest_Tolerance*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N26),IF(N26&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P26" s="130" t="s">
@@ -7842,12 +7848,12 @@
         <f t="array" ref="M27">SACCR_LambdaCRR($E27,$F27,$G27)</f>
         <v>5.5</v>
       </c>
-      <c r="N27" s="126">
-        <f>IFERROR(ABS(M27-L27),"")</f>
+      <c r="N27" s="132">
+        <f>IFERROR(ABS(M27-L27)/MAX(1,ABS(L27)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O27" s="127" t="str">
-        <f>IF(ISNUMBER(N27),IF(N27&lt;=FormulaTest_Tolerance*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N27),IF(N27&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P27" s="130" t="s">
@@ -7878,12 +7884,12 @@
         <f t="array" ref="M28">SACCR_LambdaCRR($E28,$F28,$G28)</f>
         <v>0.0</v>
       </c>
-      <c r="N28" s="126">
-        <f>IFERROR(ABS(M28-L28),"")</f>
+      <c r="N28" s="132">
+        <f>IFERROR(ABS(M28-L28)/MAX(1,ABS(L28)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O28" s="127" t="str">
-        <f>IF(ISNUMBER(N28),IF(N28&lt;=FormulaTest_Tolerance*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N28),IF(N28&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P28" s="130" t="s">
@@ -7892,7 +7898,7 @@
     </row>
   </sheetData>
   <dataValidations count="31">
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%. Below about 0.00000000000001% (1e-16, double precision) only an exact match passes." sqref="E4">
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test: a row passes when its Rel. diff, |Function - Expected| / max(1, |Expected|), is at most this value. Default 0.001%. Below about 1e-16 (double precision) only an exact match passes." sqref="E4">
       <formula1>AND(ISNUMBER(E4),E4&gt;0,E4&lt;=0.01)</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E7:E9">

</xml_diff>

<commit_message>
FormulaTest: normal CDF tail test at -4 instead of -8
Normal CDF(-8) is about 6e-16, so against max(1, |Expected|) any
function result near 0 passed and the row tested little. The row now
evaluates x = -4 (about 3.17e-5), still in the tail branch of the
rational approximation. Owner's request.

Validated: python tools/check.py, all gates pass; the VBA algorithm
transcribed to Python gives 3.167124183311601e-05 against the exact
3.1671241833119965e-05 (difference 4e-18, 1.2e-13 relative to the
value). Excel not run.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -1738,7 +1738,7 @@
     <t>=SACCR_NormCDF(1.96)</t>
   </si>
   <si>
-    <t>Normal CDF(-8)</t>
+    <t>Normal CDF(-4)</t>
   </si>
   <si>
     <t>=SACCR_NormCDF(-8)</t>
@@ -7694,19 +7694,19 @@
         <v>880</v>
       </c>
       <c r="E23" s="129">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="L23" s="125">
         <f>_xlfn.NORM.S.DIST($E23,TRUE)</f>
-        <v>6.220960574271819e-16</v>
+        <v>3.1671241833119965e-05</v>
       </c>
       <c r="M23" s="125" cm="1">
         <f t="array" ref="M23">SACCR_NormCDF($E23)</f>
-        <v>6.220960520142784e-16</v>
+        <v>3.167124183311601e-05</v>
       </c>
       <c r="N23" s="132">
         <f>IFERROR(ABS(M23-L23)/MAX(1,ABS(L23)),"")</f>
-        <v>5.4129035033506995e-24</v>
+        <v>3.957337929572091e-18</v>
       </c>
       <c r="O23" s="127" t="str">
         <f>IF(ISNUMBER(N23),IF(N23&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>

</xml_diff>

<commit_message>
FormulaTest: tolerance beside its label, row 3 removed, Rel. diff, multiplier overflow (#167)
Tolerance value in E4 beside its label (FormulaTest_Tolerance); empty
row 3 removed, so headers are on row 6 and tests on rows 7-28 like the
output sheets; the difference column is Rel. diff = |Function -
Expected| / max(1, |Expected|) in the tolerance's percentage format,
compared directly with it; the multiplier Expected returns 1 for a
positive V - C before EXP (it overflowed for V - C = 20, add-on 0.01;
review finding on #166); the normal CDF tail test uses x = -4.

Validated: python tools/check.py, all gates pass; LibreOffice with the
cached values removed recalculates the Expected values and the
tolerance rule as specified. Owner confirmed the template and asked to
merge.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -28,7 +28,7 @@
     <definedName name="BasisFactor">Params!$E$17</definedName>
     <definedName name="BusinessDaysPerYear">Params!$E$11</definedName>
     <definedName name="DaysPerYear">Params!$E$10</definedName>
-    <definedName name="FormulaTest_Tolerance">FormulaTest!$D$5</definedName>
+    <definedName name="FormulaTest_Tolerance">FormulaTest!$E$4</definedName>
     <definedName name="FX_Table">Params!$C$57:$E$62</definedName>
     <definedName name="IRBucketOffset">Params!$E$22</definedName>
     <definedName name="IRCorrBucket12">Params!$E$19</definedName>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="898">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="899">
   <si>
     <t>SA-CCR Calculator</t>
   </si>
@@ -1738,7 +1738,7 @@
     <t>=SACCR_NormCDF(1.96)</t>
   </si>
   <si>
-    <t>Normal CDF(-8)</t>
+    <t>Normal CDF(-4)</t>
   </si>
   <si>
     <t>=SACCR_NormCDF(-8)</t>
@@ -2791,13 +2791,16 @@
     <t>Rule</t>
   </si>
   <si>
-    <t>Tolerance: a test passes when |Function - Expected| &lt;= tolerance x max(1, |Expected|)</t>
+    <t>Tolerance: a test passes when its Rel. diff is at most this value</t>
   </si>
   <si>
     <t>FormulaTest</t>
   </si>
   <si>
     <t>Formula tests</t>
+  </si>
+  <si>
+    <t>Rel. diff</t>
   </si>
 </sst>
 </file>
@@ -3224,7 +3227,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3620,6 +3623,9 @@
     </xf>
     <xf numFmtId="169" fontId="8" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6948,7 +6954,7 @@
     <tabColor rgb="FF548235"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AB29"/>
+  <dimension ref="B1:AB28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="4" customWidth="1"/>
@@ -7022,98 +7028,128 @@
       <c r="AA2" s="68"/>
       <c r="AB2" s="68"/>
     </row>
-    <row r="3" ht="21" x14ac:dyDescent="0.25">
-      <c r="C3" s="1"/>
-    </row>
-    <row r="4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="2" t="s">
+    <row r="3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="2" t="s">
         <v>508</v>
       </c>
     </row>
+    <row r="4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="128" t="s">
+        <v>895</v>
+      </c>
+      <c r="E4" s="131">
+        <v>1.0000000000000001E-5</v>
+      </c>
+    </row>
     <row r="5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="128" t="s">
-        <v>895</v>
-      </c>
-      <c r="D5" s="131">
-        <v>1.0000000000000001E-5</v>
-      </c>
-    </row>
-    <row r="6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="48" t="s">
+      <c r="C5" s="48" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="54" t="s">
+    <row r="6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="54" t="s">
         <v>510</v>
       </c>
-      <c r="D7" s="54" t="s">
+      <c r="D6" s="54" t="s">
         <v>884</v>
       </c>
-      <c r="E7" s="55" t="s">
+      <c r="E6" s="55" t="s">
         <v>885</v>
       </c>
-      <c r="F7" s="55" t="s">
+      <c r="F6" s="55" t="s">
         <v>886</v>
       </c>
-      <c r="G7" s="55" t="s">
+      <c r="G6" s="55" t="s">
         <v>887</v>
       </c>
-      <c r="H7" s="55" t="s">
+      <c r="H6" s="55" t="s">
         <v>888</v>
       </c>
-      <c r="I7" s="55" t="s">
+      <c r="I6" s="55" t="s">
         <v>889</v>
       </c>
-      <c r="J7" s="55" t="s">
+      <c r="J6" s="55" t="s">
         <v>890</v>
       </c>
-      <c r="K7" s="55" t="s">
+      <c r="K6" s="55" t="s">
         <v>891</v>
       </c>
-      <c r="L7" s="55" t="s">
+      <c r="L6" s="55" t="s">
         <v>892</v>
       </c>
-      <c r="M7" s="55" t="s">
+      <c r="M6" s="55" t="s">
         <v>893</v>
       </c>
-      <c r="N7" s="55" t="s">
-        <v>514</v>
-      </c>
-      <c r="O7" s="55" t="s">
+      <c r="N6" s="55" t="s">
+        <v>898</v>
+      </c>
+      <c r="O6" s="55" t="s">
         <v>515</v>
       </c>
-      <c r="P7" s="54" t="s">
+      <c r="P6" s="54" t="s">
         <v>894</v>
+      </c>
+    </row>
+    <row r="7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="128" t="s">
+        <v>516</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>859</v>
+      </c>
+      <c r="E7" s="129">
+        <v>0</v>
+      </c>
+      <c r="F7" s="129">
+        <v>10</v>
+      </c>
+      <c r="L7" s="125">
+        <f>(EXP(-0.05*MAX($E7,0))-EXP(-0.05*$F7))/0.05</f>
+        <v>7.8693868057473315</v>
+      </c>
+      <c r="M7" s="125" cm="1">
+        <f t="array" ref="M7">SACCR_SupervisoryDuration($E7,$F7)</f>
+        <v>7.8693868057473315</v>
+      </c>
+      <c r="N7" s="132">
+        <f>IFERROR(ABS(M7-L7)/MAX(1,ABS(L7)),"")</f>
+        <v>0.0</v>
+      </c>
+      <c r="O7" s="127" t="str">
+        <f>IF(ISNUMBER(N7),IF(N7&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P7" s="130" t="s">
+        <v>860</v>
       </c>
     </row>
     <row r="8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="128" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>859</v>
       </c>
       <c r="E8" s="129">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="129">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L8" s="125">
         <f>(EXP(-0.05*MAX($E8,0))-EXP(-0.05*$F8))/0.05</f>
-        <v>7.8693868057473315</v>
+        <v>7.485592282404547</v>
       </c>
       <c r="M8" s="125" cm="1">
         <f t="array" ref="M8">SACCR_SupervisoryDuration($E8,$F8)</f>
-        <v>7.8693868057473315</v>
-      </c>
-      <c r="N8" s="126">
-        <f>IFERROR(ABS(M8-L8),"")</f>
+        <v>7.485592282404547</v>
+      </c>
+      <c r="N8" s="132">
+        <f>IFERROR(ABS(M8-L8)/MAX(1,ABS(L8)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O8" s="127" t="str">
-        <f>IF(ISNUMBER(N8),IF(N8&lt;=FormulaTest_Tolerance*MAX(1,ABS(L8)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N8),IF(N8&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P8" s="130" t="s">
@@ -7122,31 +7158,35 @@
     </row>
     <row r="9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="128" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>859</v>
+        <v>861</v>
       </c>
       <c r="E9" s="129">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="129">
-        <v>11</v>
+        <v>0.01</v>
+      </c>
+      <c r="G9" s="129">
+        <f>10/250</f>
+        <v>0.04</v>
       </c>
       <c r="L9" s="125">
-        <f>(EXP(-0.05*MAX($E9,0))-EXP(-0.05*$F9))/0.05</f>
-        <v>7.485592282404547</v>
+        <f>MAX((EXP(-0.05*MAX($E9,0))-EXP(-0.05*$F9))/0.05,$G9)</f>
+        <v>0.04</v>
       </c>
       <c r="M9" s="125" cm="1">
-        <f t="array" ref="M9">SACCR_SupervisoryDuration($E9,$F9)</f>
-        <v>7.485592282404547</v>
-      </c>
-      <c r="N9" s="126">
-        <f>IFERROR(ABS(M9-L9),"")</f>
+        <f t="array" ref="M9">SACCR_SupervisoryDuration($E9,$F9,$G9)</f>
+        <v>0.04</v>
+      </c>
+      <c r="N9" s="132">
+        <f>IFERROR(ABS(M9-L9)/MAX(1,ABS(L9)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O9" s="127" t="str">
-        <f>IF(ISNUMBER(N9),IF(N9&lt;=FormulaTest_Tolerance*MAX(1,ABS(L9)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N9),IF(N9&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P9" s="130" t="s">
@@ -7155,65 +7195,59 @@
     </row>
     <row r="10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="128" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="E10" s="129">
-        <v>0</v>
-      </c>
-      <c r="F10" s="129">
-        <v>0.01</v>
-      </c>
-      <c r="G10" s="129">
-        <f>10/250</f>
-        <v>0.04</v>
+        <v>0.75</v>
       </c>
       <c r="L10" s="125">
-        <f>MAX((EXP(-0.05*MAX($E10,0))-EXP(-0.05*$F10))/0.05,$G10)</f>
-        <v>0.04</v>
+        <f>SQRT(MIN(MAX($E10,10/250),1))</f>
+        <v>0.8660254037844386</v>
       </c>
       <c r="M10" s="125" cm="1">
-        <f t="array" ref="M10">SACCR_SupervisoryDuration($E10,$F10,$G10)</f>
-        <v>0.04</v>
-      </c>
-      <c r="N10" s="126">
-        <f>IFERROR(ABS(M10-L10),"")</f>
+        <f t="array" ref="M10">SACCR_MaturityFactor($E10)</f>
+        <v>0.8660254037844386</v>
+      </c>
+      <c r="N10" s="132">
+        <f>IFERROR(ABS(M10-L10)/MAX(1,ABS(L10)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O10" s="127" t="str">
-        <f>IF(ISNUMBER(N10),IF(N10&lt;=FormulaTest_Tolerance*MAX(1,ABS(L10)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N10),IF(N10&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P10" s="130" t="s">
-        <v>860</v>
+        <v>863</v>
       </c>
     </row>
     <row r="11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="128" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D11" s="24" t="s">
         <v>862</v>
       </c>
       <c r="E11" s="129">
-        <v>0.75</v>
+        <f>3/365</f>
+        <v>0.00821917808219178</v>
       </c>
       <c r="L11" s="125">
         <f>SQRT(MIN(MAX($E11,10/250),1))</f>
-        <v>0.8660254037844386</v>
+        <v>0.2</v>
       </c>
       <c r="M11" s="125" cm="1">
         <f t="array" ref="M11">SACCR_MaturityFactor($E11)</f>
-        <v>0.8660254037844386</v>
-      </c>
-      <c r="N11" s="126">
-        <f>IFERROR(ABS(M11-L11),"")</f>
+        <v>0.2</v>
+      </c>
+      <c r="N11" s="132">
+        <f>IFERROR(ABS(M11-L11)/MAX(1,ABS(L11)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O11" s="127" t="str">
-        <f>IF(ISNUMBER(N11),IF(N11&lt;=FormulaTest_Tolerance*MAX(1,ABS(L11)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N11),IF(N11&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P11" s="130" t="s">
@@ -7222,110 +7256,124 @@
     </row>
     <row r="12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="128" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="E12" s="129">
-        <f>3/365</f>
-        <v>0.00821917808219178</v>
+        <v>0</v>
+      </c>
+      <c r="F12" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="129">
+        <v>10</v>
       </c>
       <c r="L12" s="125">
-        <f>SQRT(MIN(MAX($E12,10/250),1))</f>
-        <v>0.2</v>
+        <f>IF($F12,1.5*SQRT($G12/250),SQRT(MIN(MAX($E12,10/250),1)))</f>
+        <v>0.30000000000000004</v>
       </c>
       <c r="M12" s="125" cm="1">
-        <f t="array" ref="M12">SACCR_MaturityFactor($E12)</f>
-        <v>0.2</v>
-      </c>
-      <c r="N12" s="126">
-        <f>IFERROR(ABS(M12-L12),"")</f>
+        <f t="array" ref="M12">SACCR_MaturityFactor($E12,$F12,$G12)</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="N12" s="132">
+        <f>IFERROR(ABS(M12-L12)/MAX(1,ABS(L12)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O12" s="127" t="str">
-        <f>IF(ISNUMBER(N12),IF(N12&lt;=FormulaTest_Tolerance*MAX(1,ABS(L12)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N12),IF(N12&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P12" s="130" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
     </row>
     <row r="13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="128" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>864</v>
+        <v>866</v>
       </c>
       <c r="E13" s="129">
+        <v>0.06</v>
+      </c>
+      <c r="F13" s="129">
+        <v>0.05</v>
+      </c>
+      <c r="G13" s="129">
+        <v>1</v>
+      </c>
+      <c r="H13" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="I13" s="129" t="b">
         <v>0</v>
       </c>
-      <c r="F13" s="129" t="b">
+      <c r="J13" s="129" t="b">
         <v>1</v>
       </c>
-      <c r="G13" s="129">
-        <v>10</v>
-      </c>
       <c r="L13" s="125">
-        <f>IF($F13,1.5*SQRT($G13/250),SQRT(MIN(MAX($E13,10/250),1)))</f>
-        <v>0.30000000000000004</v>
+        <f>IF($I13,_xlfn.NORM.S.DIST((LN(($E13+$K13)/($F13+$K13))+$H13^2*$G13/2)/($H13*SQRT($G13)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E13+$K13)/($F13+$K13))+$H13^2*$G13/2)/($H13*SQRT($G13)),TRUE))*IF($J13,1,-1)</f>
+        <v>-0.2693952177105327</v>
       </c>
       <c r="M13" s="125" cm="1">
-        <f t="array" ref="M13">SACCR_MaturityFactor($E13,$F13,$G13)</f>
-        <v>0.30000000000000004</v>
-      </c>
-      <c r="N13" s="126">
-        <f>IFERROR(ABS(M13-L13),"")</f>
+        <f t="array" ref="M13">SACCR_OptionDelta($E13,$F13,$G13,$H13,$I13,$J13)</f>
+        <v>-0.2693952177105327</v>
+      </c>
+      <c r="N13" s="132">
+        <f>IFERROR(ABS(M13-L13)/MAX(1,ABS(L13)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O13" s="127" t="str">
-        <f>IF(ISNUMBER(N13),IF(N13&lt;=FormulaTest_Tolerance*MAX(1,ABS(L13)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N13),IF(N13&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P13" s="130" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
     </row>
     <row r="14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="128" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D14" s="24" t="s">
         <v>866</v>
       </c>
       <c r="E14" s="129">
-        <v>0.06</v>
+        <v>100</v>
       </c>
       <c r="F14" s="129">
-        <v>0.05</v>
+        <v>110</v>
       </c>
       <c r="G14" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="H14" s="129">
+        <v>0.32</v>
+      </c>
+      <c r="I14" s="129" t="b">
         <v>1</v>
       </c>
-      <c r="H14" s="129">
-        <v>0.5</v>
-      </c>
-      <c r="I14" s="129" t="b">
+      <c r="J14" s="129" t="b">
         <v>0</v>
-      </c>
-      <c r="J14" s="129" t="b">
-        <v>1</v>
       </c>
       <c r="L14" s="125">
         <f>IF($I14,_xlfn.NORM.S.DIST((LN(($E14+$K14)/($F14+$K14))+$H14^2*$G14/2)/($H14*SQRT($G14)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E14+$K14)/($F14+$K14))+$H14^2*$G14/2)/($H14*SQRT($G14)),TRUE))*IF($J14,1,-1)</f>
-        <v>-0.2693952177105327</v>
+        <v>-0.37901134582780294</v>
       </c>
       <c r="M14" s="125" cm="1">
         <f t="array" ref="M14">SACCR_OptionDelta($E14,$F14,$G14,$H14,$I14,$J14)</f>
-        <v>-0.2693952177105327</v>
-      </c>
-      <c r="N14" s="126">
-        <f>IFERROR(ABS(M14-L14),"")</f>
+        <v>-0.37901134582780294</v>
+      </c>
+      <c r="N14" s="132">
+        <f>IFERROR(ABS(M14-L14)/MAX(1,ABS(L14)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O14" s="127" t="str">
-        <f>IF(ISNUMBER(N14),IF(N14&lt;=FormulaTest_Tolerance*MAX(1,ABS(L14)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N14),IF(N14&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P14" s="130" t="s">
@@ -7334,241 +7382,229 @@
     </row>
     <row r="15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="128" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>866</v>
+        <v>868</v>
       </c>
       <c r="E15" s="129">
-        <v>100</v>
+        <v>-0.002</v>
       </c>
       <c r="F15" s="129">
-        <v>110</v>
+        <v>0.001</v>
       </c>
       <c r="G15" s="129">
+        <v>2</v>
+      </c>
+      <c r="H15" s="129">
         <v>0.5</v>
-      </c>
-      <c r="H15" s="129">
-        <v>0.32</v>
       </c>
       <c r="I15" s="129" t="b">
         <v>1</v>
       </c>
       <c r="J15" s="129" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K15" s="129">
+        <v>0.01</v>
       </c>
       <c r="L15" s="125">
         <f>IF($I15,_xlfn.NORM.S.DIST((LN(($E15+$K15)/($F15+$K15))+$H15^2*$G15/2)/($H15*SQRT($G15)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E15+$K15)/($F15+$K15))+$H15^2*$G15/2)/($H15*SQRT($G15)),TRUE))*IF($J15,1,-1)</f>
-        <v>-0.37901134582780294</v>
+        <v>0.46143935794124913</v>
       </c>
       <c r="M15" s="125" cm="1">
-        <f t="array" ref="M15">SACCR_OptionDelta($E15,$F15,$G15,$H15,$I15,$J15)</f>
-        <v>-0.37901134582780294</v>
-      </c>
-      <c r="N15" s="126">
-        <f>IFERROR(ABS(M15-L15),"")</f>
+        <f t="array" ref="M15">SACCR_OptionDelta($E15,$F15,$G15,$H15,$I15,$J15,$K15)</f>
+        <v>0.46143935794124913</v>
+      </c>
+      <c r="N15" s="132">
+        <f>IFERROR(ABS(M15-L15)/MAX(1,ABS(L15)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O15" s="127" t="str">
-        <f>IF(ISNUMBER(N15),IF(N15&lt;=FormulaTest_Tolerance*MAX(1,ABS(L15)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N15),IF(N15&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P15" s="130" t="s">
-        <v>867</v>
+        <v>869</v>
       </c>
     </row>
     <row r="16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="128" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>868</v>
+        <v>870</v>
       </c>
       <c r="E16" s="129">
-        <v>-0.002</v>
+        <v>0.03</v>
       </c>
       <c r="F16" s="129">
-        <v>0.001</v>
-      </c>
-      <c r="G16" s="129">
-        <v>2</v>
-      </c>
-      <c r="H16" s="129">
-        <v>0.5</v>
-      </c>
-      <c r="I16" s="129" t="b">
+        <v>0.06</v>
+      </c>
+      <c r="G16" s="129" t="b">
         <v>1</v>
       </c>
-      <c r="J16" s="129" t="b">
-        <v>1</v>
-      </c>
-      <c r="K16" s="129">
-        <v>0.01</v>
-      </c>
       <c r="L16" s="125">
-        <f>IF($I16,_xlfn.NORM.S.DIST((LN(($E16+$K16)/($F16+$K16))+$H16^2*$G16/2)/($H16*SQRT($G16)),TRUE),-_xlfn.NORM.S.DIST(-(LN(($E16+$K16)/($F16+$K16))+$H16^2*$G16/2)/($H16*SQRT($G16)),TRUE))*IF($J16,1,-1)</f>
-        <v>0.46143935794124913</v>
+        <f>15/((1+14*$E16)*(1+14*$F16))*IF($G16,1,-1)</f>
+        <v>5.740967544396817</v>
       </c>
       <c r="M16" s="125" cm="1">
-        <f t="array" ref="M16">SACCR_OptionDelta($E16,$F16,$G16,$H16,$I16,$J16,$K16)</f>
-        <v>0.46143935794124913</v>
-      </c>
-      <c r="N16" s="126">
-        <f>IFERROR(ABS(M16-L16),"")</f>
-        <v>0.0</v>
+        <f t="array" ref="M16">SACCR_CDODelta($E16,$F16,$G16)</f>
+        <v>5.740967544396816</v>
+      </c>
+      <c r="N16" s="132">
+        <f>IFERROR(ABS(M16-L16)/MAX(1,ABS(L16)),"")</f>
+        <v>1.5470883833283245e-16</v>
       </c>
       <c r="O16" s="127" t="str">
-        <f>IF(ISNUMBER(N16),IF(N16&lt;=FormulaTest_Tolerance*MAX(1,ABS(L16)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N16),IF(N16&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P16" s="130" t="s">
-        <v>869</v>
+        <v>871</v>
       </c>
     </row>
     <row r="17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="128" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="D17" s="24" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
       <c r="E17" s="129">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F17" s="129">
-        <v>0.06</v>
-      </c>
-      <c r="G17" s="129" t="b">
-        <v>1</v>
+        <v>-36253.8493844036</v>
+      </c>
+      <c r="G17" s="129">
+        <v>78693.8680574733</v>
       </c>
       <c r="L17" s="125">
-        <f>15/((1+14*$E17)*(1+14*$F17))*IF($G17,1,-1)</f>
-        <v>5.740967544396817</v>
+        <f>SQRT(MAX($E17^2+$F17^2+$G17^2+1.4*$E17*$F17+1.4*$F17*$G17+0.6*$E17*$G17,0))</f>
+        <v>59269.963463710395</v>
       </c>
       <c r="M17" s="125" cm="1">
-        <f t="array" ref="M17">SACCR_CDODelta($E17,$F17,$G17)</f>
-        <v>5.740967544396816</v>
-      </c>
-      <c r="N17" s="126">
-        <f>IFERROR(ABS(M17-L17),"")</f>
-        <v>8.881784197001252e-16</v>
+        <f t="array" ref="M17">SACCR_IREffectiveNotional($E17,$F17,$G17)</f>
+        <v>59269.963463710395</v>
+      </c>
+      <c r="N17" s="132">
+        <f>IFERROR(ABS(M17-L17)/MAX(1,ABS(L17)),"")</f>
+        <v>0.0</v>
       </c>
       <c r="O17" s="127" t="str">
-        <f>IF(ISNUMBER(N17),IF(N17&lt;=FormulaTest_Tolerance*MAX(1,ABS(L17)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N17),IF(N17&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P17" s="130" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
     </row>
     <row r="18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="128" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="D18" s="24" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="E18" s="129">
-        <v>0</v>
+        <v>105.861937916956</v>
       </c>
       <c r="F18" s="129">
-        <v>-36253.8493844036</v>
+        <v>-279.916321663744</v>
       </c>
       <c r="G18" s="129">
-        <v>78693.8680574733</v>
+        <v>168.111404865732</v>
+      </c>
+      <c r="H18" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="I18" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="J18" s="129">
+        <v>0.8</v>
       </c>
       <c r="L18" s="125">
-        <f>SQRT(MAX($E18^2+$F18^2+$G18^2+1.4*$E18*$F18+1.4*$F18*$G18+0.6*$E18*$G18,0))</f>
-        <v>59269.963463710395</v>
+        <f>SQRT(SUMPRODUCT($E18:$G18,$H18:$J18)^2+SUMPRODUCT((1-$H18:$J18^2)*$E18:$G18^2))</f>
+        <v>282.12883185966604</v>
       </c>
       <c r="M18" s="125" cm="1">
-        <f t="array" ref="M18">SACCR_IREffectiveNotional($E18,$F18,$G18)</f>
-        <v>59269.963463710395</v>
-      </c>
-      <c r="N18" s="126">
-        <f>IFERROR(ABS(M18-L18),"")</f>
+        <f t="array" ref="M18">SACCR_FactorAggregation($E18:$G18,$H18:$J18)</f>
+        <v>282.12883185966604</v>
+      </c>
+      <c r="N18" s="132">
+        <f>IFERROR(ABS(M18-L18)/MAX(1,ABS(L18)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O18" s="127" t="str">
-        <f>IF(ISNUMBER(N18),IF(N18&lt;=FormulaTest_Tolerance*MAX(1,ABS(L18)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N18),IF(N18&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P18" s="130" t="s">
-        <v>873</v>
+        <v>875</v>
       </c>
     </row>
     <row r="19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="128" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="E19" s="129">
-        <v>105.861937916956</v>
+        <v>-20</v>
       </c>
       <c r="F19" s="129">
-        <v>-279.916321663744</v>
-      </c>
-      <c r="G19" s="129">
-        <v>168.111404865732</v>
-      </c>
-      <c r="H19" s="129">
-        <v>0.5</v>
-      </c>
-      <c r="I19" s="129">
-        <v>0.5</v>
-      </c>
-      <c r="J19" s="129">
-        <v>0.8</v>
+        <v>282</v>
       </c>
       <c r="L19" s="125">
-        <f>SQRT(SUMPRODUCT($E19:$G19,$H19:$J19)^2+SUMPRODUCT((1-$H19:$J19^2)*$E19:$G19^2))</f>
-        <v>282.12883185966604</v>
+        <f>IF(OR($F19&lt;=0,$E19&gt;0),1,MIN(1,0.05+0.95*EXP($E19/(2*0.95*$F19))))</f>
+        <v>0.9651926811871945</v>
       </c>
       <c r="M19" s="125" cm="1">
-        <f t="array" ref="M19">SACCR_FactorAggregation($E19:$G19,$H19:$J19)</f>
-        <v>282.12883185966604</v>
-      </c>
-      <c r="N19" s="126">
-        <f>IFERROR(ABS(M19-L19),"")</f>
+        <f t="array" ref="M19">SACCR_Multiplier($E19,$F19)</f>
+        <v>0.9651926811871945</v>
+      </c>
+      <c r="N19" s="132">
+        <f>IFERROR(ABS(M19-L19)/MAX(1,ABS(L19)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O19" s="127" t="str">
-        <f>IF(ISNUMBER(N19),IF(N19&lt;=FormulaTest_Tolerance*MAX(1,ABS(L19)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N19),IF(N19&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P19" s="130" t="s">
-        <v>875</v>
+        <v>877</v>
       </c>
     </row>
     <row r="20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="128" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D20" s="24" t="s">
         <v>876</v>
       </c>
       <c r="E20" s="129">
-        <v>-20</v>
+        <v>10</v>
       </c>
       <c r="F20" s="129">
         <v>282</v>
       </c>
       <c r="L20" s="125">
-        <f>IF($F20&lt;=0,1,MIN(1,0.05+0.95*EXP($E20/(2*0.95*$F20))))</f>
-        <v>0.9651926811871945</v>
+        <f>IF(OR($F20&lt;=0,$E20&gt;0),1,MIN(1,0.05+0.95*EXP($E20/(2*0.95*$F20))))</f>
+        <v>1</v>
       </c>
       <c r="M20" s="125" cm="1">
         <f t="array" ref="M20">SACCR_Multiplier($E20,$F20)</f>
-        <v>0.9651926811871945</v>
-      </c>
-      <c r="N20" s="126">
-        <f>IFERROR(ABS(M20-L20),"")</f>
+        <v>1.0</v>
+      </c>
+      <c r="N20" s="132">
+        <f>IFERROR(ABS(M20-L20)/MAX(1,ABS(L20)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O20" s="127" t="str">
-        <f>IF(ISNUMBER(N20),IF(N20&lt;=FormulaTest_Tolerance*MAX(1,ABS(L20)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N20),IF(N20&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P20" s="130" t="s">
@@ -7577,106 +7613,103 @@
     </row>
     <row r="21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="128" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D21" s="24" t="s">
-        <v>876</v>
+        <v>878</v>
       </c>
       <c r="E21" s="129">
+        <v>5</v>
+      </c>
+      <c r="F21" s="129">
         <v>10</v>
       </c>
-      <c r="F21" s="129">
-        <v>282</v>
+      <c r="G21" s="129" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="129">
+        <v>0</v>
+      </c>
+      <c r="I21" s="129">
+        <v>10</v>
+      </c>
+      <c r="J21" s="129">
+        <v>2</v>
       </c>
       <c r="L21" s="125">
-        <f>IF($F21&lt;=0,1,MIN(1,0.05+0.95*EXP($E21/(2*0.95*$F21))))</f>
-        <v>1</v>
+        <f>IF($G21,MAX($E21-$F21,$H21+$I21-$J21,0),MAX($E21-$F21,0))</f>
+        <v>8</v>
       </c>
       <c r="M21" s="125" cm="1">
-        <f t="array" ref="M21">SACCR_Multiplier($E21,$F21)</f>
-        <v>1.0</v>
-      </c>
-      <c r="N21" s="126">
-        <f>IFERROR(ABS(M21-L21),"")</f>
+        <f t="array" ref="M21">SACCR_ReplacementCost($E21,$F21,$G21,$H21,$I21,$J21)</f>
+        <v>8.0</v>
+      </c>
+      <c r="N21" s="132">
+        <f>IFERROR(ABS(M21-L21)/MAX(1,ABS(L21)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O21" s="127" t="str">
-        <f>IF(ISNUMBER(N21),IF(N21&lt;=FormulaTest_Tolerance*MAX(1,ABS(L21)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N21),IF(N21&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P21" s="130" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
     </row>
     <row r="22" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="128" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D22" s="24" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="E22" s="129">
-        <v>5</v>
-      </c>
-      <c r="F22" s="129">
-        <v>10</v>
-      </c>
-      <c r="G22" s="129" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="129">
-        <v>0</v>
-      </c>
-      <c r="I22" s="129">
-        <v>10</v>
-      </c>
-      <c r="J22" s="129">
-        <v>2</v>
+        <v>1.96</v>
       </c>
       <c r="L22" s="125">
-        <f>IF($G22,MAX($E22-$F22,$H22+$I22-$J22,0),MAX($E22-$F22,0))</f>
-        <v>8</v>
+        <f>_xlfn.NORM.S.DIST($E22,TRUE)</f>
+        <v>0.9750021048517795</v>
       </c>
       <c r="M22" s="125" cm="1">
-        <f t="array" ref="M22">SACCR_ReplacementCost($E22,$F22,$G22,$H22,$I22,$J22)</f>
-        <v>8.0</v>
-      </c>
-      <c r="N22" s="126">
-        <f>IFERROR(ABS(M22-L22),"")</f>
+        <f t="array" ref="M22">SACCR_NormCDF($E22)</f>
+        <v>0.9750021048517795</v>
+      </c>
+      <c r="N22" s="132">
+        <f>IFERROR(ABS(M22-L22)/MAX(1,ABS(L22)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O22" s="127" t="str">
-        <f>IF(ISNUMBER(N22),IF(N22&lt;=FormulaTest_Tolerance*MAX(1,ABS(L22)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N22),IF(N22&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P22" s="130" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
     </row>
     <row r="23" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="128" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D23" s="24" t="s">
         <v>880</v>
       </c>
       <c r="E23" s="129">
-        <v>1.96</v>
+        <v>-4</v>
       </c>
       <c r="L23" s="125">
         <f>_xlfn.NORM.S.DIST($E23,TRUE)</f>
-        <v>0.9750021048517795</v>
+        <v>3.1671241833119965e-05</v>
       </c>
       <c r="M23" s="125" cm="1">
         <f t="array" ref="M23">SACCR_NormCDF($E23)</f>
-        <v>0.9750021048517795</v>
-      </c>
-      <c r="N23" s="126">
-        <f>IFERROR(ABS(M23-L23),"")</f>
-        <v>0.0</v>
+        <v>3.167124183311601e-05</v>
+      </c>
+      <c r="N23" s="132">
+        <f>IFERROR(ABS(M23-L23)/MAX(1,ABS(L23)),"")</f>
+        <v>3.957337929572091e-18</v>
       </c>
       <c r="O23" s="127" t="str">
-        <f>IF(ISNUMBER(N23),IF(N23&lt;=FormulaTest_Tolerance*MAX(1,ABS(L23)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N23),IF(N23&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P23" s="130" t="s">
@@ -7685,64 +7718,70 @@
     </row>
     <row r="24" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="128" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D24" s="24" t="s">
-        <v>880</v>
+        <v>882</v>
       </c>
       <c r="E24" s="129">
-        <v>-8</v>
+        <v>-0.002</v>
+      </c>
+      <c r="F24" s="129">
+        <v>0.001</v>
+      </c>
+      <c r="G24" s="129" t="b">
+        <v>1</v>
       </c>
       <c r="L24" s="125">
-        <f>_xlfn.NORM.S.DIST($E24,TRUE)</f>
-        <v>6.220960574271819e-16</v>
+        <f>IF($G24,MAX(0.001-MIN($E24,$F24),0),MAX(-(1+0.1)*MIN($E24,$F24),0))</f>
+        <v>0.003</v>
       </c>
       <c r="M24" s="125" cm="1">
-        <f t="array" ref="M24">SACCR_NormCDF($E24)</f>
-        <v>6.220960520142784e-16</v>
-      </c>
-      <c r="N24" s="126">
-        <f>IFERROR(ABS(M24-L24),"")</f>
-        <v>5.4129035033506995e-24</v>
+        <f t="array" ref="M24">SACCR_LambdaCRR($E24,$F24,$G24)</f>
+        <v>0.003</v>
+      </c>
+      <c r="N24" s="132">
+        <f>IFERROR(ABS(M24-L24)/MAX(1,ABS(L24)),"")</f>
+        <v>0.0</v>
       </c>
       <c r="O24" s="127" t="str">
-        <f>IF(ISNUMBER(N24),IF(N24&lt;=FormulaTest_Tolerance*MAX(1,ABS(L24)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N24),IF(N24&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P24" s="130" t="s">
-        <v>881</v>
+        <v>883</v>
       </c>
     </row>
     <row r="25" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="128" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D25" s="24" t="s">
         <v>882</v>
       </c>
       <c r="E25" s="129">
-        <v>-0.002</v>
+        <v>0.02</v>
       </c>
       <c r="F25" s="129">
-        <v>0.001</v>
+        <v>0.03</v>
       </c>
       <c r="G25" s="129" t="b">
         <v>1</v>
       </c>
       <c r="L25" s="125">
         <f>IF($G25,MAX(0.001-MIN($E25,$F25),0),MAX(-(1+0.1)*MIN($E25,$F25),0))</f>
-        <v>0.003</v>
+        <v>0</v>
       </c>
       <c r="M25" s="125" cm="1">
         <f t="array" ref="M25">SACCR_LambdaCRR($E25,$F25,$G25)</f>
-        <v>0.003</v>
-      </c>
-      <c r="N25" s="126">
-        <f>IFERROR(ABS(M25-L25),"")</f>
         <v>0.0</v>
       </c>
+      <c r="N25" s="132">
+        <f>IFERROR(ABS(M25-L25)/MAX(1,ABS(L25)),"")</f>
+        <v>0.0</v>
+      </c>
       <c r="O25" s="127" t="str">
-        <f>IF(ISNUMBER(N25),IF(N25&lt;=FormulaTest_Tolerance*MAX(1,ABS(L25)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N25),IF(N25&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P25" s="130" t="s">
@@ -7751,34 +7790,34 @@
     </row>
     <row r="26" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="128" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="D26" s="24" t="s">
         <v>882</v>
       </c>
       <c r="E26" s="129">
-        <v>0.02</v>
+        <v>0.0005</v>
       </c>
       <c r="F26" s="129">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="G26" s="129" t="b">
         <v>1</v>
       </c>
       <c r="L26" s="125">
         <f>IF($G26,MAX(0.001-MIN($E26,$F26),0),MAX(-(1+0.1)*MIN($E26,$F26),0))</f>
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="M26" s="125" cm="1">
         <f t="array" ref="M26">SACCR_LambdaCRR($E26,$F26,$G26)</f>
+        <v>0.0005</v>
+      </c>
+      <c r="N26" s="132">
+        <f>IFERROR(ABS(M26-L26)/MAX(1,ABS(L26)),"")</f>
         <v>0.0</v>
       </c>
-      <c r="N26" s="126">
-        <f>IFERROR(ABS(M26-L26),"")</f>
-        <v>0.0</v>
-      </c>
       <c r="O26" s="127" t="str">
-        <f>IF(ISNUMBER(N26),IF(N26&lt;=FormulaTest_Tolerance*MAX(1,ABS(L26)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N26),IF(N26&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P26" s="130" t="s">
@@ -7787,34 +7826,34 @@
     </row>
     <row r="27" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="128" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D27" s="24" t="s">
         <v>882</v>
       </c>
       <c r="E27" s="129">
-        <v>0.0005</v>
+        <v>-5</v>
       </c>
       <c r="F27" s="129">
-        <v>0.01</v>
+        <v>-4</v>
       </c>
       <c r="G27" s="129" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L27" s="125">
         <f>IF($G27,MAX(0.001-MIN($E27,$F27),0),MAX(-(1+0.1)*MIN($E27,$F27),0))</f>
-        <v>0.0005</v>
+        <v>5.5</v>
       </c>
       <c r="M27" s="125" cm="1">
         <f t="array" ref="M27">SACCR_LambdaCRR($E27,$F27,$G27)</f>
-        <v>0.0005</v>
-      </c>
-      <c r="N27" s="126">
-        <f>IFERROR(ABS(M27-L27),"")</f>
+        <v>5.5</v>
+      </c>
+      <c r="N27" s="132">
+        <f>IFERROR(ABS(M27-L27)/MAX(1,ABS(L27)),"")</f>
         <v>0.0</v>
       </c>
       <c r="O27" s="127" t="str">
-        <f>IF(ISNUMBER(N27),IF(N27&lt;=FormulaTest_Tolerance*MAX(1,ABS(L27)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N27),IF(N27&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P27" s="130" t="s">
@@ -7823,175 +7862,139 @@
     </row>
     <row r="28" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C28" s="128" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="D28" s="24" t="s">
         <v>882</v>
       </c>
       <c r="E28" s="129">
-        <v>-5</v>
+        <v>40</v>
       </c>
       <c r="F28" s="129">
-        <v>-4</v>
+        <v>35</v>
       </c>
       <c r="G28" s="129" t="b">
         <v>0</v>
       </c>
       <c r="L28" s="125">
         <f>IF($G28,MAX(0.001-MIN($E28,$F28),0),MAX(-(1+0.1)*MIN($E28,$F28),0))</f>
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="M28" s="125" cm="1">
         <f t="array" ref="M28">SACCR_LambdaCRR($E28,$F28,$G28)</f>
-        <v>5.5</v>
-      </c>
-      <c r="N28" s="126">
-        <f>IFERROR(ABS(M28-L28),"")</f>
         <v>0.0</v>
       </c>
+      <c r="N28" s="132">
+        <f>IFERROR(ABS(M28-L28)/MAX(1,ABS(L28)),"")</f>
+        <v>0.0</v>
+      </c>
       <c r="O28" s="127" t="str">
-        <f>IF(ISNUMBER(N28),IF(N28&lt;=FormulaTest_Tolerance*MAX(1,ABS(L28)),"PASS","FAIL"),"FAIL")</f>
+        <f>IF(ISNUMBER(N28),IF(N28&lt;=FormulaTest_Tolerance,"PASS","FAIL"),"FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P28" s="130" t="s">
         <v>883</v>
       </c>
     </row>
-    <row r="29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C29" s="128" t="s">
-        <v>558</v>
-      </c>
-      <c r="D29" s="24" t="s">
-        <v>882</v>
-      </c>
-      <c r="E29" s="129">
-        <v>40</v>
-      </c>
-      <c r="F29" s="129">
-        <v>35</v>
-      </c>
-      <c r="G29" s="129" t="b">
-        <v>0</v>
-      </c>
-      <c r="L29" s="125">
-        <f>IF($G29,MAX(0.001-MIN($E29,$F29),0),MAX(-(1+0.1)*MIN($E29,$F29),0))</f>
-        <v>0</v>
-      </c>
-      <c r="M29" s="125" cm="1">
-        <f t="array" ref="M29">SACCR_LambdaCRR($E29,$F29,$G29)</f>
-        <v>0.0</v>
-      </c>
-      <c r="N29" s="126">
-        <f>IFERROR(ABS(M29-L29),"")</f>
-        <v>0.0</v>
-      </c>
-      <c r="O29" s="127" t="str">
-        <f>IF(ISNUMBER(N29),IF(N29&lt;=FormulaTest_Tolerance*MAX(1,ABS(L29)),"PASS","FAIL"),"FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P29" s="130" t="s">
-        <v>883</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="31">
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test, applied to max(1, |Expected|). Default 0.001%. Below about 0.00000000000001% (1e-16, double precision) only an exact match passes." sqref="D5">
-      <formula1>AND(ISNUMBER(D5),D5&gt;0,D5&lt;=0.01)</formula1>
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid tolerance" error="Enter a percentage above 0% and at most 1%." promptTitle="Tolerance" prompt="Relative tolerance of every unit test: a row passes when its Rel. diff, |Function - Expected| / max(1, |Expected|), is at most this value. Default 0.001%. Below about 1e-16 (double precision) only an exact match passes." sqref="E4">
+      <formula1>AND(ISNUMBER(E4),E4&gt;0,E4&lt;=0.01)</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E8:E10">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid start date" error="Enter a number of years from -50 to 50." promptTitle="Start date S (years)" prompt="Years from today to the start of the period referenced. Zero or negative means already started and is floored at 0 (CRE52.34; CRR Art. 279b(1)(a))." sqref="E7:E9">
       <formula1>-50</formula1>
       <formula2>50</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid end date" error="Enter a number of years after the start date and after 0, at most 50." promptTitle="End date E (years)" prompt="Years from today to the end of the period referenced: after the start date and after today, at most 50 (CRE52.34)." sqref="F8:F10">
-      <formula1>AND(ISNUMBER(F8),F8&gt;MAX(E8,0),F8&lt;=50)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid end date" error="Enter a number of years after the start date and after 0, at most 50." promptTitle="End date E (years)" prompt="Years from today to the end of the period referenced: after the start date and after today, at most 50 (CRE52.34)." sqref="F7:F9">
+      <formula1>AND(ISNUMBER(F7),F7&gt;MAX(E7,0),F7&lt;=50)</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid floor" error="Enter a number of years from 0 to 1." promptTitle="SD floor (years)" prompt="Floor on the supervisory duration, in years: 10 business days = 10/250 (CRE52.34)." sqref="G10">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid floor" error="Enter a number of years from 0 to 1." promptTitle="SD floor (years)" prompt="Floor on the supervisory duration, in years: 10 business days = 10/250 (CRE52.34)." sqref="G9">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid maturity" error="Enter a number of years from 0 to 50." promptTitle="Maturity M (years)" prompt="Remaining maturity in years. The unmargined factor floors it at 10 business days and caps it at 1 year (CRE52.48; CRR Art. 279c(1)(a))." sqref="E11:E13">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid maturity" error="Enter a number of years from 0 to 50." promptTitle="Maturity M (years)" prompt="Remaining maturity in years. The unmargined factor floors it at 10 business days and caps it at 1 year (CRE52.48; CRR Art. 279c(1)(a))." sqref="E10:E12">
       <formula1>0</formula1>
       <formula2>50</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined factor 1.5 x sqrt(MPOR / 250) (CRE52.52; CRR Art. 279c(1)(b)). FALSE = unmargined factor from M." sqref="F13">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined factor 1.5 x sqrt(MPOR / 250) (CRE52.52; CRR Art. 279c(1)(b)). FALSE = unmargined factor from M." sqref="F12">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid MPOR" error="Enter a whole number of business days from 1 to 250." promptTitle="MPOR (business days)" prompt="Margin period of risk in business days, used when margined (CRE52.50-52; CRR Art. 285)." sqref="G13">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid MPOR" error="Enter a whole number of business days from 1 to 250." promptTitle="MPOR (business days)" prompt="Margin period of risk in business days, used when margined (CRE52.50-52; CRR Art. 285)." sqref="G12">
       <formula1>1</formula1>
       <formula2>250</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid price" error="Enter a number; P plus lambda (Input 7) must be above 0." promptTitle="Price P" prompt="Price of the underlying (forward rate for IR options). P plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="E14:E16">
-      <formula1>AND(ISNUMBER(E14),E14+$K14&gt;0)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid price" error="Enter a number; P plus lambda (Input 7) must be above 0." promptTitle="Price P" prompt="Price of the underlying (forward rate for IR options). P plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="E13:E15">
+      <formula1>AND(ISNUMBER(E13),E13+$K13&gt;0)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid strike" error="Enter a number; K plus lambda (Input 7) must be above 0." promptTitle="Strike K" prompt="Strike of the option. K plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="F14:F16">
-      <formula1>AND(ISNUMBER(F14),F14+$K14&gt;0)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid strike" error="Enter a number; K plus lambda (Input 7) must be above 0." promptTitle="Strike K" prompt="Strike of the option. K plus lambda (Input 7) must be above 0 (CRE52.40)." sqref="F13:F15">
+      <formula1>AND(ISNUMBER(F13),F13+$K13&gt;0)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid expiry" error="Enter a number of years above 0, at most 100." promptTitle="Expiry T (years)" prompt="Latest contractual exercise date, in years from today, above 0 (CRE52.40; CRR Art. 279a(1)(a))." sqref="G14:G16">
-      <formula1>AND(ISNUMBER(G14),G14&gt;0,G14&lt;=100)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid expiry" error="Enter a number of years above 0, at most 100." promptTitle="Expiry T (years)" prompt="Latest contractual exercise date, in years from today, above 0 (CRE52.40; CRR Art. 279a(1)(a))." sqref="G13:G15">
+      <formula1>AND(ISNUMBER(G13),G13&gt;0,G13&lt;=100)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid volatility" error="Enter a decimal above 0, at most 5." promptTitle="Supervisory volatility" prompt="Supervisory option volatility as a decimal (0.5 = 50%), above 0 and at most 5 (CRE52.72; CRR Art. 279a)." sqref="H14:H16">
-      <formula1>AND(ISNUMBER(H14),H14&gt;0,H14&lt;=5)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid volatility" error="Enter a decimal above 0, at most 5." promptTitle="Supervisory volatility" prompt="Supervisory option volatility as a decimal (0.5 = 50%), above 0 and at most 5 (CRE52.72; CRR Art. 279a)." sqref="H13:H15">
+      <formula1>AND(ISNUMBER(H13),H13&gt;0,H13&lt;=5)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Call" prompt="TRUE = call option; FALSE = put option (CRE52.40)." sqref="I14:I16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Call" prompt="TRUE = call option; FALSE = put option (CRE52.40)." sqref="I13:I15">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Bought" prompt="TRUE = bought option (long); FALSE = sold option (short) (CRE52.40)." sqref="J14:J16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Bought" prompt="TRUE = bought option (long); FALSE = sold option (short) (CRE52.40)." sqref="J13:J15">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Lambda shift" prompt="Shift added to P and K so that both are above 0 (CRE52.40 FAQ; CRR-RTS Art. 5). 0 or more." sqref="K16">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Lambda shift" prompt="Shift added to P and K so that both are above 0 (CRE52.40 FAQ; CRR-RTS Art. 5). 0 or more." sqref="K15">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid attachment" error="Enter a decimal from 0 to below 1, e.g. 0.03 for 3%." promptTitle="Attachment A" prompt="Attachment point of the tranche, from 0 to below 1 (CRE52.41)." sqref="E17">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid attachment" error="Enter a decimal from 0 to below 1, e.g. 0.03 for 3%." promptTitle="Attachment A" prompt="Attachment point of the tranche, from 0 to below 1 (CRE52.41)." sqref="E16">
       <formula1>0</formula1>
       <formula2>0.9999</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid detachment" error="Enter a decimal above the attachment point and at most 1." promptTitle="Detachment D" prompt="Detachment point, above the attachment and at most 1 (CRE52.41)." sqref="F17">
-      <formula1>AND(ISNUMBER(F17),F17&gt;E17,F17&lt;=1)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid detachment" error="Enter a decimal above the attachment point and at most 1." promptTitle="Detachment D" prompt="Detachment point, above the attachment and at most 1 (CRE52.41)." sqref="F16">
+      <formula1>AND(ISNUMBER(F16),F16&gt;E16,F16&lt;=1)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Long" prompt="TRUE = long in the tranche (positive delta); FALSE = short (CRE52.41)." sqref="G17">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Long" prompt="TRUE = long in the tranche (positive delta); FALSE = short (CRE52.41)." sqref="G16">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Bucket effective notional" prompt="Signed effective notional D of maturity bucket 1, 2 or 3 (under 1 year, 1 to 5 years, over 5 years) (CRE52.57)." sqref="E18:G18">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Bucket effective notional" prompt="Signed effective notional D of maturity bucket 1, 2 or 3 (under 1 year, 1 to 5 years, over 5 years) (CRE52.57)." sqref="E17:G17">
+      <formula1>ISNUMBER(E17)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Entity add-on" prompt="Add-on of entity or commodity type k, signed by direction (CRE52.61; CRR Art. 280c)." sqref="E18:G18">
       <formula1>ISNUMBER(E18)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Entity add-on" prompt="Add-on of entity or commodity type k, signed by direction (CRE52.61; CRR Art. 280c)." sqref="E19:G19">
-      <formula1>ISNUMBER(E19)</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid correlation" error="Enter a decimal from 0 to 1." promptTitle="Correlation" prompt="Correlation of entity k, as a decimal from 0 to 1: credit 0.5 single name, 0.8 index (CRE52.61)." sqref="H19:J19">
+    <dataValidation type="decimal" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid correlation" error="Enter a decimal from 0 to 1." promptTitle="Correlation" prompt="Correlation of entity k, as a decimal from 0 to 1: credit 0.5 single name, 0.8 index (CRE52.61)." sqref="H18:J18">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V - C" prompt="Net market value of the netting set less collateral, signed (CRE52.23; CRR Art. 278(3))." sqref="E20:E21">
-      <formula1>ISNUMBER(E20)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V - C" prompt="Net market value of the netting set less collateral, signed (CRE52.23; CRR Art. 278(3))." sqref="E19:E20">
+      <formula1>ISNUMBER(E19)</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Aggregate add-on" prompt="Aggregate add-on of the netting set, 0 or more; 0 gives a multiplier of 1 (CRE52.23)." sqref="F20:F21">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Aggregate add-on" prompt="Aggregate add-on of the netting set, 0 or more; 0 gives a multiplier of 1 (CRE52.23)." sqref="F19:F20">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V" prompt="Net market value of the trades in the netting set, signed (CRE52.10; CRR Art. 275)." sqref="E22">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="V" prompt="Net market value of the trades in the netting set, signed (CRE52.10; CRR Art. 275)." sqref="E21">
+      <formula1>ISNUMBER(E21)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="C" prompt="Net collateral held after haircuts; negative if posted (CRE52.10; CRR Art. 275)." sqref="F21">
+      <formula1>ISNUMBER(F21)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined RC max(V - C, TH + MTA - NICA, 0) (CRE52.18); FALSE = max(V - C, 0) (CRE52.10)." sqref="G21">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Threshold TH" prompt="Threshold of the margin agreement, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="H21">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Minimum transfer amount" prompt="Minimum transfer amount MTA, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="I21">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="NICA" prompt="Net independent collateral amount, signed; negative if posted (CRE52.13; CRR Art. 275(2))." sqref="J21">
+      <formula1>ISNUMBER(J21)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="x" prompt="Point at which the standard normal distribution function is evaluated." sqref="E22:E23">
       <formula1>ISNUMBER(E22)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="C" prompt="Net collateral held after haircuts; negative if posted (CRE52.10; CRR Art. 275)." sqref="F22">
-      <formula1>ISNUMBER(F22)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Price or strike" prompt="Price P (Input 1) or strike K (Input 2) of the option; negative values allowed (CRR-RTS Art. 5(2))." sqref="E24:F28">
+      <formula1>ISNUMBER(E24)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Margined" prompt="TRUE = margined RC max(V - C, TH + MTA - NICA, 0) (CRE52.18); FALSE = max(V - C, 0) (CRE52.10)." sqref="G22">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Threshold TH" prompt="Threshold of the margin agreement, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="H22">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Enter a number of 0 or more." promptTitle="Minimum transfer amount" prompt="Minimum transfer amount MTA, 0 or more (CRE52.18; CRR Art. 275(2))." sqref="I22">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="NICA" prompt="Net independent collateral amount, signed; negative if posted (CRE52.13; CRR Art. 275(2))." sqref="J22">
-      <formula1>ISNUMBER(J22)</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="x" prompt="Point at which the standard normal distribution function is evaluated." sqref="E23:E24">
-      <formula1>ISNUMBER(E23)</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid number" error="Enter a number." promptTitle="Price or strike" prompt="Price P (Input 1) or strike K (Input 2) of the option; negative values allowed (CRR-RTS Art. 5(2))." sqref="E25:F29">
-      <formula1>ISNUMBER(E25)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Interest rate" prompt="TRUE = interest-rate option (threshold 0.10%); FALSE = commodity option (threshold 0.1) (CRR-RTS Art. 5(2))." sqref="G25:G29">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose TRUE or FALSE." promptTitle="Interest rate" prompt="TRUE = interest-rate option (threshold 0.10%); FALSE = commodity option (threshold 0.1) (CRR-RTS Art. 5(2))." sqref="G24:G28">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reject malformed reporting currencies; test remargin bounds (#147) (#168)
The reporting currency must be three letters A to Z, in the engine
(LoadParams, Like "[A-Z][A-Z][A-Z]" after UTxt) and in the Params E7
validation (through ReportingCcy); case and surrounding spaces are
ignored, and only the format is checked, not ISO 4217 membership. A
malformed code such as E1R stopped nothing and was added to the FX table
at rate 1. TEST_InputValidation covers digits, punctuation, two and four
letters, blank and lower case, and the remargining frequency at 0.5,
10000 (MPOR 10009) and 10001: 97 cases, 129 checks.

Validated: python tools/check.py, all gates pass; CI green; Codex review
without findings. Excel (owner): compile, TEST_InputValidation PASS
97/129, demo unchanged, E1R refused by the validation and stopping the
run when pasted, other suites PASS.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -12759,8 +12759,8 @@
       <formula1>36526</formula1>
       <formula2>73415</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid currency" error="Enter a three-letter ISO currency code, e.g. EUR." promptTitle="Reporting currency" prompt="ISO code, e.g. EUR. Every amount is converted into it with the FX table below." sqref="E7" xr:uid="{00000000-0002-0000-0100-000001000000}">
-      <formula1>AND(ISTEXT(ReportingCcy),LEN(ReportingCcy)=3)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid currency" error="Enter three letters A to Z, e.g. EUR." promptTitle="Reporting currency" prompt="Three-letter currency code, e.g. EUR: letters A to Z only; case and surrounding spaces are ignored. The format is checked, not ISO membership. Every amount is converted into it with the FX table below." sqref="E7" xr:uid="{00000000-0002-0000-0100-000001000000}">
+      <formula1>AND(ISTEXT(ReportingCcy),LEN(TRIM(ReportingCcy))=3,ABS(CODE(MID(UPPER(TRIM(ReportingCcy)),1,1))-77.5)&lt;13,ABS(CODE(MID(UPPER(TRIM(ReportingCcy)),2,1))-77.5)&lt;13,ABS(CODE(MID(UPPER(TRIM(ReportingCcy)),3,1))-77.5)&lt;13)</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid alpha" error="Alpha must be a number greater than zero. Regulatory value: 1.4." promptTitle="Alpha" prompt="Multiplier on RC + PFE. Regulatory value 1.4 (CRE52.1, CRR Art. 274(2))." sqref="E8" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
Say in the template that IR and credit options need a start date (#40)
The template still told users that a blank start date means "already
started" (README D19 and the input message of Trades column Q), which
now rejects an IR or credit option. Both now say that such an option
needs the start of its underlying: a swaption's exercise date, the
earliest one if Bermudan, or a cap's or floor's first period.

The two strings were replaced in xl/sharedStrings.xml and
xl/worksheets/sheet4.xml inside the package, every other part copied
byte for byte, so the data validation extensions that openpyxl would
drop are kept. CHANGELOG updated.

Validated: python tools/check.py passes; the package opens in openpyxl
with the new README text and passes a zip integrity test. Not yet
opened in Excel.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -172,7 +172,7 @@
     <t>Dates</t>
   </si>
   <si>
-    <t>Start (S, IR/CR only, blank = already started), End (E, IR/CR, also defines the IR maturity bucket), Maturity (M, maturity factor; defaults to End, then Expiry), Option expiry (T, options). Year fractions = days / DaysPerYear.</t>
+    <t>Start (S, IR/CR only; blank = already started, except for IR/CR options, which need the start of the underlying: a swaption's exercise date, the earliest one if Bermudan, or a cap's or floor's first period; CRE52.31, CRE52.42), End (E, IR/CR, also defines the IR maturity bucket), Maturity (M, maturity factor; defaults to End, then Expiry), Option expiry (T, options). Year fractions = days / DaysPerYear.</t>
   </si>
   <si>
     <t>Nature</t>
@@ -48027,7 +48027,7 @@
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid MtM" error="Enter a number (0 if the trade has no value)." promptTitle="MtM" prompt="Mark-to-market value, signed: positive is an asset. Enter 0 if the trade has no value." sqref="O5:O5000" xr:uid="{00000000-0002-0000-0300-00000C000000}">
       <formula1>ISNUMBER(O5)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid date" error="Enter a date between 1950 and 2200." promptTitle="Start date (S)" prompt="IR and credit: start of the time period referenced; blank = already started (CRE52.31)." sqref="Q5:Q5000" xr:uid="{00000000-0002-0000-0300-00000E000000}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid date" error="Enter a date between 1950 and 2200." promptTitle="Start date (S)" prompt="IR and credit: start of the time period referenced; blank = already started (CRE52.31). Required for IR/credit options: a swaption's exercise date, the earliest if Bermudan." sqref="Q5:Q5000" xr:uid="{00000000-0002-0000-0300-00000E000000}">
       <formula1>AND(ISNUMBER(Q5),Q5&gt;=DATE(1950,1,1),Q5&lt;=DATE(2200,12,31))</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid end date" error="Enter a date between 1950 and 2200, after the start date." promptTitle="End date (E)" prompt="IR and credit: end of the time period referenced (CRE52.31)." sqref="R5:R5000" xr:uid="{00000000-0002-0000-0300-00000F000000}">

</xml_diff>

<commit_message>
Link the README sheet to the EAD reference card
Add a hyperlink in README!D23, on the "Methodology (per netting set)"
heading row, to docs/assets/SACCR_EAD_reference.svg on main:
=HYPERLINK(url, "One-page reference card: all formulas and parameters
(opens on GitHub)"). The cell gets a new style (Aptos 9, underlined,
link blue, right-aligned, the heading's bottom border); no rows, names
or other cells move. The link resolves once the card reaches main.

The template was patched at XML level (styles.xml, sheet1.xml) so the
data-validation extensions are preserved. CHANGELOG notes the link.

Validation: package integrity checked; openpyxl reads D23 with the
formula and style; LibreOffice render of README shows the link on the
heading row; python tools/check.py passes. Not yet opened in Excel.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -2818,7 +2818,7 @@
     <numFmt numFmtId="171" formatCode="0.0E+00"/>
     <numFmt numFmtId="172" formatCode="0.000000000"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2996,6 +2996,13 @@
       <b/>
       <sz val="9"/>
       <color rgb="FF375623"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color rgb="FF0563C1"/>
       <name val="Aptos"/>
       <family val="2"/>
     </font>
@@ -3227,7 +3234,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3626,6 +3633,9 @@
     </xf>
     <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4838,7 +4848,10 @@
       <c r="C23" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="37"/>
+      <c r="D23" s="133" t="str">
+        <f>HYPERLINK("https://github.com/danielep71/VBA-SACCR-Toolkit/blob/main/docs/assets/SACCR_EAD_reference.svg","One-page reference card: all formulas and parameters (opens on GitHub)")</f>
+        <v>One-page reference card: all formulas and parameters (opens on GitHub)</v>
+      </c>
     </row>
     <row r="24" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="25" t="s">

</xml_diff>

<commit_message>
Link the README sheet to the EAD reference card (#225)
README!D23, on the "Methodology (per netting set)" heading row, holds =HYPERLINK to docs/assets/SACCR_EAD_reference.svg on main, styled Aptos 9, underlined, link blue, right-aligned, with the heading's bottom border. No rows, names or other cells move. The template was patched at XML level so the data-validation extensions are preserved. The link resolves once the card reaches main.

Validation: package integrity, openpyxl read of D23, LibreOffice render; python tools/check.py passes; Codex review with no findings. Owner Excel check of the template (2026-10-15): link shown in D23 with the expected style, URL correct, rest of the sheet unchanged.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -2818,7 +2818,7 @@
     <numFmt numFmtId="171" formatCode="0.0E+00"/>
     <numFmt numFmtId="172" formatCode="0.000000000"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2996,6 +2996,13 @@
       <b/>
       <sz val="9"/>
       <color rgb="FF375623"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color rgb="FF0563C1"/>
       <name val="Aptos"/>
       <family val="2"/>
     </font>
@@ -3227,7 +3234,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3626,6 +3633,9 @@
     </xf>
     <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4838,7 +4848,10 @@
       <c r="C23" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="37"/>
+      <c r="D23" s="133" t="str">
+        <f>HYPERLINK("https://github.com/danielep71/VBA-SACCR-Toolkit/blob/main/docs/assets/SACCR_EAD_reference.svg","One-page reference card: all formulas and parameters (opens on GitHub)")</f>
+        <v>One-page reference card: all formulas and parameters (opens on GitHub)</v>
+      </c>
     </row>
     <row r="24" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="25" t="s">

</xml_diff>

<commit_message>
Widen README column C and border its sections
README sheet: column C goes from 46 to 55. Every section table (How to
use, Sign and input conventions, Methodology, Sheets, Worksheet
functions, Scope and limitations, Code) gets a thin outer border and
dashed lines between rows and between columns C and D.

The borders come from eight new cell styles, copies of the existing
label (C) and text (D) styles with a border added; fonts, alignment
and wrapping are unchanged, and no row, name or value moves. Patched
at XML level, so the data-validation extensions are preserved.

Validation: package integrity checked; openpyxl reads the width and
the borders; LibreOffice render of the README sheet shows every
section framed; python tools/check.py passes. Not yet opened in Excel.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -3057,7 +3057,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -3228,13 +3228,133 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3636,6 +3756,30 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4683,7 +4827,7 @@
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="4" customWidth="1"/>
-    <col min="3" max="3" width="46" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
     <col min="4" max="4" width="126.875" customWidth="1"/>
     <col min="5" max="5" width="4.75" customWidth="1"/>
     <col min="6" max="24" width="0" hidden="1" customWidth="1"/>
@@ -4719,58 +4863,58 @@
       <c r="D5" s="3"/>
     </row>
     <row r="6" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="134" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="138" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="135" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="139" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="135" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="139" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="9" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="135" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="139" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="135" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="D10" s="139" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="11" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="135" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="139" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="136" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="34" t="s">
+      <c r="D12" s="140" t="s">
         <v>16</v>
       </c>
     </row>
@@ -4785,58 +4929,58 @@
       <c r="D14" s="37"/>
     </row>
     <row r="15" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="134" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="138" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" spans="2:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="135" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="139" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="17" spans="3:4" ht="24" x14ac:dyDescent="0.25">
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="135" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="139" t="s">
         <v>801</v>
       </c>
     </row>
     <row r="18" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="135" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="34" t="s">
+      <c r="D18" s="139" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="135" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="34" t="s">
+      <c r="D19" s="139" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="20" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="135" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="34" t="s">
+      <c r="D20" s="139" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="21" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="136" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="34" t="s">
+      <c r="D21" s="140" t="s">
         <v>30</v>
       </c>
     </row>
@@ -4854,90 +4998,90 @@
       </c>
     </row>
     <row r="24" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="25" t="s">
+      <c r="C24" s="134" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="34" t="s">
+      <c r="D24" s="138" t="s">
         <v>815</v>
       </c>
     </row>
     <row r="25" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="25" t="s">
+      <c r="C25" s="135" t="s">
         <v>33</v>
       </c>
-      <c r="D25" s="34" t="s">
+      <c r="D25" s="139" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="26" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="25" t="s">
+      <c r="C26" s="135" t="s">
         <v>35</v>
       </c>
-      <c r="D26" s="34" t="s">
+      <c r="D26" s="139" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="27" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="25" t="s">
+      <c r="C27" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="D27" s="34" t="s">
+      <c r="D27" s="139" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="28" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C28" s="25" t="s">
+      <c r="C28" s="135" t="s">
         <v>39</v>
       </c>
-      <c r="D28" s="34" t="s">
+      <c r="D28" s="139" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="29" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C29" s="25" t="s">
+      <c r="C29" s="135" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="34" t="s">
+      <c r="D29" s="139" t="s">
         <v>816</v>
       </c>
     </row>
     <row r="30" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C30" s="25" t="s">
+      <c r="C30" s="135" t="s">
         <v>42</v>
       </c>
-      <c r="D30" s="34" t="s">
+      <c r="D30" s="139" t="s">
         <v>802</v>
       </c>
     </row>
     <row r="31" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C31" s="25" t="s">
+      <c r="C31" s="135" t="s">
         <v>43</v>
       </c>
-      <c r="D31" s="34" t="s">
+      <c r="D31" s="139" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="32" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C32" s="25" t="s">
+      <c r="C32" s="135" t="s">
         <v>45</v>
       </c>
-      <c r="D32" s="34" t="s">
+      <c r="D32" s="139" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="33" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C33" s="25" t="s">
+      <c r="C33" s="135" t="s">
         <v>47</v>
       </c>
-      <c r="D33" s="34" t="s">
+      <c r="D33" s="139" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="34" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C34" s="25" t="s">
+      <c r="C34" s="136" t="s">
         <v>49</v>
       </c>
-      <c r="D34" s="34" t="s">
+      <c r="D34" s="140" t="s">
         <v>50</v>
       </c>
     </row>
@@ -4952,90 +5096,90 @@
       <c r="D36" s="37"/>
     </row>
     <row r="37" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C37" s="25" t="s">
+      <c r="C37" s="134" t="s">
         <v>52</v>
       </c>
-      <c r="D37" s="34" t="s">
+      <c r="D37" s="138" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="38" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C38" s="25" t="s">
+      <c r="C38" s="135" t="s">
         <v>54</v>
       </c>
-      <c r="D38" s="34" t="s">
+      <c r="D38" s="139" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="39" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="25" t="s">
+      <c r="C39" s="135" t="s">
         <v>56</v>
       </c>
-      <c r="D39" s="34" t="s">
+      <c r="D39" s="139" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="40" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C40" s="25" t="s">
+      <c r="C40" s="135" t="s">
         <v>58</v>
       </c>
-      <c r="D40" s="34" t="s">
+      <c r="D40" s="139" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="41" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C41" s="25" t="s">
+      <c r="C41" s="135" t="s">
         <v>60</v>
       </c>
-      <c r="D41" s="34" t="s">
+      <c r="D41" s="139" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="42" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C42" s="25" t="s">
+      <c r="C42" s="135" t="s">
         <v>62</v>
       </c>
-      <c r="D42" s="34" t="s">
+      <c r="D42" s="139" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="43" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C43" s="25" t="s">
+      <c r="C43" s="135" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="34" t="s">
+      <c r="D43" s="139" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="44" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C44" s="25" t="s">
+      <c r="C44" s="135" t="s">
         <v>66</v>
       </c>
-      <c r="D44" s="34" t="s">
+      <c r="D44" s="139" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="45" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C45" s="25" t="s">
+      <c r="C45" s="135" t="s">
         <v>68</v>
       </c>
-      <c r="D45" s="34" t="s">
+      <c r="D45" s="139" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="46" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="25" t="s">
+      <c r="C46" s="135" t="s">
         <v>896</v>
       </c>
-      <c r="D46" s="34" t="s">
+      <c r="D46" s="139" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="47" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="25" t="s">
+      <c r="C47" s="136" t="s">
         <v>72</v>
       </c>
-      <c r="D47" s="34" t="s">
+      <c r="D47" s="140" t="s">
         <v>73</v>
       </c>
     </row>
@@ -5050,82 +5194,82 @@
       <c r="D49" s="37"/>
     </row>
     <row r="50" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="25" t="s">
+      <c r="C50" s="134" t="s">
         <v>75</v>
       </c>
-      <c r="D50" s="34" t="s">
+      <c r="D50" s="138" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="51" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C51" s="25" t="s">
+      <c r="C51" s="135" t="s">
         <v>77</v>
       </c>
-      <c r="D51" s="34" t="s">
+      <c r="D51" s="139" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="52" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C52" s="25" t="s">
+      <c r="C52" s="135" t="s">
         <v>78</v>
       </c>
-      <c r="D52" s="34" t="s">
+      <c r="D52" s="139" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="53" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C53" s="25" t="s">
+      <c r="C53" s="135" t="s">
         <v>80</v>
       </c>
-      <c r="D53" s="34" t="s">
+      <c r="D53" s="139" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="54" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="25" t="s">
+      <c r="C54" s="135" t="s">
         <v>82</v>
       </c>
-      <c r="D54" s="34" t="s">
+      <c r="D54" s="139" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="55" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="25" t="s">
+      <c r="C55" s="135" t="s">
         <v>84</v>
       </c>
-      <c r="D55" s="34" t="s">
+      <c r="D55" s="139" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="56" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C56" s="25" t="s">
+      <c r="C56" s="135" t="s">
         <v>86</v>
       </c>
-      <c r="D56" s="34" t="s">
+      <c r="D56" s="139" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="57" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C57" s="25" t="s">
+      <c r="C57" s="135" t="s">
         <v>88</v>
       </c>
-      <c r="D57" s="34" t="s">
+      <c r="D57" s="139" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="58" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C58" s="25" t="s">
+      <c r="C58" s="135" t="s">
         <v>90</v>
       </c>
-      <c r="D58" s="34" t="s">
+      <c r="D58" s="139" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="59" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C59" s="25" t="s">
+      <c r="C59" s="136" t="s">
         <v>92</v>
       </c>
-      <c r="D59" s="34" t="s">
+      <c r="D59" s="140" t="s">
         <v>93</v>
       </c>
     </row>
@@ -5140,50 +5284,50 @@
       <c r="D61" s="37"/>
     </row>
     <row r="62" spans="3:4" ht="36" x14ac:dyDescent="0.25">
-      <c r="C62" s="25" t="s">
+      <c r="C62" s="134" t="s">
         <v>95</v>
       </c>
-      <c r="D62" s="34" t="s">
+      <c r="D62" s="138" t="s">
         <v>803</v>
       </c>
     </row>
     <row r="63" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C63" s="25" t="s">
+      <c r="C63" s="135" t="s">
         <v>805</v>
       </c>
-      <c r="D63" s="34" t="s">
+      <c r="D63" s="139" t="s">
         <v>804</v>
       </c>
     </row>
     <row r="64" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C64" s="25" t="s">
+      <c r="C64" s="135" t="s">
         <v>96</v>
       </c>
-      <c r="D64" s="34" t="s">
+      <c r="D64" s="139" t="s">
         <v>817</v>
       </c>
     </row>
     <row r="65" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C65" s="25" t="s">
+      <c r="C65" s="135" t="s">
         <v>97</v>
       </c>
-      <c r="D65" s="34" t="s">
+      <c r="D65" s="139" t="s">
         <v>838</v>
       </c>
     </row>
     <row r="66" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C66" s="25" t="s">
+      <c r="C66" s="135" t="s">
         <v>98</v>
       </c>
-      <c r="D66" s="34" t="s">
+      <c r="D66" s="139" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="67" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C67" s="25" t="s">
+      <c r="C67" s="136" t="s">
         <v>100</v>
       </c>
-      <c r="D67" s="34" t="s">
+      <c r="D67" s="140" t="s">
         <v>101</v>
       </c>
     </row>
@@ -5198,10 +5342,10 @@
       <c r="D69" s="37"/>
     </row>
     <row r="70" spans="3:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="25" t="s">
+      <c r="C70" s="137" t="s">
         <v>103</v>
       </c>
-      <c r="D70" s="34" t="s">
+      <c r="D70" s="141" t="s">
         <v>104</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Show each leg's Economic trade ID on TradeReconciliation (#246)
Last step of #45. TradeReconciliation gains a last column, Economic trade ID (TRC_ECON, TRC_NCOLS = 13; template header O6), filled by M_Main.WithEconomicTradeIds from Trades by Trade ID as the comparison matches it, blank for a whole trade or a leg not on Trades. The columns are read with CORE_Util.ColumnValues, now Public, so a single Trades row works. CORE_Reconcile still reads no sheet; Reconciliation keeps 12 columns. The column is cleared, written, fingerprinted and exported with the sheet. TEST_Reconcile: 18 cases, 137 checks. README, INSTALLATION and CHANGELOG updated.

Validated: python tools/check.py (all gates), check_vba_calls clean, no case-insensitive identifier collisions, template renders in LibreOffice. Excel (owner, on f9393dd): TEST_Reconcile RESULT=PASS cases=18 checks=137 failures=0; Test_RunAll RESULT=PASS suites=8 passed=8. Codex review clean on f9393dd.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -23123,7 +23123,7 @@
     <tabColor rgb="FF2E75B6"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="4" customWidth="1"/>
@@ -23139,9 +23139,10 @@
     <col min="12" max="12" width="12.75" style="16" customWidth="1"/>
     <col min="13" max="13" width="22.75" style="7" customWidth="1"/>
     <col min="14" max="14" width="80.75" style="7" customWidth="1"/>
+    <col min="15" max="15" width="18.75" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
@@ -23157,8 +23158,9 @@
       <c r="L1" s="66"/>
       <c r="M1" s="66"/>
       <c r="N1" s="66"/>
-    </row>
-    <row r="2" spans="2:14" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O1" s="66"/>
+    </row>
+    <row r="2" spans="2:15" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="30" t="s">
         <v>943</v>
       </c>
@@ -23174,22 +23176,23 @@
       <c r="L2" s="68"/>
       <c r="M2" s="68"/>
       <c r="N2" s="68"/>
-    </row>
-    <row r="3" spans="2:14" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O2" s="68"/>
+    </row>
+    <row r="3" spans="2:15" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C4" s="14" t="s">
         <v>944</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C5" s="14" t="str" cm="1">
         <f t="array" ref="C5">TradeReconciliationStatusText(SACCR_TradeReconInputs,SACCR_RunInputs,BankTrades!$1:$1048576,NettingSets!$C:$Q,Trades!$C:$AA,Params!$1:$1048576)</f>
         <v>No reconciliation: enter bank figures on BankTrades and press Run SA-CCR.</v>
       </c>
     </row>
-    <row r="6" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="15" t="s">
         <v>294</v>
       </c>
@@ -23225,6 +23228,9 @@
       </c>
       <c r="N6" s="15" t="s">
         <v>570</v>
+      </c>
+      <c r="O6" s="15" t="s">
+        <v>856</v>
       </c>
     </row>
   </sheetData>

</xml_diff>